<commit_message>
Daily Δ NET is blank past the pulled days again, under Fill all sims as well as live
The Δ NET block's =IFERROR(CURNET-NEWNET,"") relied on the LIVE spill emitting '' text
cells, which make the subtraction error and the Δ blank. Fill all sims writes VALUES; a
written '' is an empty cell, an empty cell subtracts as 0, and on LIVE_OPS_V3 (1) days
2..33 of Δ NET read a false 0.00 under a one-day live feed. Now
=IF(OR(CUR="",NEW=""),"",IFERROR(CUR-NEW,"")) - X="" is TRUE for an empty cell and for ''
text alike. Title no longer claims day 1 is a Wednesday (D64 reads the weekday row).
display/EcoGainsSim_Daily_v3.xlsx rebuilt; _display_formulas.json re-dumped (builder
parity still green: _mock_simfill 76/0 collections, 78/0 --data v3b).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/display/EcoGainsSim_Daily_v3.xlsx
+++ b/display/EcoGainsSim_Daily_v3.xlsx
@@ -778,7 +778,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>DAILY RESOURCE GAINS + NET — data vs sim, 33-day calendar, per earner (day 1 = Wednesday)</t>
+          <t>DAILY RESOURCE GAINS + NET — data vs sim, 33-day calendar, per earner (weekdays from the calendar sheets)</t>
         </is>
       </c>
       <c r="FP1" s="2" t="inlineStr">
@@ -2021,83 +2021,83 @@
       <c r="DW9" s="18" t="n"/>
       <c r="DX9" s="18" t="n"/>
       <c r="DZ9" s="17">
-        <f>IFERROR(CJ9-DE9,"")</f>
+        <f>IF(OR(CJ9="",DE9=""),"",IFERROR(CJ9-DE9,""))</f>
         <v/>
       </c>
       <c r="EA9" s="17">
-        <f>IFERROR(CK9-DF9,"")</f>
+        <f>IF(OR(CK9="",DF9=""),"",IFERROR(CK9-DF9,""))</f>
         <v/>
       </c>
       <c r="EB9" s="17">
-        <f>IFERROR(CL9-DG9,"")</f>
+        <f>IF(OR(CL9="",DG9=""),"",IFERROR(CL9-DG9,""))</f>
         <v/>
       </c>
       <c r="EC9" s="17">
-        <f>IFERROR(CM9-DH9,"")</f>
+        <f>IF(OR(CM9="",DH9=""),"",IFERROR(CM9-DH9,""))</f>
         <v/>
       </c>
       <c r="ED9" s="17">
-        <f>IFERROR(CN9-DI9,"")</f>
+        <f>IF(OR(CN9="",DI9=""),"",IFERROR(CN9-DI9,""))</f>
         <v/>
       </c>
       <c r="EE9" s="17">
-        <f>IFERROR(CO9-DJ9,"")</f>
+        <f>IF(OR(CO9="",DJ9=""),"",IFERROR(CO9-DJ9,""))</f>
         <v/>
       </c>
       <c r="EF9" s="17">
-        <f>IFERROR(CP9-DK9,"")</f>
+        <f>IF(OR(CP9="",DK9=""),"",IFERROR(CP9-DK9,""))</f>
         <v/>
       </c>
       <c r="EG9" s="17">
-        <f>IFERROR(CQ9-DL9,"")</f>
+        <f>IF(OR(CQ9="",DL9=""),"",IFERROR(CQ9-DL9,""))</f>
         <v/>
       </c>
       <c r="EH9" s="17">
-        <f>IFERROR(CR9-DM9,"")</f>
+        <f>IF(OR(CR9="",DM9=""),"",IFERROR(CR9-DM9,""))</f>
         <v/>
       </c>
       <c r="EI9" s="17">
-        <f>IFERROR(CS9-DN9,"")</f>
+        <f>IF(OR(CS9="",DN9=""),"",IFERROR(CS9-DN9,""))</f>
         <v/>
       </c>
       <c r="EJ9" s="17">
-        <f>IFERROR(CT9-DO9,"")</f>
+        <f>IF(OR(CT9="",DO9=""),"",IFERROR(CT9-DO9,""))</f>
         <v/>
       </c>
       <c r="EK9" s="17">
-        <f>IFERROR(CU9-DP9,"")</f>
+        <f>IF(OR(CU9="",DP9=""),"",IFERROR(CU9-DP9,""))</f>
         <v/>
       </c>
       <c r="EL9" s="17">
-        <f>IFERROR(CV9-DQ9,"")</f>
+        <f>IF(OR(CV9="",DQ9=""),"",IFERROR(CV9-DQ9,""))</f>
         <v/>
       </c>
       <c r="EM9" s="17">
-        <f>IFERROR(CW9-DR9,"")</f>
+        <f>IF(OR(CW9="",DR9=""),"",IFERROR(CW9-DR9,""))</f>
         <v/>
       </c>
       <c r="EN9" s="17">
-        <f>IFERROR(CX9-DS9,"")</f>
+        <f>IF(OR(CX9="",DS9=""),"",IFERROR(CX9-DS9,""))</f>
         <v/>
       </c>
       <c r="EO9" s="17">
-        <f>IFERROR(CY9-DT9,"")</f>
+        <f>IF(OR(CY9="",DT9=""),"",IFERROR(CY9-DT9,""))</f>
         <v/>
       </c>
       <c r="EP9" s="17">
-        <f>IFERROR(CZ9-DU9,"")</f>
+        <f>IF(OR(CZ9="",DU9=""),"",IFERROR(CZ9-DU9,""))</f>
         <v/>
       </c>
       <c r="EQ9" s="17">
-        <f>IFERROR(DA9-DV9,"")</f>
+        <f>IF(OR(DA9="",DV9=""),"",IFERROR(DA9-DV9,""))</f>
         <v/>
       </c>
       <c r="ER9" s="17">
-        <f>IFERROR(DB9-DW9,"")</f>
+        <f>IF(OR(DB9="",DW9=""),"",IFERROR(DB9-DW9,""))</f>
         <v/>
       </c>
       <c r="ES9" s="17">
-        <f>IFERROR(DC9-DX9,"")</f>
+        <f>IF(OR(DC9="",DX9=""),"",IFERROR(DC9-DX9,""))</f>
         <v/>
       </c>
       <c r="EU9" s="16">
@@ -2259,83 +2259,83 @@
       <c r="DW10" s="18" t="n"/>
       <c r="DX10" s="18" t="n"/>
       <c r="DZ10" s="17">
-        <f>IFERROR(CJ10-DE10,"")</f>
+        <f>IF(OR(CJ10="",DE10=""),"",IFERROR(CJ10-DE10,""))</f>
         <v/>
       </c>
       <c r="EA10" s="17">
-        <f>IFERROR(CK10-DF10,"")</f>
+        <f>IF(OR(CK10="",DF10=""),"",IFERROR(CK10-DF10,""))</f>
         <v/>
       </c>
       <c r="EB10" s="17">
-        <f>IFERROR(CL10-DG10,"")</f>
+        <f>IF(OR(CL10="",DG10=""),"",IFERROR(CL10-DG10,""))</f>
         <v/>
       </c>
       <c r="EC10" s="17">
-        <f>IFERROR(CM10-DH10,"")</f>
+        <f>IF(OR(CM10="",DH10=""),"",IFERROR(CM10-DH10,""))</f>
         <v/>
       </c>
       <c r="ED10" s="17">
-        <f>IFERROR(CN10-DI10,"")</f>
+        <f>IF(OR(CN10="",DI10=""),"",IFERROR(CN10-DI10,""))</f>
         <v/>
       </c>
       <c r="EE10" s="17">
-        <f>IFERROR(CO10-DJ10,"")</f>
+        <f>IF(OR(CO10="",DJ10=""),"",IFERROR(CO10-DJ10,""))</f>
         <v/>
       </c>
       <c r="EF10" s="17">
-        <f>IFERROR(CP10-DK10,"")</f>
+        <f>IF(OR(CP10="",DK10=""),"",IFERROR(CP10-DK10,""))</f>
         <v/>
       </c>
       <c r="EG10" s="17">
-        <f>IFERROR(CQ10-DL10,"")</f>
+        <f>IF(OR(CQ10="",DL10=""),"",IFERROR(CQ10-DL10,""))</f>
         <v/>
       </c>
       <c r="EH10" s="17">
-        <f>IFERROR(CR10-DM10,"")</f>
+        <f>IF(OR(CR10="",DM10=""),"",IFERROR(CR10-DM10,""))</f>
         <v/>
       </c>
       <c r="EI10" s="17">
-        <f>IFERROR(CS10-DN10,"")</f>
+        <f>IF(OR(CS10="",DN10=""),"",IFERROR(CS10-DN10,""))</f>
         <v/>
       </c>
       <c r="EJ10" s="17">
-        <f>IFERROR(CT10-DO10,"")</f>
+        <f>IF(OR(CT10="",DO10=""),"",IFERROR(CT10-DO10,""))</f>
         <v/>
       </c>
       <c r="EK10" s="17">
-        <f>IFERROR(CU10-DP10,"")</f>
+        <f>IF(OR(CU10="",DP10=""),"",IFERROR(CU10-DP10,""))</f>
         <v/>
       </c>
       <c r="EL10" s="17">
-        <f>IFERROR(CV10-DQ10,"")</f>
+        <f>IF(OR(CV10="",DQ10=""),"",IFERROR(CV10-DQ10,""))</f>
         <v/>
       </c>
       <c r="EM10" s="17">
-        <f>IFERROR(CW10-DR10,"")</f>
+        <f>IF(OR(CW10="",DR10=""),"",IFERROR(CW10-DR10,""))</f>
         <v/>
       </c>
       <c r="EN10" s="17">
-        <f>IFERROR(CX10-DS10,"")</f>
+        <f>IF(OR(CX10="",DS10=""),"",IFERROR(CX10-DS10,""))</f>
         <v/>
       </c>
       <c r="EO10" s="17">
-        <f>IFERROR(CY10-DT10,"")</f>
+        <f>IF(OR(CY10="",DT10=""),"",IFERROR(CY10-DT10,""))</f>
         <v/>
       </c>
       <c r="EP10" s="17">
-        <f>IFERROR(CZ10-DU10,"")</f>
+        <f>IF(OR(CZ10="",DU10=""),"",IFERROR(CZ10-DU10,""))</f>
         <v/>
       </c>
       <c r="EQ10" s="17">
-        <f>IFERROR(DA10-DV10,"")</f>
+        <f>IF(OR(DA10="",DV10=""),"",IFERROR(DA10-DV10,""))</f>
         <v/>
       </c>
       <c r="ER10" s="17">
-        <f>IFERROR(DB10-DW10,"")</f>
+        <f>IF(OR(DB10="",DW10=""),"",IFERROR(DB10-DW10,""))</f>
         <v/>
       </c>
       <c r="ES10" s="17">
-        <f>IFERROR(DC10-DX10,"")</f>
+        <f>IF(OR(DC10="",DX10=""),"",IFERROR(DC10-DX10,""))</f>
         <v/>
       </c>
       <c r="EU10" s="16" t="n"/>
@@ -2494,83 +2494,83 @@
       <c r="DW11" s="18" t="n"/>
       <c r="DX11" s="18" t="n"/>
       <c r="DZ11" s="17">
-        <f>IFERROR(CJ11-DE11,"")</f>
+        <f>IF(OR(CJ11="",DE11=""),"",IFERROR(CJ11-DE11,""))</f>
         <v/>
       </c>
       <c r="EA11" s="17">
-        <f>IFERROR(CK11-DF11,"")</f>
+        <f>IF(OR(CK11="",DF11=""),"",IFERROR(CK11-DF11,""))</f>
         <v/>
       </c>
       <c r="EB11" s="17">
-        <f>IFERROR(CL11-DG11,"")</f>
+        <f>IF(OR(CL11="",DG11=""),"",IFERROR(CL11-DG11,""))</f>
         <v/>
       </c>
       <c r="EC11" s="17">
-        <f>IFERROR(CM11-DH11,"")</f>
+        <f>IF(OR(CM11="",DH11=""),"",IFERROR(CM11-DH11,""))</f>
         <v/>
       </c>
       <c r="ED11" s="17">
-        <f>IFERROR(CN11-DI11,"")</f>
+        <f>IF(OR(CN11="",DI11=""),"",IFERROR(CN11-DI11,""))</f>
         <v/>
       </c>
       <c r="EE11" s="17">
-        <f>IFERROR(CO11-DJ11,"")</f>
+        <f>IF(OR(CO11="",DJ11=""),"",IFERROR(CO11-DJ11,""))</f>
         <v/>
       </c>
       <c r="EF11" s="17">
-        <f>IFERROR(CP11-DK11,"")</f>
+        <f>IF(OR(CP11="",DK11=""),"",IFERROR(CP11-DK11,""))</f>
         <v/>
       </c>
       <c r="EG11" s="17">
-        <f>IFERROR(CQ11-DL11,"")</f>
+        <f>IF(OR(CQ11="",DL11=""),"",IFERROR(CQ11-DL11,""))</f>
         <v/>
       </c>
       <c r="EH11" s="17">
-        <f>IFERROR(CR11-DM11,"")</f>
+        <f>IF(OR(CR11="",DM11=""),"",IFERROR(CR11-DM11,""))</f>
         <v/>
       </c>
       <c r="EI11" s="17">
-        <f>IFERROR(CS11-DN11,"")</f>
+        <f>IF(OR(CS11="",DN11=""),"",IFERROR(CS11-DN11,""))</f>
         <v/>
       </c>
       <c r="EJ11" s="17">
-        <f>IFERROR(CT11-DO11,"")</f>
+        <f>IF(OR(CT11="",DO11=""),"",IFERROR(CT11-DO11,""))</f>
         <v/>
       </c>
       <c r="EK11" s="17">
-        <f>IFERROR(CU11-DP11,"")</f>
+        <f>IF(OR(CU11="",DP11=""),"",IFERROR(CU11-DP11,""))</f>
         <v/>
       </c>
       <c r="EL11" s="17">
-        <f>IFERROR(CV11-DQ11,"")</f>
+        <f>IF(OR(CV11="",DQ11=""),"",IFERROR(CV11-DQ11,""))</f>
         <v/>
       </c>
       <c r="EM11" s="17">
-        <f>IFERROR(CW11-DR11,"")</f>
+        <f>IF(OR(CW11="",DR11=""),"",IFERROR(CW11-DR11,""))</f>
         <v/>
       </c>
       <c r="EN11" s="17">
-        <f>IFERROR(CX11-DS11,"")</f>
+        <f>IF(OR(CX11="",DS11=""),"",IFERROR(CX11-DS11,""))</f>
         <v/>
       </c>
       <c r="EO11" s="17">
-        <f>IFERROR(CY11-DT11,"")</f>
+        <f>IF(OR(CY11="",DT11=""),"",IFERROR(CY11-DT11,""))</f>
         <v/>
       </c>
       <c r="EP11" s="17">
-        <f>IFERROR(CZ11-DU11,"")</f>
+        <f>IF(OR(CZ11="",DU11=""),"",IFERROR(CZ11-DU11,""))</f>
         <v/>
       </c>
       <c r="EQ11" s="17">
-        <f>IFERROR(DA11-DV11,"")</f>
+        <f>IF(OR(DA11="",DV11=""),"",IFERROR(DA11-DV11,""))</f>
         <v/>
       </c>
       <c r="ER11" s="17">
-        <f>IFERROR(DB11-DW11,"")</f>
+        <f>IF(OR(DB11="",DW11=""),"",IFERROR(DB11-DW11,""))</f>
         <v/>
       </c>
       <c r="ES11" s="17">
-        <f>IFERROR(DC11-DX11,"")</f>
+        <f>IF(OR(DC11="",DX11=""),"",IFERROR(DC11-DX11,""))</f>
         <v/>
       </c>
       <c r="EU11" s="16" t="n"/>
@@ -2729,83 +2729,83 @@
       <c r="DW12" s="18" t="n"/>
       <c r="DX12" s="18" t="n"/>
       <c r="DZ12" s="17">
-        <f>IFERROR(CJ12-DE12,"")</f>
+        <f>IF(OR(CJ12="",DE12=""),"",IFERROR(CJ12-DE12,""))</f>
         <v/>
       </c>
       <c r="EA12" s="17">
-        <f>IFERROR(CK12-DF12,"")</f>
+        <f>IF(OR(CK12="",DF12=""),"",IFERROR(CK12-DF12,""))</f>
         <v/>
       </c>
       <c r="EB12" s="17">
-        <f>IFERROR(CL12-DG12,"")</f>
+        <f>IF(OR(CL12="",DG12=""),"",IFERROR(CL12-DG12,""))</f>
         <v/>
       </c>
       <c r="EC12" s="17">
-        <f>IFERROR(CM12-DH12,"")</f>
+        <f>IF(OR(CM12="",DH12=""),"",IFERROR(CM12-DH12,""))</f>
         <v/>
       </c>
       <c r="ED12" s="17">
-        <f>IFERROR(CN12-DI12,"")</f>
+        <f>IF(OR(CN12="",DI12=""),"",IFERROR(CN12-DI12,""))</f>
         <v/>
       </c>
       <c r="EE12" s="17">
-        <f>IFERROR(CO12-DJ12,"")</f>
+        <f>IF(OR(CO12="",DJ12=""),"",IFERROR(CO12-DJ12,""))</f>
         <v/>
       </c>
       <c r="EF12" s="17">
-        <f>IFERROR(CP12-DK12,"")</f>
+        <f>IF(OR(CP12="",DK12=""),"",IFERROR(CP12-DK12,""))</f>
         <v/>
       </c>
       <c r="EG12" s="17">
-        <f>IFERROR(CQ12-DL12,"")</f>
+        <f>IF(OR(CQ12="",DL12=""),"",IFERROR(CQ12-DL12,""))</f>
         <v/>
       </c>
       <c r="EH12" s="17">
-        <f>IFERROR(CR12-DM12,"")</f>
+        <f>IF(OR(CR12="",DM12=""),"",IFERROR(CR12-DM12,""))</f>
         <v/>
       </c>
       <c r="EI12" s="17">
-        <f>IFERROR(CS12-DN12,"")</f>
+        <f>IF(OR(CS12="",DN12=""),"",IFERROR(CS12-DN12,""))</f>
         <v/>
       </c>
       <c r="EJ12" s="17">
-        <f>IFERROR(CT12-DO12,"")</f>
+        <f>IF(OR(CT12="",DO12=""),"",IFERROR(CT12-DO12,""))</f>
         <v/>
       </c>
       <c r="EK12" s="17">
-        <f>IFERROR(CU12-DP12,"")</f>
+        <f>IF(OR(CU12="",DP12=""),"",IFERROR(CU12-DP12,""))</f>
         <v/>
       </c>
       <c r="EL12" s="17">
-        <f>IFERROR(CV12-DQ12,"")</f>
+        <f>IF(OR(CV12="",DQ12=""),"",IFERROR(CV12-DQ12,""))</f>
         <v/>
       </c>
       <c r="EM12" s="17">
-        <f>IFERROR(CW12-DR12,"")</f>
+        <f>IF(OR(CW12="",DR12=""),"",IFERROR(CW12-DR12,""))</f>
         <v/>
       </c>
       <c r="EN12" s="17">
-        <f>IFERROR(CX12-DS12,"")</f>
+        <f>IF(OR(CX12="",DS12=""),"",IFERROR(CX12-DS12,""))</f>
         <v/>
       </c>
       <c r="EO12" s="17">
-        <f>IFERROR(CY12-DT12,"")</f>
+        <f>IF(OR(CY12="",DT12=""),"",IFERROR(CY12-DT12,""))</f>
         <v/>
       </c>
       <c r="EP12" s="17">
-        <f>IFERROR(CZ12-DU12,"")</f>
+        <f>IF(OR(CZ12="",DU12=""),"",IFERROR(CZ12-DU12,""))</f>
         <v/>
       </c>
       <c r="EQ12" s="17">
-        <f>IFERROR(DA12-DV12,"")</f>
+        <f>IF(OR(DA12="",DV12=""),"",IFERROR(DA12-DV12,""))</f>
         <v/>
       </c>
       <c r="ER12" s="17">
-        <f>IFERROR(DB12-DW12,"")</f>
+        <f>IF(OR(DB12="",DW12=""),"",IFERROR(DB12-DW12,""))</f>
         <v/>
       </c>
       <c r="ES12" s="17">
-        <f>IFERROR(DC12-DX12,"")</f>
+        <f>IF(OR(DC12="",DX12=""),"",IFERROR(DC12-DX12,""))</f>
         <v/>
       </c>
       <c r="EU12" s="16" t="n"/>
@@ -2964,83 +2964,83 @@
       <c r="DW13" s="18" t="n"/>
       <c r="DX13" s="18" t="n"/>
       <c r="DZ13" s="17">
-        <f>IFERROR(CJ13-DE13,"")</f>
+        <f>IF(OR(CJ13="",DE13=""),"",IFERROR(CJ13-DE13,""))</f>
         <v/>
       </c>
       <c r="EA13" s="17">
-        <f>IFERROR(CK13-DF13,"")</f>
+        <f>IF(OR(CK13="",DF13=""),"",IFERROR(CK13-DF13,""))</f>
         <v/>
       </c>
       <c r="EB13" s="17">
-        <f>IFERROR(CL13-DG13,"")</f>
+        <f>IF(OR(CL13="",DG13=""),"",IFERROR(CL13-DG13,""))</f>
         <v/>
       </c>
       <c r="EC13" s="17">
-        <f>IFERROR(CM13-DH13,"")</f>
+        <f>IF(OR(CM13="",DH13=""),"",IFERROR(CM13-DH13,""))</f>
         <v/>
       </c>
       <c r="ED13" s="17">
-        <f>IFERROR(CN13-DI13,"")</f>
+        <f>IF(OR(CN13="",DI13=""),"",IFERROR(CN13-DI13,""))</f>
         <v/>
       </c>
       <c r="EE13" s="17">
-        <f>IFERROR(CO13-DJ13,"")</f>
+        <f>IF(OR(CO13="",DJ13=""),"",IFERROR(CO13-DJ13,""))</f>
         <v/>
       </c>
       <c r="EF13" s="17">
-        <f>IFERROR(CP13-DK13,"")</f>
+        <f>IF(OR(CP13="",DK13=""),"",IFERROR(CP13-DK13,""))</f>
         <v/>
       </c>
       <c r="EG13" s="17">
-        <f>IFERROR(CQ13-DL13,"")</f>
+        <f>IF(OR(CQ13="",DL13=""),"",IFERROR(CQ13-DL13,""))</f>
         <v/>
       </c>
       <c r="EH13" s="17">
-        <f>IFERROR(CR13-DM13,"")</f>
+        <f>IF(OR(CR13="",DM13=""),"",IFERROR(CR13-DM13,""))</f>
         <v/>
       </c>
       <c r="EI13" s="17">
-        <f>IFERROR(CS13-DN13,"")</f>
+        <f>IF(OR(CS13="",DN13=""),"",IFERROR(CS13-DN13,""))</f>
         <v/>
       </c>
       <c r="EJ13" s="17">
-        <f>IFERROR(CT13-DO13,"")</f>
+        <f>IF(OR(CT13="",DO13=""),"",IFERROR(CT13-DO13,""))</f>
         <v/>
       </c>
       <c r="EK13" s="17">
-        <f>IFERROR(CU13-DP13,"")</f>
+        <f>IF(OR(CU13="",DP13=""),"",IFERROR(CU13-DP13,""))</f>
         <v/>
       </c>
       <c r="EL13" s="17">
-        <f>IFERROR(CV13-DQ13,"")</f>
+        <f>IF(OR(CV13="",DQ13=""),"",IFERROR(CV13-DQ13,""))</f>
         <v/>
       </c>
       <c r="EM13" s="17">
-        <f>IFERROR(CW13-DR13,"")</f>
+        <f>IF(OR(CW13="",DR13=""),"",IFERROR(CW13-DR13,""))</f>
         <v/>
       </c>
       <c r="EN13" s="17">
-        <f>IFERROR(CX13-DS13,"")</f>
+        <f>IF(OR(CX13="",DS13=""),"",IFERROR(CX13-DS13,""))</f>
         <v/>
       </c>
       <c r="EO13" s="17">
-        <f>IFERROR(CY13-DT13,"")</f>
+        <f>IF(OR(CY13="",DT13=""),"",IFERROR(CY13-DT13,""))</f>
         <v/>
       </c>
       <c r="EP13" s="17">
-        <f>IFERROR(CZ13-DU13,"")</f>
+        <f>IF(OR(CZ13="",DU13=""),"",IFERROR(CZ13-DU13,""))</f>
         <v/>
       </c>
       <c r="EQ13" s="17">
-        <f>IFERROR(DA13-DV13,"")</f>
+        <f>IF(OR(DA13="",DV13=""),"",IFERROR(DA13-DV13,""))</f>
         <v/>
       </c>
       <c r="ER13" s="17">
-        <f>IFERROR(DB13-DW13,"")</f>
+        <f>IF(OR(DB13="",DW13=""),"",IFERROR(DB13-DW13,""))</f>
         <v/>
       </c>
       <c r="ES13" s="17">
-        <f>IFERROR(DC13-DX13,"")</f>
+        <f>IF(OR(DC13="",DX13=""),"",IFERROR(DC13-DX13,""))</f>
         <v/>
       </c>
       <c r="EU13" s="16" t="n"/>
@@ -3199,83 +3199,83 @@
       <c r="DW14" s="18" t="n"/>
       <c r="DX14" s="18" t="n"/>
       <c r="DZ14" s="17">
-        <f>IFERROR(CJ14-DE14,"")</f>
+        <f>IF(OR(CJ14="",DE14=""),"",IFERROR(CJ14-DE14,""))</f>
         <v/>
       </c>
       <c r="EA14" s="17">
-        <f>IFERROR(CK14-DF14,"")</f>
+        <f>IF(OR(CK14="",DF14=""),"",IFERROR(CK14-DF14,""))</f>
         <v/>
       </c>
       <c r="EB14" s="17">
-        <f>IFERROR(CL14-DG14,"")</f>
+        <f>IF(OR(CL14="",DG14=""),"",IFERROR(CL14-DG14,""))</f>
         <v/>
       </c>
       <c r="EC14" s="17">
-        <f>IFERROR(CM14-DH14,"")</f>
+        <f>IF(OR(CM14="",DH14=""),"",IFERROR(CM14-DH14,""))</f>
         <v/>
       </c>
       <c r="ED14" s="17">
-        <f>IFERROR(CN14-DI14,"")</f>
+        <f>IF(OR(CN14="",DI14=""),"",IFERROR(CN14-DI14,""))</f>
         <v/>
       </c>
       <c r="EE14" s="17">
-        <f>IFERROR(CO14-DJ14,"")</f>
+        <f>IF(OR(CO14="",DJ14=""),"",IFERROR(CO14-DJ14,""))</f>
         <v/>
       </c>
       <c r="EF14" s="17">
-        <f>IFERROR(CP14-DK14,"")</f>
+        <f>IF(OR(CP14="",DK14=""),"",IFERROR(CP14-DK14,""))</f>
         <v/>
       </c>
       <c r="EG14" s="17">
-        <f>IFERROR(CQ14-DL14,"")</f>
+        <f>IF(OR(CQ14="",DL14=""),"",IFERROR(CQ14-DL14,""))</f>
         <v/>
       </c>
       <c r="EH14" s="17">
-        <f>IFERROR(CR14-DM14,"")</f>
+        <f>IF(OR(CR14="",DM14=""),"",IFERROR(CR14-DM14,""))</f>
         <v/>
       </c>
       <c r="EI14" s="17">
-        <f>IFERROR(CS14-DN14,"")</f>
+        <f>IF(OR(CS14="",DN14=""),"",IFERROR(CS14-DN14,""))</f>
         <v/>
       </c>
       <c r="EJ14" s="17">
-        <f>IFERROR(CT14-DO14,"")</f>
+        <f>IF(OR(CT14="",DO14=""),"",IFERROR(CT14-DO14,""))</f>
         <v/>
       </c>
       <c r="EK14" s="17">
-        <f>IFERROR(CU14-DP14,"")</f>
+        <f>IF(OR(CU14="",DP14=""),"",IFERROR(CU14-DP14,""))</f>
         <v/>
       </c>
       <c r="EL14" s="17">
-        <f>IFERROR(CV14-DQ14,"")</f>
+        <f>IF(OR(CV14="",DQ14=""),"",IFERROR(CV14-DQ14,""))</f>
         <v/>
       </c>
       <c r="EM14" s="17">
-        <f>IFERROR(CW14-DR14,"")</f>
+        <f>IF(OR(CW14="",DR14=""),"",IFERROR(CW14-DR14,""))</f>
         <v/>
       </c>
       <c r="EN14" s="17">
-        <f>IFERROR(CX14-DS14,"")</f>
+        <f>IF(OR(CX14="",DS14=""),"",IFERROR(CX14-DS14,""))</f>
         <v/>
       </c>
       <c r="EO14" s="17">
-        <f>IFERROR(CY14-DT14,"")</f>
+        <f>IF(OR(CY14="",DT14=""),"",IFERROR(CY14-DT14,""))</f>
         <v/>
       </c>
       <c r="EP14" s="17">
-        <f>IFERROR(CZ14-DU14,"")</f>
+        <f>IF(OR(CZ14="",DU14=""),"",IFERROR(CZ14-DU14,""))</f>
         <v/>
       </c>
       <c r="EQ14" s="17">
-        <f>IFERROR(DA14-DV14,"")</f>
+        <f>IF(OR(DA14="",DV14=""),"",IFERROR(DA14-DV14,""))</f>
         <v/>
       </c>
       <c r="ER14" s="17">
-        <f>IFERROR(DB14-DW14,"")</f>
+        <f>IF(OR(DB14="",DW14=""),"",IFERROR(DB14-DW14,""))</f>
         <v/>
       </c>
       <c r="ES14" s="17">
-        <f>IFERROR(DC14-DX14,"")</f>
+        <f>IF(OR(DC14="",DX14=""),"",IFERROR(DC14-DX14,""))</f>
         <v/>
       </c>
       <c r="EU14" s="16" t="n"/>
@@ -3434,83 +3434,83 @@
       <c r="DW15" s="18" t="n"/>
       <c r="DX15" s="18" t="n"/>
       <c r="DZ15" s="17">
-        <f>IFERROR(CJ15-DE15,"")</f>
+        <f>IF(OR(CJ15="",DE15=""),"",IFERROR(CJ15-DE15,""))</f>
         <v/>
       </c>
       <c r="EA15" s="17">
-        <f>IFERROR(CK15-DF15,"")</f>
+        <f>IF(OR(CK15="",DF15=""),"",IFERROR(CK15-DF15,""))</f>
         <v/>
       </c>
       <c r="EB15" s="17">
-        <f>IFERROR(CL15-DG15,"")</f>
+        <f>IF(OR(CL15="",DG15=""),"",IFERROR(CL15-DG15,""))</f>
         <v/>
       </c>
       <c r="EC15" s="17">
-        <f>IFERROR(CM15-DH15,"")</f>
+        <f>IF(OR(CM15="",DH15=""),"",IFERROR(CM15-DH15,""))</f>
         <v/>
       </c>
       <c r="ED15" s="17">
-        <f>IFERROR(CN15-DI15,"")</f>
+        <f>IF(OR(CN15="",DI15=""),"",IFERROR(CN15-DI15,""))</f>
         <v/>
       </c>
       <c r="EE15" s="17">
-        <f>IFERROR(CO15-DJ15,"")</f>
+        <f>IF(OR(CO15="",DJ15=""),"",IFERROR(CO15-DJ15,""))</f>
         <v/>
       </c>
       <c r="EF15" s="17">
-        <f>IFERROR(CP15-DK15,"")</f>
+        <f>IF(OR(CP15="",DK15=""),"",IFERROR(CP15-DK15,""))</f>
         <v/>
       </c>
       <c r="EG15" s="17">
-        <f>IFERROR(CQ15-DL15,"")</f>
+        <f>IF(OR(CQ15="",DL15=""),"",IFERROR(CQ15-DL15,""))</f>
         <v/>
       </c>
       <c r="EH15" s="17">
-        <f>IFERROR(CR15-DM15,"")</f>
+        <f>IF(OR(CR15="",DM15=""),"",IFERROR(CR15-DM15,""))</f>
         <v/>
       </c>
       <c r="EI15" s="17">
-        <f>IFERROR(CS15-DN15,"")</f>
+        <f>IF(OR(CS15="",DN15=""),"",IFERROR(CS15-DN15,""))</f>
         <v/>
       </c>
       <c r="EJ15" s="17">
-        <f>IFERROR(CT15-DO15,"")</f>
+        <f>IF(OR(CT15="",DO15=""),"",IFERROR(CT15-DO15,""))</f>
         <v/>
       </c>
       <c r="EK15" s="17">
-        <f>IFERROR(CU15-DP15,"")</f>
+        <f>IF(OR(CU15="",DP15=""),"",IFERROR(CU15-DP15,""))</f>
         <v/>
       </c>
       <c r="EL15" s="17">
-        <f>IFERROR(CV15-DQ15,"")</f>
+        <f>IF(OR(CV15="",DQ15=""),"",IFERROR(CV15-DQ15,""))</f>
         <v/>
       </c>
       <c r="EM15" s="17">
-        <f>IFERROR(CW15-DR15,"")</f>
+        <f>IF(OR(CW15="",DR15=""),"",IFERROR(CW15-DR15,""))</f>
         <v/>
       </c>
       <c r="EN15" s="17">
-        <f>IFERROR(CX15-DS15,"")</f>
+        <f>IF(OR(CX15="",DS15=""),"",IFERROR(CX15-DS15,""))</f>
         <v/>
       </c>
       <c r="EO15" s="17">
-        <f>IFERROR(CY15-DT15,"")</f>
+        <f>IF(OR(CY15="",DT15=""),"",IFERROR(CY15-DT15,""))</f>
         <v/>
       </c>
       <c r="EP15" s="17">
-        <f>IFERROR(CZ15-DU15,"")</f>
+        <f>IF(OR(CZ15="",DU15=""),"",IFERROR(CZ15-DU15,""))</f>
         <v/>
       </c>
       <c r="EQ15" s="17">
-        <f>IFERROR(DA15-DV15,"")</f>
+        <f>IF(OR(DA15="",DV15=""),"",IFERROR(DA15-DV15,""))</f>
         <v/>
       </c>
       <c r="ER15" s="17">
-        <f>IFERROR(DB15-DW15,"")</f>
+        <f>IF(OR(DB15="",DW15=""),"",IFERROR(DB15-DW15,""))</f>
         <v/>
       </c>
       <c r="ES15" s="17">
-        <f>IFERROR(DC15-DX15,"")</f>
+        <f>IF(OR(DC15="",DX15=""),"",IFERROR(DC15-DX15,""))</f>
         <v/>
       </c>
       <c r="EU15" s="16" t="n"/>
@@ -3669,83 +3669,83 @@
       <c r="DW16" s="18" t="n"/>
       <c r="DX16" s="18" t="n"/>
       <c r="DZ16" s="17">
-        <f>IFERROR(CJ16-DE16,"")</f>
+        <f>IF(OR(CJ16="",DE16=""),"",IFERROR(CJ16-DE16,""))</f>
         <v/>
       </c>
       <c r="EA16" s="17">
-        <f>IFERROR(CK16-DF16,"")</f>
+        <f>IF(OR(CK16="",DF16=""),"",IFERROR(CK16-DF16,""))</f>
         <v/>
       </c>
       <c r="EB16" s="17">
-        <f>IFERROR(CL16-DG16,"")</f>
+        <f>IF(OR(CL16="",DG16=""),"",IFERROR(CL16-DG16,""))</f>
         <v/>
       </c>
       <c r="EC16" s="17">
-        <f>IFERROR(CM16-DH16,"")</f>
+        <f>IF(OR(CM16="",DH16=""),"",IFERROR(CM16-DH16,""))</f>
         <v/>
       </c>
       <c r="ED16" s="17">
-        <f>IFERROR(CN16-DI16,"")</f>
+        <f>IF(OR(CN16="",DI16=""),"",IFERROR(CN16-DI16,""))</f>
         <v/>
       </c>
       <c r="EE16" s="17">
-        <f>IFERROR(CO16-DJ16,"")</f>
+        <f>IF(OR(CO16="",DJ16=""),"",IFERROR(CO16-DJ16,""))</f>
         <v/>
       </c>
       <c r="EF16" s="17">
-        <f>IFERROR(CP16-DK16,"")</f>
+        <f>IF(OR(CP16="",DK16=""),"",IFERROR(CP16-DK16,""))</f>
         <v/>
       </c>
       <c r="EG16" s="17">
-        <f>IFERROR(CQ16-DL16,"")</f>
+        <f>IF(OR(CQ16="",DL16=""),"",IFERROR(CQ16-DL16,""))</f>
         <v/>
       </c>
       <c r="EH16" s="17">
-        <f>IFERROR(CR16-DM16,"")</f>
+        <f>IF(OR(CR16="",DM16=""),"",IFERROR(CR16-DM16,""))</f>
         <v/>
       </c>
       <c r="EI16" s="17">
-        <f>IFERROR(CS16-DN16,"")</f>
+        <f>IF(OR(CS16="",DN16=""),"",IFERROR(CS16-DN16,""))</f>
         <v/>
       </c>
       <c r="EJ16" s="17">
-        <f>IFERROR(CT16-DO16,"")</f>
+        <f>IF(OR(CT16="",DO16=""),"",IFERROR(CT16-DO16,""))</f>
         <v/>
       </c>
       <c r="EK16" s="17">
-        <f>IFERROR(CU16-DP16,"")</f>
+        <f>IF(OR(CU16="",DP16=""),"",IFERROR(CU16-DP16,""))</f>
         <v/>
       </c>
       <c r="EL16" s="17">
-        <f>IFERROR(CV16-DQ16,"")</f>
+        <f>IF(OR(CV16="",DQ16=""),"",IFERROR(CV16-DQ16,""))</f>
         <v/>
       </c>
       <c r="EM16" s="17">
-        <f>IFERROR(CW16-DR16,"")</f>
+        <f>IF(OR(CW16="",DR16=""),"",IFERROR(CW16-DR16,""))</f>
         <v/>
       </c>
       <c r="EN16" s="17">
-        <f>IFERROR(CX16-DS16,"")</f>
+        <f>IF(OR(CX16="",DS16=""),"",IFERROR(CX16-DS16,""))</f>
         <v/>
       </c>
       <c r="EO16" s="17">
-        <f>IFERROR(CY16-DT16,"")</f>
+        <f>IF(OR(CY16="",DT16=""),"",IFERROR(CY16-DT16,""))</f>
         <v/>
       </c>
       <c r="EP16" s="17">
-        <f>IFERROR(CZ16-DU16,"")</f>
+        <f>IF(OR(CZ16="",DU16=""),"",IFERROR(CZ16-DU16,""))</f>
         <v/>
       </c>
       <c r="EQ16" s="17">
-        <f>IFERROR(DA16-DV16,"")</f>
+        <f>IF(OR(DA16="",DV16=""),"",IFERROR(DA16-DV16,""))</f>
         <v/>
       </c>
       <c r="ER16" s="17">
-        <f>IFERROR(DB16-DW16,"")</f>
+        <f>IF(OR(DB16="",DW16=""),"",IFERROR(DB16-DW16,""))</f>
         <v/>
       </c>
       <c r="ES16" s="17">
-        <f>IFERROR(DC16-DX16,"")</f>
+        <f>IF(OR(DC16="",DX16=""),"",IFERROR(DC16-DX16,""))</f>
         <v/>
       </c>
       <c r="EU16" s="16" t="n"/>
@@ -3904,83 +3904,83 @@
       <c r="DW17" s="18" t="n"/>
       <c r="DX17" s="18" t="n"/>
       <c r="DZ17" s="17">
-        <f>IFERROR(CJ17-DE17,"")</f>
+        <f>IF(OR(CJ17="",DE17=""),"",IFERROR(CJ17-DE17,""))</f>
         <v/>
       </c>
       <c r="EA17" s="17">
-        <f>IFERROR(CK17-DF17,"")</f>
+        <f>IF(OR(CK17="",DF17=""),"",IFERROR(CK17-DF17,""))</f>
         <v/>
       </c>
       <c r="EB17" s="17">
-        <f>IFERROR(CL17-DG17,"")</f>
+        <f>IF(OR(CL17="",DG17=""),"",IFERROR(CL17-DG17,""))</f>
         <v/>
       </c>
       <c r="EC17" s="17">
-        <f>IFERROR(CM17-DH17,"")</f>
+        <f>IF(OR(CM17="",DH17=""),"",IFERROR(CM17-DH17,""))</f>
         <v/>
       </c>
       <c r="ED17" s="17">
-        <f>IFERROR(CN17-DI17,"")</f>
+        <f>IF(OR(CN17="",DI17=""),"",IFERROR(CN17-DI17,""))</f>
         <v/>
       </c>
       <c r="EE17" s="17">
-        <f>IFERROR(CO17-DJ17,"")</f>
+        <f>IF(OR(CO17="",DJ17=""),"",IFERROR(CO17-DJ17,""))</f>
         <v/>
       </c>
       <c r="EF17" s="17">
-        <f>IFERROR(CP17-DK17,"")</f>
+        <f>IF(OR(CP17="",DK17=""),"",IFERROR(CP17-DK17,""))</f>
         <v/>
       </c>
       <c r="EG17" s="17">
-        <f>IFERROR(CQ17-DL17,"")</f>
+        <f>IF(OR(CQ17="",DL17=""),"",IFERROR(CQ17-DL17,""))</f>
         <v/>
       </c>
       <c r="EH17" s="17">
-        <f>IFERROR(CR17-DM17,"")</f>
+        <f>IF(OR(CR17="",DM17=""),"",IFERROR(CR17-DM17,""))</f>
         <v/>
       </c>
       <c r="EI17" s="17">
-        <f>IFERROR(CS17-DN17,"")</f>
+        <f>IF(OR(CS17="",DN17=""),"",IFERROR(CS17-DN17,""))</f>
         <v/>
       </c>
       <c r="EJ17" s="17">
-        <f>IFERROR(CT17-DO17,"")</f>
+        <f>IF(OR(CT17="",DO17=""),"",IFERROR(CT17-DO17,""))</f>
         <v/>
       </c>
       <c r="EK17" s="17">
-        <f>IFERROR(CU17-DP17,"")</f>
+        <f>IF(OR(CU17="",DP17=""),"",IFERROR(CU17-DP17,""))</f>
         <v/>
       </c>
       <c r="EL17" s="17">
-        <f>IFERROR(CV17-DQ17,"")</f>
+        <f>IF(OR(CV17="",DQ17=""),"",IFERROR(CV17-DQ17,""))</f>
         <v/>
       </c>
       <c r="EM17" s="17">
-        <f>IFERROR(CW17-DR17,"")</f>
+        <f>IF(OR(CW17="",DR17=""),"",IFERROR(CW17-DR17,""))</f>
         <v/>
       </c>
       <c r="EN17" s="17">
-        <f>IFERROR(CX17-DS17,"")</f>
+        <f>IF(OR(CX17="",DS17=""),"",IFERROR(CX17-DS17,""))</f>
         <v/>
       </c>
       <c r="EO17" s="17">
-        <f>IFERROR(CY17-DT17,"")</f>
+        <f>IF(OR(CY17="",DT17=""),"",IFERROR(CY17-DT17,""))</f>
         <v/>
       </c>
       <c r="EP17" s="17">
-        <f>IFERROR(CZ17-DU17,"")</f>
+        <f>IF(OR(CZ17="",DU17=""),"",IFERROR(CZ17-DU17,""))</f>
         <v/>
       </c>
       <c r="EQ17" s="17">
-        <f>IFERROR(DA17-DV17,"")</f>
+        <f>IF(OR(DA17="",DV17=""),"",IFERROR(DA17-DV17,""))</f>
         <v/>
       </c>
       <c r="ER17" s="17">
-        <f>IFERROR(DB17-DW17,"")</f>
+        <f>IF(OR(DB17="",DW17=""),"",IFERROR(DB17-DW17,""))</f>
         <v/>
       </c>
       <c r="ES17" s="17">
-        <f>IFERROR(DC17-DX17,"")</f>
+        <f>IF(OR(DC17="",DX17=""),"",IFERROR(DC17-DX17,""))</f>
         <v/>
       </c>
       <c r="EU17" s="16" t="n"/>
@@ -4139,83 +4139,83 @@
       <c r="DW18" s="18" t="n"/>
       <c r="DX18" s="18" t="n"/>
       <c r="DZ18" s="17">
-        <f>IFERROR(CJ18-DE18,"")</f>
+        <f>IF(OR(CJ18="",DE18=""),"",IFERROR(CJ18-DE18,""))</f>
         <v/>
       </c>
       <c r="EA18" s="17">
-        <f>IFERROR(CK18-DF18,"")</f>
+        <f>IF(OR(CK18="",DF18=""),"",IFERROR(CK18-DF18,""))</f>
         <v/>
       </c>
       <c r="EB18" s="17">
-        <f>IFERROR(CL18-DG18,"")</f>
+        <f>IF(OR(CL18="",DG18=""),"",IFERROR(CL18-DG18,""))</f>
         <v/>
       </c>
       <c r="EC18" s="17">
-        <f>IFERROR(CM18-DH18,"")</f>
+        <f>IF(OR(CM18="",DH18=""),"",IFERROR(CM18-DH18,""))</f>
         <v/>
       </c>
       <c r="ED18" s="17">
-        <f>IFERROR(CN18-DI18,"")</f>
+        <f>IF(OR(CN18="",DI18=""),"",IFERROR(CN18-DI18,""))</f>
         <v/>
       </c>
       <c r="EE18" s="17">
-        <f>IFERROR(CO18-DJ18,"")</f>
+        <f>IF(OR(CO18="",DJ18=""),"",IFERROR(CO18-DJ18,""))</f>
         <v/>
       </c>
       <c r="EF18" s="17">
-        <f>IFERROR(CP18-DK18,"")</f>
+        <f>IF(OR(CP18="",DK18=""),"",IFERROR(CP18-DK18,""))</f>
         <v/>
       </c>
       <c r="EG18" s="17">
-        <f>IFERROR(CQ18-DL18,"")</f>
+        <f>IF(OR(CQ18="",DL18=""),"",IFERROR(CQ18-DL18,""))</f>
         <v/>
       </c>
       <c r="EH18" s="17">
-        <f>IFERROR(CR18-DM18,"")</f>
+        <f>IF(OR(CR18="",DM18=""),"",IFERROR(CR18-DM18,""))</f>
         <v/>
       </c>
       <c r="EI18" s="17">
-        <f>IFERROR(CS18-DN18,"")</f>
+        <f>IF(OR(CS18="",DN18=""),"",IFERROR(CS18-DN18,""))</f>
         <v/>
       </c>
       <c r="EJ18" s="17">
-        <f>IFERROR(CT18-DO18,"")</f>
+        <f>IF(OR(CT18="",DO18=""),"",IFERROR(CT18-DO18,""))</f>
         <v/>
       </c>
       <c r="EK18" s="17">
-        <f>IFERROR(CU18-DP18,"")</f>
+        <f>IF(OR(CU18="",DP18=""),"",IFERROR(CU18-DP18,""))</f>
         <v/>
       </c>
       <c r="EL18" s="17">
-        <f>IFERROR(CV18-DQ18,"")</f>
+        <f>IF(OR(CV18="",DQ18=""),"",IFERROR(CV18-DQ18,""))</f>
         <v/>
       </c>
       <c r="EM18" s="17">
-        <f>IFERROR(CW18-DR18,"")</f>
+        <f>IF(OR(CW18="",DR18=""),"",IFERROR(CW18-DR18,""))</f>
         <v/>
       </c>
       <c r="EN18" s="17">
-        <f>IFERROR(CX18-DS18,"")</f>
+        <f>IF(OR(CX18="",DS18=""),"",IFERROR(CX18-DS18,""))</f>
         <v/>
       </c>
       <c r="EO18" s="17">
-        <f>IFERROR(CY18-DT18,"")</f>
+        <f>IF(OR(CY18="",DT18=""),"",IFERROR(CY18-DT18,""))</f>
         <v/>
       </c>
       <c r="EP18" s="17">
-        <f>IFERROR(CZ18-DU18,"")</f>
+        <f>IF(OR(CZ18="",DU18=""),"",IFERROR(CZ18-DU18,""))</f>
         <v/>
       </c>
       <c r="EQ18" s="17">
-        <f>IFERROR(DA18-DV18,"")</f>
+        <f>IF(OR(DA18="",DV18=""),"",IFERROR(DA18-DV18,""))</f>
         <v/>
       </c>
       <c r="ER18" s="17">
-        <f>IFERROR(DB18-DW18,"")</f>
+        <f>IF(OR(DB18="",DW18=""),"",IFERROR(DB18-DW18,""))</f>
         <v/>
       </c>
       <c r="ES18" s="17">
-        <f>IFERROR(DC18-DX18,"")</f>
+        <f>IF(OR(DC18="",DX18=""),"",IFERROR(DC18-DX18,""))</f>
         <v/>
       </c>
       <c r="EU18" s="16" t="n"/>
@@ -4374,83 +4374,83 @@
       <c r="DW19" s="18" t="n"/>
       <c r="DX19" s="18" t="n"/>
       <c r="DZ19" s="17">
-        <f>IFERROR(CJ19-DE19,"")</f>
+        <f>IF(OR(CJ19="",DE19=""),"",IFERROR(CJ19-DE19,""))</f>
         <v/>
       </c>
       <c r="EA19" s="17">
-        <f>IFERROR(CK19-DF19,"")</f>
+        <f>IF(OR(CK19="",DF19=""),"",IFERROR(CK19-DF19,""))</f>
         <v/>
       </c>
       <c r="EB19" s="17">
-        <f>IFERROR(CL19-DG19,"")</f>
+        <f>IF(OR(CL19="",DG19=""),"",IFERROR(CL19-DG19,""))</f>
         <v/>
       </c>
       <c r="EC19" s="17">
-        <f>IFERROR(CM19-DH19,"")</f>
+        <f>IF(OR(CM19="",DH19=""),"",IFERROR(CM19-DH19,""))</f>
         <v/>
       </c>
       <c r="ED19" s="17">
-        <f>IFERROR(CN19-DI19,"")</f>
+        <f>IF(OR(CN19="",DI19=""),"",IFERROR(CN19-DI19,""))</f>
         <v/>
       </c>
       <c r="EE19" s="17">
-        <f>IFERROR(CO19-DJ19,"")</f>
+        <f>IF(OR(CO19="",DJ19=""),"",IFERROR(CO19-DJ19,""))</f>
         <v/>
       </c>
       <c r="EF19" s="17">
-        <f>IFERROR(CP19-DK19,"")</f>
+        <f>IF(OR(CP19="",DK19=""),"",IFERROR(CP19-DK19,""))</f>
         <v/>
       </c>
       <c r="EG19" s="17">
-        <f>IFERROR(CQ19-DL19,"")</f>
+        <f>IF(OR(CQ19="",DL19=""),"",IFERROR(CQ19-DL19,""))</f>
         <v/>
       </c>
       <c r="EH19" s="17">
-        <f>IFERROR(CR19-DM19,"")</f>
+        <f>IF(OR(CR19="",DM19=""),"",IFERROR(CR19-DM19,""))</f>
         <v/>
       </c>
       <c r="EI19" s="17">
-        <f>IFERROR(CS19-DN19,"")</f>
+        <f>IF(OR(CS19="",DN19=""),"",IFERROR(CS19-DN19,""))</f>
         <v/>
       </c>
       <c r="EJ19" s="17">
-        <f>IFERROR(CT19-DO19,"")</f>
+        <f>IF(OR(CT19="",DO19=""),"",IFERROR(CT19-DO19,""))</f>
         <v/>
       </c>
       <c r="EK19" s="17">
-        <f>IFERROR(CU19-DP19,"")</f>
+        <f>IF(OR(CU19="",DP19=""),"",IFERROR(CU19-DP19,""))</f>
         <v/>
       </c>
       <c r="EL19" s="17">
-        <f>IFERROR(CV19-DQ19,"")</f>
+        <f>IF(OR(CV19="",DQ19=""),"",IFERROR(CV19-DQ19,""))</f>
         <v/>
       </c>
       <c r="EM19" s="17">
-        <f>IFERROR(CW19-DR19,"")</f>
+        <f>IF(OR(CW19="",DR19=""),"",IFERROR(CW19-DR19,""))</f>
         <v/>
       </c>
       <c r="EN19" s="17">
-        <f>IFERROR(CX19-DS19,"")</f>
+        <f>IF(OR(CX19="",DS19=""),"",IFERROR(CX19-DS19,""))</f>
         <v/>
       </c>
       <c r="EO19" s="17">
-        <f>IFERROR(CY19-DT19,"")</f>
+        <f>IF(OR(CY19="",DT19=""),"",IFERROR(CY19-DT19,""))</f>
         <v/>
       </c>
       <c r="EP19" s="17">
-        <f>IFERROR(CZ19-DU19,"")</f>
+        <f>IF(OR(CZ19="",DU19=""),"",IFERROR(CZ19-DU19,""))</f>
         <v/>
       </c>
       <c r="EQ19" s="17">
-        <f>IFERROR(DA19-DV19,"")</f>
+        <f>IF(OR(DA19="",DV19=""),"",IFERROR(DA19-DV19,""))</f>
         <v/>
       </c>
       <c r="ER19" s="17">
-        <f>IFERROR(DB19-DW19,"")</f>
+        <f>IF(OR(DB19="",DW19=""),"",IFERROR(DB19-DW19,""))</f>
         <v/>
       </c>
       <c r="ES19" s="17">
-        <f>IFERROR(DC19-DX19,"")</f>
+        <f>IF(OR(DC19="",DX19=""),"",IFERROR(DC19-DX19,""))</f>
         <v/>
       </c>
       <c r="EU19" s="16" t="n"/>
@@ -4609,83 +4609,83 @@
       <c r="DW20" s="18" t="n"/>
       <c r="DX20" s="18" t="n"/>
       <c r="DZ20" s="17">
-        <f>IFERROR(CJ20-DE20,"")</f>
+        <f>IF(OR(CJ20="",DE20=""),"",IFERROR(CJ20-DE20,""))</f>
         <v/>
       </c>
       <c r="EA20" s="17">
-        <f>IFERROR(CK20-DF20,"")</f>
+        <f>IF(OR(CK20="",DF20=""),"",IFERROR(CK20-DF20,""))</f>
         <v/>
       </c>
       <c r="EB20" s="17">
-        <f>IFERROR(CL20-DG20,"")</f>
+        <f>IF(OR(CL20="",DG20=""),"",IFERROR(CL20-DG20,""))</f>
         <v/>
       </c>
       <c r="EC20" s="17">
-        <f>IFERROR(CM20-DH20,"")</f>
+        <f>IF(OR(CM20="",DH20=""),"",IFERROR(CM20-DH20,""))</f>
         <v/>
       </c>
       <c r="ED20" s="17">
-        <f>IFERROR(CN20-DI20,"")</f>
+        <f>IF(OR(CN20="",DI20=""),"",IFERROR(CN20-DI20,""))</f>
         <v/>
       </c>
       <c r="EE20" s="17">
-        <f>IFERROR(CO20-DJ20,"")</f>
+        <f>IF(OR(CO20="",DJ20=""),"",IFERROR(CO20-DJ20,""))</f>
         <v/>
       </c>
       <c r="EF20" s="17">
-        <f>IFERROR(CP20-DK20,"")</f>
+        <f>IF(OR(CP20="",DK20=""),"",IFERROR(CP20-DK20,""))</f>
         <v/>
       </c>
       <c r="EG20" s="17">
-        <f>IFERROR(CQ20-DL20,"")</f>
+        <f>IF(OR(CQ20="",DL20=""),"",IFERROR(CQ20-DL20,""))</f>
         <v/>
       </c>
       <c r="EH20" s="17">
-        <f>IFERROR(CR20-DM20,"")</f>
+        <f>IF(OR(CR20="",DM20=""),"",IFERROR(CR20-DM20,""))</f>
         <v/>
       </c>
       <c r="EI20" s="17">
-        <f>IFERROR(CS20-DN20,"")</f>
+        <f>IF(OR(CS20="",DN20=""),"",IFERROR(CS20-DN20,""))</f>
         <v/>
       </c>
       <c r="EJ20" s="17">
-        <f>IFERROR(CT20-DO20,"")</f>
+        <f>IF(OR(CT20="",DO20=""),"",IFERROR(CT20-DO20,""))</f>
         <v/>
       </c>
       <c r="EK20" s="17">
-        <f>IFERROR(CU20-DP20,"")</f>
+        <f>IF(OR(CU20="",DP20=""),"",IFERROR(CU20-DP20,""))</f>
         <v/>
       </c>
       <c r="EL20" s="17">
-        <f>IFERROR(CV20-DQ20,"")</f>
+        <f>IF(OR(CV20="",DQ20=""),"",IFERROR(CV20-DQ20,""))</f>
         <v/>
       </c>
       <c r="EM20" s="17">
-        <f>IFERROR(CW20-DR20,"")</f>
+        <f>IF(OR(CW20="",DR20=""),"",IFERROR(CW20-DR20,""))</f>
         <v/>
       </c>
       <c r="EN20" s="17">
-        <f>IFERROR(CX20-DS20,"")</f>
+        <f>IF(OR(CX20="",DS20=""),"",IFERROR(CX20-DS20,""))</f>
         <v/>
       </c>
       <c r="EO20" s="17">
-        <f>IFERROR(CY20-DT20,"")</f>
+        <f>IF(OR(CY20="",DT20=""),"",IFERROR(CY20-DT20,""))</f>
         <v/>
       </c>
       <c r="EP20" s="17">
-        <f>IFERROR(CZ20-DU20,"")</f>
+        <f>IF(OR(CZ20="",DU20=""),"",IFERROR(CZ20-DU20,""))</f>
         <v/>
       </c>
       <c r="EQ20" s="17">
-        <f>IFERROR(DA20-DV20,"")</f>
+        <f>IF(OR(DA20="",DV20=""),"",IFERROR(DA20-DV20,""))</f>
         <v/>
       </c>
       <c r="ER20" s="17">
-        <f>IFERROR(DB20-DW20,"")</f>
+        <f>IF(OR(DB20="",DW20=""),"",IFERROR(DB20-DW20,""))</f>
         <v/>
       </c>
       <c r="ES20" s="17">
-        <f>IFERROR(DC20-DX20,"")</f>
+        <f>IF(OR(DC20="",DX20=""),"",IFERROR(DC20-DX20,""))</f>
         <v/>
       </c>
       <c r="EU20" s="16" t="n"/>
@@ -4844,83 +4844,83 @@
       <c r="DW21" s="18" t="n"/>
       <c r="DX21" s="18" t="n"/>
       <c r="DZ21" s="17">
-        <f>IFERROR(CJ21-DE21,"")</f>
+        <f>IF(OR(CJ21="",DE21=""),"",IFERROR(CJ21-DE21,""))</f>
         <v/>
       </c>
       <c r="EA21" s="17">
-        <f>IFERROR(CK21-DF21,"")</f>
+        <f>IF(OR(CK21="",DF21=""),"",IFERROR(CK21-DF21,""))</f>
         <v/>
       </c>
       <c r="EB21" s="17">
-        <f>IFERROR(CL21-DG21,"")</f>
+        <f>IF(OR(CL21="",DG21=""),"",IFERROR(CL21-DG21,""))</f>
         <v/>
       </c>
       <c r="EC21" s="17">
-        <f>IFERROR(CM21-DH21,"")</f>
+        <f>IF(OR(CM21="",DH21=""),"",IFERROR(CM21-DH21,""))</f>
         <v/>
       </c>
       <c r="ED21" s="17">
-        <f>IFERROR(CN21-DI21,"")</f>
+        <f>IF(OR(CN21="",DI21=""),"",IFERROR(CN21-DI21,""))</f>
         <v/>
       </c>
       <c r="EE21" s="17">
-        <f>IFERROR(CO21-DJ21,"")</f>
+        <f>IF(OR(CO21="",DJ21=""),"",IFERROR(CO21-DJ21,""))</f>
         <v/>
       </c>
       <c r="EF21" s="17">
-        <f>IFERROR(CP21-DK21,"")</f>
+        <f>IF(OR(CP21="",DK21=""),"",IFERROR(CP21-DK21,""))</f>
         <v/>
       </c>
       <c r="EG21" s="17">
-        <f>IFERROR(CQ21-DL21,"")</f>
+        <f>IF(OR(CQ21="",DL21=""),"",IFERROR(CQ21-DL21,""))</f>
         <v/>
       </c>
       <c r="EH21" s="17">
-        <f>IFERROR(CR21-DM21,"")</f>
+        <f>IF(OR(CR21="",DM21=""),"",IFERROR(CR21-DM21,""))</f>
         <v/>
       </c>
       <c r="EI21" s="17">
-        <f>IFERROR(CS21-DN21,"")</f>
+        <f>IF(OR(CS21="",DN21=""),"",IFERROR(CS21-DN21,""))</f>
         <v/>
       </c>
       <c r="EJ21" s="17">
-        <f>IFERROR(CT21-DO21,"")</f>
+        <f>IF(OR(CT21="",DO21=""),"",IFERROR(CT21-DO21,""))</f>
         <v/>
       </c>
       <c r="EK21" s="17">
-        <f>IFERROR(CU21-DP21,"")</f>
+        <f>IF(OR(CU21="",DP21=""),"",IFERROR(CU21-DP21,""))</f>
         <v/>
       </c>
       <c r="EL21" s="17">
-        <f>IFERROR(CV21-DQ21,"")</f>
+        <f>IF(OR(CV21="",DQ21=""),"",IFERROR(CV21-DQ21,""))</f>
         <v/>
       </c>
       <c r="EM21" s="17">
-        <f>IFERROR(CW21-DR21,"")</f>
+        <f>IF(OR(CW21="",DR21=""),"",IFERROR(CW21-DR21,""))</f>
         <v/>
       </c>
       <c r="EN21" s="17">
-        <f>IFERROR(CX21-DS21,"")</f>
+        <f>IF(OR(CX21="",DS21=""),"",IFERROR(CX21-DS21,""))</f>
         <v/>
       </c>
       <c r="EO21" s="17">
-        <f>IFERROR(CY21-DT21,"")</f>
+        <f>IF(OR(CY21="",DT21=""),"",IFERROR(CY21-DT21,""))</f>
         <v/>
       </c>
       <c r="EP21" s="17">
-        <f>IFERROR(CZ21-DU21,"")</f>
+        <f>IF(OR(CZ21="",DU21=""),"",IFERROR(CZ21-DU21,""))</f>
         <v/>
       </c>
       <c r="EQ21" s="17">
-        <f>IFERROR(DA21-DV21,"")</f>
+        <f>IF(OR(DA21="",DV21=""),"",IFERROR(DA21-DV21,""))</f>
         <v/>
       </c>
       <c r="ER21" s="17">
-        <f>IFERROR(DB21-DW21,"")</f>
+        <f>IF(OR(DB21="",DW21=""),"",IFERROR(DB21-DW21,""))</f>
         <v/>
       </c>
       <c r="ES21" s="17">
-        <f>IFERROR(DC21-DX21,"")</f>
+        <f>IF(OR(DC21="",DX21=""),"",IFERROR(DC21-DX21,""))</f>
         <v/>
       </c>
       <c r="EU21" s="16" t="n"/>
@@ -5079,83 +5079,83 @@
       <c r="DW22" s="18" t="n"/>
       <c r="DX22" s="18" t="n"/>
       <c r="DZ22" s="17">
-        <f>IFERROR(CJ22-DE22,"")</f>
+        <f>IF(OR(CJ22="",DE22=""),"",IFERROR(CJ22-DE22,""))</f>
         <v/>
       </c>
       <c r="EA22" s="17">
-        <f>IFERROR(CK22-DF22,"")</f>
+        <f>IF(OR(CK22="",DF22=""),"",IFERROR(CK22-DF22,""))</f>
         <v/>
       </c>
       <c r="EB22" s="17">
-        <f>IFERROR(CL22-DG22,"")</f>
+        <f>IF(OR(CL22="",DG22=""),"",IFERROR(CL22-DG22,""))</f>
         <v/>
       </c>
       <c r="EC22" s="17">
-        <f>IFERROR(CM22-DH22,"")</f>
+        <f>IF(OR(CM22="",DH22=""),"",IFERROR(CM22-DH22,""))</f>
         <v/>
       </c>
       <c r="ED22" s="17">
-        <f>IFERROR(CN22-DI22,"")</f>
+        <f>IF(OR(CN22="",DI22=""),"",IFERROR(CN22-DI22,""))</f>
         <v/>
       </c>
       <c r="EE22" s="17">
-        <f>IFERROR(CO22-DJ22,"")</f>
+        <f>IF(OR(CO22="",DJ22=""),"",IFERROR(CO22-DJ22,""))</f>
         <v/>
       </c>
       <c r="EF22" s="17">
-        <f>IFERROR(CP22-DK22,"")</f>
+        <f>IF(OR(CP22="",DK22=""),"",IFERROR(CP22-DK22,""))</f>
         <v/>
       </c>
       <c r="EG22" s="17">
-        <f>IFERROR(CQ22-DL22,"")</f>
+        <f>IF(OR(CQ22="",DL22=""),"",IFERROR(CQ22-DL22,""))</f>
         <v/>
       </c>
       <c r="EH22" s="17">
-        <f>IFERROR(CR22-DM22,"")</f>
+        <f>IF(OR(CR22="",DM22=""),"",IFERROR(CR22-DM22,""))</f>
         <v/>
       </c>
       <c r="EI22" s="17">
-        <f>IFERROR(CS22-DN22,"")</f>
+        <f>IF(OR(CS22="",DN22=""),"",IFERROR(CS22-DN22,""))</f>
         <v/>
       </c>
       <c r="EJ22" s="17">
-        <f>IFERROR(CT22-DO22,"")</f>
+        <f>IF(OR(CT22="",DO22=""),"",IFERROR(CT22-DO22,""))</f>
         <v/>
       </c>
       <c r="EK22" s="17">
-        <f>IFERROR(CU22-DP22,"")</f>
+        <f>IF(OR(CU22="",DP22=""),"",IFERROR(CU22-DP22,""))</f>
         <v/>
       </c>
       <c r="EL22" s="17">
-        <f>IFERROR(CV22-DQ22,"")</f>
+        <f>IF(OR(CV22="",DQ22=""),"",IFERROR(CV22-DQ22,""))</f>
         <v/>
       </c>
       <c r="EM22" s="17">
-        <f>IFERROR(CW22-DR22,"")</f>
+        <f>IF(OR(CW22="",DR22=""),"",IFERROR(CW22-DR22,""))</f>
         <v/>
       </c>
       <c r="EN22" s="17">
-        <f>IFERROR(CX22-DS22,"")</f>
+        <f>IF(OR(CX22="",DS22=""),"",IFERROR(CX22-DS22,""))</f>
         <v/>
       </c>
       <c r="EO22" s="17">
-        <f>IFERROR(CY22-DT22,"")</f>
+        <f>IF(OR(CY22="",DT22=""),"",IFERROR(CY22-DT22,""))</f>
         <v/>
       </c>
       <c r="EP22" s="17">
-        <f>IFERROR(CZ22-DU22,"")</f>
+        <f>IF(OR(CZ22="",DU22=""),"",IFERROR(CZ22-DU22,""))</f>
         <v/>
       </c>
       <c r="EQ22" s="17">
-        <f>IFERROR(DA22-DV22,"")</f>
+        <f>IF(OR(DA22="",DV22=""),"",IFERROR(DA22-DV22,""))</f>
         <v/>
       </c>
       <c r="ER22" s="17">
-        <f>IFERROR(DB22-DW22,"")</f>
+        <f>IF(OR(DB22="",DW22=""),"",IFERROR(DB22-DW22,""))</f>
         <v/>
       </c>
       <c r="ES22" s="17">
-        <f>IFERROR(DC22-DX22,"")</f>
+        <f>IF(OR(DC22="",DX22=""),"",IFERROR(DC22-DX22,""))</f>
         <v/>
       </c>
       <c r="EU22" s="16" t="n"/>
@@ -5314,83 +5314,83 @@
       <c r="DW23" s="18" t="n"/>
       <c r="DX23" s="18" t="n"/>
       <c r="DZ23" s="17">
-        <f>IFERROR(CJ23-DE23,"")</f>
+        <f>IF(OR(CJ23="",DE23=""),"",IFERROR(CJ23-DE23,""))</f>
         <v/>
       </c>
       <c r="EA23" s="17">
-        <f>IFERROR(CK23-DF23,"")</f>
+        <f>IF(OR(CK23="",DF23=""),"",IFERROR(CK23-DF23,""))</f>
         <v/>
       </c>
       <c r="EB23" s="17">
-        <f>IFERROR(CL23-DG23,"")</f>
+        <f>IF(OR(CL23="",DG23=""),"",IFERROR(CL23-DG23,""))</f>
         <v/>
       </c>
       <c r="EC23" s="17">
-        <f>IFERROR(CM23-DH23,"")</f>
+        <f>IF(OR(CM23="",DH23=""),"",IFERROR(CM23-DH23,""))</f>
         <v/>
       </c>
       <c r="ED23" s="17">
-        <f>IFERROR(CN23-DI23,"")</f>
+        <f>IF(OR(CN23="",DI23=""),"",IFERROR(CN23-DI23,""))</f>
         <v/>
       </c>
       <c r="EE23" s="17">
-        <f>IFERROR(CO23-DJ23,"")</f>
+        <f>IF(OR(CO23="",DJ23=""),"",IFERROR(CO23-DJ23,""))</f>
         <v/>
       </c>
       <c r="EF23" s="17">
-        <f>IFERROR(CP23-DK23,"")</f>
+        <f>IF(OR(CP23="",DK23=""),"",IFERROR(CP23-DK23,""))</f>
         <v/>
       </c>
       <c r="EG23" s="17">
-        <f>IFERROR(CQ23-DL23,"")</f>
+        <f>IF(OR(CQ23="",DL23=""),"",IFERROR(CQ23-DL23,""))</f>
         <v/>
       </c>
       <c r="EH23" s="17">
-        <f>IFERROR(CR23-DM23,"")</f>
+        <f>IF(OR(CR23="",DM23=""),"",IFERROR(CR23-DM23,""))</f>
         <v/>
       </c>
       <c r="EI23" s="17">
-        <f>IFERROR(CS23-DN23,"")</f>
+        <f>IF(OR(CS23="",DN23=""),"",IFERROR(CS23-DN23,""))</f>
         <v/>
       </c>
       <c r="EJ23" s="17">
-        <f>IFERROR(CT23-DO23,"")</f>
+        <f>IF(OR(CT23="",DO23=""),"",IFERROR(CT23-DO23,""))</f>
         <v/>
       </c>
       <c r="EK23" s="17">
-        <f>IFERROR(CU23-DP23,"")</f>
+        <f>IF(OR(CU23="",DP23=""),"",IFERROR(CU23-DP23,""))</f>
         <v/>
       </c>
       <c r="EL23" s="17">
-        <f>IFERROR(CV23-DQ23,"")</f>
+        <f>IF(OR(CV23="",DQ23=""),"",IFERROR(CV23-DQ23,""))</f>
         <v/>
       </c>
       <c r="EM23" s="17">
-        <f>IFERROR(CW23-DR23,"")</f>
+        <f>IF(OR(CW23="",DR23=""),"",IFERROR(CW23-DR23,""))</f>
         <v/>
       </c>
       <c r="EN23" s="17">
-        <f>IFERROR(CX23-DS23,"")</f>
+        <f>IF(OR(CX23="",DS23=""),"",IFERROR(CX23-DS23,""))</f>
         <v/>
       </c>
       <c r="EO23" s="17">
-        <f>IFERROR(CY23-DT23,"")</f>
+        <f>IF(OR(CY23="",DT23=""),"",IFERROR(CY23-DT23,""))</f>
         <v/>
       </c>
       <c r="EP23" s="17">
-        <f>IFERROR(CZ23-DU23,"")</f>
+        <f>IF(OR(CZ23="",DU23=""),"",IFERROR(CZ23-DU23,""))</f>
         <v/>
       </c>
       <c r="EQ23" s="17">
-        <f>IFERROR(DA23-DV23,"")</f>
+        <f>IF(OR(DA23="",DV23=""),"",IFERROR(DA23-DV23,""))</f>
         <v/>
       </c>
       <c r="ER23" s="17">
-        <f>IFERROR(DB23-DW23,"")</f>
+        <f>IF(OR(DB23="",DW23=""),"",IFERROR(DB23-DW23,""))</f>
         <v/>
       </c>
       <c r="ES23" s="17">
-        <f>IFERROR(DC23-DX23,"")</f>
+        <f>IF(OR(DC23="",DX23=""),"",IFERROR(DC23-DX23,""))</f>
         <v/>
       </c>
       <c r="EU23" s="16" t="n"/>
@@ -5549,83 +5549,83 @@
       <c r="DW24" s="18" t="n"/>
       <c r="DX24" s="18" t="n"/>
       <c r="DZ24" s="17">
-        <f>IFERROR(CJ24-DE24,"")</f>
+        <f>IF(OR(CJ24="",DE24=""),"",IFERROR(CJ24-DE24,""))</f>
         <v/>
       </c>
       <c r="EA24" s="17">
-        <f>IFERROR(CK24-DF24,"")</f>
+        <f>IF(OR(CK24="",DF24=""),"",IFERROR(CK24-DF24,""))</f>
         <v/>
       </c>
       <c r="EB24" s="17">
-        <f>IFERROR(CL24-DG24,"")</f>
+        <f>IF(OR(CL24="",DG24=""),"",IFERROR(CL24-DG24,""))</f>
         <v/>
       </c>
       <c r="EC24" s="17">
-        <f>IFERROR(CM24-DH24,"")</f>
+        <f>IF(OR(CM24="",DH24=""),"",IFERROR(CM24-DH24,""))</f>
         <v/>
       </c>
       <c r="ED24" s="17">
-        <f>IFERROR(CN24-DI24,"")</f>
+        <f>IF(OR(CN24="",DI24=""),"",IFERROR(CN24-DI24,""))</f>
         <v/>
       </c>
       <c r="EE24" s="17">
-        <f>IFERROR(CO24-DJ24,"")</f>
+        <f>IF(OR(CO24="",DJ24=""),"",IFERROR(CO24-DJ24,""))</f>
         <v/>
       </c>
       <c r="EF24" s="17">
-        <f>IFERROR(CP24-DK24,"")</f>
+        <f>IF(OR(CP24="",DK24=""),"",IFERROR(CP24-DK24,""))</f>
         <v/>
       </c>
       <c r="EG24" s="17">
-        <f>IFERROR(CQ24-DL24,"")</f>
+        <f>IF(OR(CQ24="",DL24=""),"",IFERROR(CQ24-DL24,""))</f>
         <v/>
       </c>
       <c r="EH24" s="17">
-        <f>IFERROR(CR24-DM24,"")</f>
+        <f>IF(OR(CR24="",DM24=""),"",IFERROR(CR24-DM24,""))</f>
         <v/>
       </c>
       <c r="EI24" s="17">
-        <f>IFERROR(CS24-DN24,"")</f>
+        <f>IF(OR(CS24="",DN24=""),"",IFERROR(CS24-DN24,""))</f>
         <v/>
       </c>
       <c r="EJ24" s="17">
-        <f>IFERROR(CT24-DO24,"")</f>
+        <f>IF(OR(CT24="",DO24=""),"",IFERROR(CT24-DO24,""))</f>
         <v/>
       </c>
       <c r="EK24" s="17">
-        <f>IFERROR(CU24-DP24,"")</f>
+        <f>IF(OR(CU24="",DP24=""),"",IFERROR(CU24-DP24,""))</f>
         <v/>
       </c>
       <c r="EL24" s="17">
-        <f>IFERROR(CV24-DQ24,"")</f>
+        <f>IF(OR(CV24="",DQ24=""),"",IFERROR(CV24-DQ24,""))</f>
         <v/>
       </c>
       <c r="EM24" s="17">
-        <f>IFERROR(CW24-DR24,"")</f>
+        <f>IF(OR(CW24="",DR24=""),"",IFERROR(CW24-DR24,""))</f>
         <v/>
       </c>
       <c r="EN24" s="17">
-        <f>IFERROR(CX24-DS24,"")</f>
+        <f>IF(OR(CX24="",DS24=""),"",IFERROR(CX24-DS24,""))</f>
         <v/>
       </c>
       <c r="EO24" s="17">
-        <f>IFERROR(CY24-DT24,"")</f>
+        <f>IF(OR(CY24="",DT24=""),"",IFERROR(CY24-DT24,""))</f>
         <v/>
       </c>
       <c r="EP24" s="17">
-        <f>IFERROR(CZ24-DU24,"")</f>
+        <f>IF(OR(CZ24="",DU24=""),"",IFERROR(CZ24-DU24,""))</f>
         <v/>
       </c>
       <c r="EQ24" s="17">
-        <f>IFERROR(DA24-DV24,"")</f>
+        <f>IF(OR(DA24="",DV24=""),"",IFERROR(DA24-DV24,""))</f>
         <v/>
       </c>
       <c r="ER24" s="17">
-        <f>IFERROR(DB24-DW24,"")</f>
+        <f>IF(OR(DB24="",DW24=""),"",IFERROR(DB24-DW24,""))</f>
         <v/>
       </c>
       <c r="ES24" s="17">
-        <f>IFERROR(DC24-DX24,"")</f>
+        <f>IF(OR(DC24="",DX24=""),"",IFERROR(DC24-DX24,""))</f>
         <v/>
       </c>
       <c r="EU24" s="16" t="n"/>
@@ -5784,83 +5784,83 @@
       <c r="DW25" s="18" t="n"/>
       <c r="DX25" s="18" t="n"/>
       <c r="DZ25" s="17">
-        <f>IFERROR(CJ25-DE25,"")</f>
+        <f>IF(OR(CJ25="",DE25=""),"",IFERROR(CJ25-DE25,""))</f>
         <v/>
       </c>
       <c r="EA25" s="17">
-        <f>IFERROR(CK25-DF25,"")</f>
+        <f>IF(OR(CK25="",DF25=""),"",IFERROR(CK25-DF25,""))</f>
         <v/>
       </c>
       <c r="EB25" s="17">
-        <f>IFERROR(CL25-DG25,"")</f>
+        <f>IF(OR(CL25="",DG25=""),"",IFERROR(CL25-DG25,""))</f>
         <v/>
       </c>
       <c r="EC25" s="17">
-        <f>IFERROR(CM25-DH25,"")</f>
+        <f>IF(OR(CM25="",DH25=""),"",IFERROR(CM25-DH25,""))</f>
         <v/>
       </c>
       <c r="ED25" s="17">
-        <f>IFERROR(CN25-DI25,"")</f>
+        <f>IF(OR(CN25="",DI25=""),"",IFERROR(CN25-DI25,""))</f>
         <v/>
       </c>
       <c r="EE25" s="17">
-        <f>IFERROR(CO25-DJ25,"")</f>
+        <f>IF(OR(CO25="",DJ25=""),"",IFERROR(CO25-DJ25,""))</f>
         <v/>
       </c>
       <c r="EF25" s="17">
-        <f>IFERROR(CP25-DK25,"")</f>
+        <f>IF(OR(CP25="",DK25=""),"",IFERROR(CP25-DK25,""))</f>
         <v/>
       </c>
       <c r="EG25" s="17">
-        <f>IFERROR(CQ25-DL25,"")</f>
+        <f>IF(OR(CQ25="",DL25=""),"",IFERROR(CQ25-DL25,""))</f>
         <v/>
       </c>
       <c r="EH25" s="17">
-        <f>IFERROR(CR25-DM25,"")</f>
+        <f>IF(OR(CR25="",DM25=""),"",IFERROR(CR25-DM25,""))</f>
         <v/>
       </c>
       <c r="EI25" s="17">
-        <f>IFERROR(CS25-DN25,"")</f>
+        <f>IF(OR(CS25="",DN25=""),"",IFERROR(CS25-DN25,""))</f>
         <v/>
       </c>
       <c r="EJ25" s="17">
-        <f>IFERROR(CT25-DO25,"")</f>
+        <f>IF(OR(CT25="",DO25=""),"",IFERROR(CT25-DO25,""))</f>
         <v/>
       </c>
       <c r="EK25" s="17">
-        <f>IFERROR(CU25-DP25,"")</f>
+        <f>IF(OR(CU25="",DP25=""),"",IFERROR(CU25-DP25,""))</f>
         <v/>
       </c>
       <c r="EL25" s="17">
-        <f>IFERROR(CV25-DQ25,"")</f>
+        <f>IF(OR(CV25="",DQ25=""),"",IFERROR(CV25-DQ25,""))</f>
         <v/>
       </c>
       <c r="EM25" s="17">
-        <f>IFERROR(CW25-DR25,"")</f>
+        <f>IF(OR(CW25="",DR25=""),"",IFERROR(CW25-DR25,""))</f>
         <v/>
       </c>
       <c r="EN25" s="17">
-        <f>IFERROR(CX25-DS25,"")</f>
+        <f>IF(OR(CX25="",DS25=""),"",IFERROR(CX25-DS25,""))</f>
         <v/>
       </c>
       <c r="EO25" s="17">
-        <f>IFERROR(CY25-DT25,"")</f>
+        <f>IF(OR(CY25="",DT25=""),"",IFERROR(CY25-DT25,""))</f>
         <v/>
       </c>
       <c r="EP25" s="17">
-        <f>IFERROR(CZ25-DU25,"")</f>
+        <f>IF(OR(CZ25="",DU25=""),"",IFERROR(CZ25-DU25,""))</f>
         <v/>
       </c>
       <c r="EQ25" s="17">
-        <f>IFERROR(DA25-DV25,"")</f>
+        <f>IF(OR(DA25="",DV25=""),"",IFERROR(DA25-DV25,""))</f>
         <v/>
       </c>
       <c r="ER25" s="17">
-        <f>IFERROR(DB25-DW25,"")</f>
+        <f>IF(OR(DB25="",DW25=""),"",IFERROR(DB25-DW25,""))</f>
         <v/>
       </c>
       <c r="ES25" s="17">
-        <f>IFERROR(DC25-DX25,"")</f>
+        <f>IF(OR(DC25="",DX25=""),"",IFERROR(DC25-DX25,""))</f>
         <v/>
       </c>
       <c r="EU25" s="16" t="n"/>
@@ -6019,83 +6019,83 @@
       <c r="DW26" s="18" t="n"/>
       <c r="DX26" s="18" t="n"/>
       <c r="DZ26" s="17">
-        <f>IFERROR(CJ26-DE26,"")</f>
+        <f>IF(OR(CJ26="",DE26=""),"",IFERROR(CJ26-DE26,""))</f>
         <v/>
       </c>
       <c r="EA26" s="17">
-        <f>IFERROR(CK26-DF26,"")</f>
+        <f>IF(OR(CK26="",DF26=""),"",IFERROR(CK26-DF26,""))</f>
         <v/>
       </c>
       <c r="EB26" s="17">
-        <f>IFERROR(CL26-DG26,"")</f>
+        <f>IF(OR(CL26="",DG26=""),"",IFERROR(CL26-DG26,""))</f>
         <v/>
       </c>
       <c r="EC26" s="17">
-        <f>IFERROR(CM26-DH26,"")</f>
+        <f>IF(OR(CM26="",DH26=""),"",IFERROR(CM26-DH26,""))</f>
         <v/>
       </c>
       <c r="ED26" s="17">
-        <f>IFERROR(CN26-DI26,"")</f>
+        <f>IF(OR(CN26="",DI26=""),"",IFERROR(CN26-DI26,""))</f>
         <v/>
       </c>
       <c r="EE26" s="17">
-        <f>IFERROR(CO26-DJ26,"")</f>
+        <f>IF(OR(CO26="",DJ26=""),"",IFERROR(CO26-DJ26,""))</f>
         <v/>
       </c>
       <c r="EF26" s="17">
-        <f>IFERROR(CP26-DK26,"")</f>
+        <f>IF(OR(CP26="",DK26=""),"",IFERROR(CP26-DK26,""))</f>
         <v/>
       </c>
       <c r="EG26" s="17">
-        <f>IFERROR(CQ26-DL26,"")</f>
+        <f>IF(OR(CQ26="",DL26=""),"",IFERROR(CQ26-DL26,""))</f>
         <v/>
       </c>
       <c r="EH26" s="17">
-        <f>IFERROR(CR26-DM26,"")</f>
+        <f>IF(OR(CR26="",DM26=""),"",IFERROR(CR26-DM26,""))</f>
         <v/>
       </c>
       <c r="EI26" s="17">
-        <f>IFERROR(CS26-DN26,"")</f>
+        <f>IF(OR(CS26="",DN26=""),"",IFERROR(CS26-DN26,""))</f>
         <v/>
       </c>
       <c r="EJ26" s="17">
-        <f>IFERROR(CT26-DO26,"")</f>
+        <f>IF(OR(CT26="",DO26=""),"",IFERROR(CT26-DO26,""))</f>
         <v/>
       </c>
       <c r="EK26" s="17">
-        <f>IFERROR(CU26-DP26,"")</f>
+        <f>IF(OR(CU26="",DP26=""),"",IFERROR(CU26-DP26,""))</f>
         <v/>
       </c>
       <c r="EL26" s="17">
-        <f>IFERROR(CV26-DQ26,"")</f>
+        <f>IF(OR(CV26="",DQ26=""),"",IFERROR(CV26-DQ26,""))</f>
         <v/>
       </c>
       <c r="EM26" s="17">
-        <f>IFERROR(CW26-DR26,"")</f>
+        <f>IF(OR(CW26="",DR26=""),"",IFERROR(CW26-DR26,""))</f>
         <v/>
       </c>
       <c r="EN26" s="17">
-        <f>IFERROR(CX26-DS26,"")</f>
+        <f>IF(OR(CX26="",DS26=""),"",IFERROR(CX26-DS26,""))</f>
         <v/>
       </c>
       <c r="EO26" s="17">
-        <f>IFERROR(CY26-DT26,"")</f>
+        <f>IF(OR(CY26="",DT26=""),"",IFERROR(CY26-DT26,""))</f>
         <v/>
       </c>
       <c r="EP26" s="17">
-        <f>IFERROR(CZ26-DU26,"")</f>
+        <f>IF(OR(CZ26="",DU26=""),"",IFERROR(CZ26-DU26,""))</f>
         <v/>
       </c>
       <c r="EQ26" s="17">
-        <f>IFERROR(DA26-DV26,"")</f>
+        <f>IF(OR(DA26="",DV26=""),"",IFERROR(DA26-DV26,""))</f>
         <v/>
       </c>
       <c r="ER26" s="17">
-        <f>IFERROR(DB26-DW26,"")</f>
+        <f>IF(OR(DB26="",DW26=""),"",IFERROR(DB26-DW26,""))</f>
         <v/>
       </c>
       <c r="ES26" s="17">
-        <f>IFERROR(DC26-DX26,"")</f>
+        <f>IF(OR(DC26="",DX26=""),"",IFERROR(DC26-DX26,""))</f>
         <v/>
       </c>
       <c r="EU26" s="16" t="n"/>
@@ -6254,83 +6254,83 @@
       <c r="DW27" s="18" t="n"/>
       <c r="DX27" s="18" t="n"/>
       <c r="DZ27" s="17">
-        <f>IFERROR(CJ27-DE27,"")</f>
+        <f>IF(OR(CJ27="",DE27=""),"",IFERROR(CJ27-DE27,""))</f>
         <v/>
       </c>
       <c r="EA27" s="17">
-        <f>IFERROR(CK27-DF27,"")</f>
+        <f>IF(OR(CK27="",DF27=""),"",IFERROR(CK27-DF27,""))</f>
         <v/>
       </c>
       <c r="EB27" s="17">
-        <f>IFERROR(CL27-DG27,"")</f>
+        <f>IF(OR(CL27="",DG27=""),"",IFERROR(CL27-DG27,""))</f>
         <v/>
       </c>
       <c r="EC27" s="17">
-        <f>IFERROR(CM27-DH27,"")</f>
+        <f>IF(OR(CM27="",DH27=""),"",IFERROR(CM27-DH27,""))</f>
         <v/>
       </c>
       <c r="ED27" s="17">
-        <f>IFERROR(CN27-DI27,"")</f>
+        <f>IF(OR(CN27="",DI27=""),"",IFERROR(CN27-DI27,""))</f>
         <v/>
       </c>
       <c r="EE27" s="17">
-        <f>IFERROR(CO27-DJ27,"")</f>
+        <f>IF(OR(CO27="",DJ27=""),"",IFERROR(CO27-DJ27,""))</f>
         <v/>
       </c>
       <c r="EF27" s="17">
-        <f>IFERROR(CP27-DK27,"")</f>
+        <f>IF(OR(CP27="",DK27=""),"",IFERROR(CP27-DK27,""))</f>
         <v/>
       </c>
       <c r="EG27" s="17">
-        <f>IFERROR(CQ27-DL27,"")</f>
+        <f>IF(OR(CQ27="",DL27=""),"",IFERROR(CQ27-DL27,""))</f>
         <v/>
       </c>
       <c r="EH27" s="17">
-        <f>IFERROR(CR27-DM27,"")</f>
+        <f>IF(OR(CR27="",DM27=""),"",IFERROR(CR27-DM27,""))</f>
         <v/>
       </c>
       <c r="EI27" s="17">
-        <f>IFERROR(CS27-DN27,"")</f>
+        <f>IF(OR(CS27="",DN27=""),"",IFERROR(CS27-DN27,""))</f>
         <v/>
       </c>
       <c r="EJ27" s="17">
-        <f>IFERROR(CT27-DO27,"")</f>
+        <f>IF(OR(CT27="",DO27=""),"",IFERROR(CT27-DO27,""))</f>
         <v/>
       </c>
       <c r="EK27" s="17">
-        <f>IFERROR(CU27-DP27,"")</f>
+        <f>IF(OR(CU27="",DP27=""),"",IFERROR(CU27-DP27,""))</f>
         <v/>
       </c>
       <c r="EL27" s="17">
-        <f>IFERROR(CV27-DQ27,"")</f>
+        <f>IF(OR(CV27="",DQ27=""),"",IFERROR(CV27-DQ27,""))</f>
         <v/>
       </c>
       <c r="EM27" s="17">
-        <f>IFERROR(CW27-DR27,"")</f>
+        <f>IF(OR(CW27="",DR27=""),"",IFERROR(CW27-DR27,""))</f>
         <v/>
       </c>
       <c r="EN27" s="17">
-        <f>IFERROR(CX27-DS27,"")</f>
+        <f>IF(OR(CX27="",DS27=""),"",IFERROR(CX27-DS27,""))</f>
         <v/>
       </c>
       <c r="EO27" s="17">
-        <f>IFERROR(CY27-DT27,"")</f>
+        <f>IF(OR(CY27="",DT27=""),"",IFERROR(CY27-DT27,""))</f>
         <v/>
       </c>
       <c r="EP27" s="17">
-        <f>IFERROR(CZ27-DU27,"")</f>
+        <f>IF(OR(CZ27="",DU27=""),"",IFERROR(CZ27-DU27,""))</f>
         <v/>
       </c>
       <c r="EQ27" s="17">
-        <f>IFERROR(DA27-DV27,"")</f>
+        <f>IF(OR(DA27="",DV27=""),"",IFERROR(DA27-DV27,""))</f>
         <v/>
       </c>
       <c r="ER27" s="17">
-        <f>IFERROR(DB27-DW27,"")</f>
+        <f>IF(OR(DB27="",DW27=""),"",IFERROR(DB27-DW27,""))</f>
         <v/>
       </c>
       <c r="ES27" s="17">
-        <f>IFERROR(DC27-DX27,"")</f>
+        <f>IF(OR(DC27="",DX27=""),"",IFERROR(DC27-DX27,""))</f>
         <v/>
       </c>
       <c r="EU27" s="16" t="n"/>
@@ -6489,83 +6489,83 @@
       <c r="DW28" s="18" t="n"/>
       <c r="DX28" s="18" t="n"/>
       <c r="DZ28" s="17">
-        <f>IFERROR(CJ28-DE28,"")</f>
+        <f>IF(OR(CJ28="",DE28=""),"",IFERROR(CJ28-DE28,""))</f>
         <v/>
       </c>
       <c r="EA28" s="17">
-        <f>IFERROR(CK28-DF28,"")</f>
+        <f>IF(OR(CK28="",DF28=""),"",IFERROR(CK28-DF28,""))</f>
         <v/>
       </c>
       <c r="EB28" s="17">
-        <f>IFERROR(CL28-DG28,"")</f>
+        <f>IF(OR(CL28="",DG28=""),"",IFERROR(CL28-DG28,""))</f>
         <v/>
       </c>
       <c r="EC28" s="17">
-        <f>IFERROR(CM28-DH28,"")</f>
+        <f>IF(OR(CM28="",DH28=""),"",IFERROR(CM28-DH28,""))</f>
         <v/>
       </c>
       <c r="ED28" s="17">
-        <f>IFERROR(CN28-DI28,"")</f>
+        <f>IF(OR(CN28="",DI28=""),"",IFERROR(CN28-DI28,""))</f>
         <v/>
       </c>
       <c r="EE28" s="17">
-        <f>IFERROR(CO28-DJ28,"")</f>
+        <f>IF(OR(CO28="",DJ28=""),"",IFERROR(CO28-DJ28,""))</f>
         <v/>
       </c>
       <c r="EF28" s="17">
-        <f>IFERROR(CP28-DK28,"")</f>
+        <f>IF(OR(CP28="",DK28=""),"",IFERROR(CP28-DK28,""))</f>
         <v/>
       </c>
       <c r="EG28" s="17">
-        <f>IFERROR(CQ28-DL28,"")</f>
+        <f>IF(OR(CQ28="",DL28=""),"",IFERROR(CQ28-DL28,""))</f>
         <v/>
       </c>
       <c r="EH28" s="17">
-        <f>IFERROR(CR28-DM28,"")</f>
+        <f>IF(OR(CR28="",DM28=""),"",IFERROR(CR28-DM28,""))</f>
         <v/>
       </c>
       <c r="EI28" s="17">
-        <f>IFERROR(CS28-DN28,"")</f>
+        <f>IF(OR(CS28="",DN28=""),"",IFERROR(CS28-DN28,""))</f>
         <v/>
       </c>
       <c r="EJ28" s="17">
-        <f>IFERROR(CT28-DO28,"")</f>
+        <f>IF(OR(CT28="",DO28=""),"",IFERROR(CT28-DO28,""))</f>
         <v/>
       </c>
       <c r="EK28" s="17">
-        <f>IFERROR(CU28-DP28,"")</f>
+        <f>IF(OR(CU28="",DP28=""),"",IFERROR(CU28-DP28,""))</f>
         <v/>
       </c>
       <c r="EL28" s="17">
-        <f>IFERROR(CV28-DQ28,"")</f>
+        <f>IF(OR(CV28="",DQ28=""),"",IFERROR(CV28-DQ28,""))</f>
         <v/>
       </c>
       <c r="EM28" s="17">
-        <f>IFERROR(CW28-DR28,"")</f>
+        <f>IF(OR(CW28="",DR28=""),"",IFERROR(CW28-DR28,""))</f>
         <v/>
       </c>
       <c r="EN28" s="17">
-        <f>IFERROR(CX28-DS28,"")</f>
+        <f>IF(OR(CX28="",DS28=""),"",IFERROR(CX28-DS28,""))</f>
         <v/>
       </c>
       <c r="EO28" s="17">
-        <f>IFERROR(CY28-DT28,"")</f>
+        <f>IF(OR(CY28="",DT28=""),"",IFERROR(CY28-DT28,""))</f>
         <v/>
       </c>
       <c r="EP28" s="17">
-        <f>IFERROR(CZ28-DU28,"")</f>
+        <f>IF(OR(CZ28="",DU28=""),"",IFERROR(CZ28-DU28,""))</f>
         <v/>
       </c>
       <c r="EQ28" s="17">
-        <f>IFERROR(DA28-DV28,"")</f>
+        <f>IF(OR(DA28="",DV28=""),"",IFERROR(DA28-DV28,""))</f>
         <v/>
       </c>
       <c r="ER28" s="17">
-        <f>IFERROR(DB28-DW28,"")</f>
+        <f>IF(OR(DB28="",DW28=""),"",IFERROR(DB28-DW28,""))</f>
         <v/>
       </c>
       <c r="ES28" s="17">
-        <f>IFERROR(DC28-DX28,"")</f>
+        <f>IF(OR(DC28="",DX28=""),"",IFERROR(DC28-DX28,""))</f>
         <v/>
       </c>
       <c r="EU28" s="16" t="n"/>
@@ -6719,83 +6719,83 @@
       <c r="DW29" s="18" t="n"/>
       <c r="DX29" s="18" t="n"/>
       <c r="DZ29" s="17">
-        <f>IFERROR(CJ29-DE29,"")</f>
+        <f>IF(OR(CJ29="",DE29=""),"",IFERROR(CJ29-DE29,""))</f>
         <v/>
       </c>
       <c r="EA29" s="17">
-        <f>IFERROR(CK29-DF29,"")</f>
+        <f>IF(OR(CK29="",DF29=""),"",IFERROR(CK29-DF29,""))</f>
         <v/>
       </c>
       <c r="EB29" s="17">
-        <f>IFERROR(CL29-DG29,"")</f>
+        <f>IF(OR(CL29="",DG29=""),"",IFERROR(CL29-DG29,""))</f>
         <v/>
       </c>
       <c r="EC29" s="17">
-        <f>IFERROR(CM29-DH29,"")</f>
+        <f>IF(OR(CM29="",DH29=""),"",IFERROR(CM29-DH29,""))</f>
         <v/>
       </c>
       <c r="ED29" s="17">
-        <f>IFERROR(CN29-DI29,"")</f>
+        <f>IF(OR(CN29="",DI29=""),"",IFERROR(CN29-DI29,""))</f>
         <v/>
       </c>
       <c r="EE29" s="17">
-        <f>IFERROR(CO29-DJ29,"")</f>
+        <f>IF(OR(CO29="",DJ29=""),"",IFERROR(CO29-DJ29,""))</f>
         <v/>
       </c>
       <c r="EF29" s="17">
-        <f>IFERROR(CP29-DK29,"")</f>
+        <f>IF(OR(CP29="",DK29=""),"",IFERROR(CP29-DK29,""))</f>
         <v/>
       </c>
       <c r="EG29" s="17">
-        <f>IFERROR(CQ29-DL29,"")</f>
+        <f>IF(OR(CQ29="",DL29=""),"",IFERROR(CQ29-DL29,""))</f>
         <v/>
       </c>
       <c r="EH29" s="17">
-        <f>IFERROR(CR29-DM29,"")</f>
+        <f>IF(OR(CR29="",DM29=""),"",IFERROR(CR29-DM29,""))</f>
         <v/>
       </c>
       <c r="EI29" s="17">
-        <f>IFERROR(CS29-DN29,"")</f>
+        <f>IF(OR(CS29="",DN29=""),"",IFERROR(CS29-DN29,""))</f>
         <v/>
       </c>
       <c r="EJ29" s="17">
-        <f>IFERROR(CT29-DO29,"")</f>
+        <f>IF(OR(CT29="",DO29=""),"",IFERROR(CT29-DO29,""))</f>
         <v/>
       </c>
       <c r="EK29" s="17">
-        <f>IFERROR(CU29-DP29,"")</f>
+        <f>IF(OR(CU29="",DP29=""),"",IFERROR(CU29-DP29,""))</f>
         <v/>
       </c>
       <c r="EL29" s="17">
-        <f>IFERROR(CV29-DQ29,"")</f>
+        <f>IF(OR(CV29="",DQ29=""),"",IFERROR(CV29-DQ29,""))</f>
         <v/>
       </c>
       <c r="EM29" s="17">
-        <f>IFERROR(CW29-DR29,"")</f>
+        <f>IF(OR(CW29="",DR29=""),"",IFERROR(CW29-DR29,""))</f>
         <v/>
       </c>
       <c r="EN29" s="17">
-        <f>IFERROR(CX29-DS29,"")</f>
+        <f>IF(OR(CX29="",DS29=""),"",IFERROR(CX29-DS29,""))</f>
         <v/>
       </c>
       <c r="EO29" s="17">
-        <f>IFERROR(CY29-DT29,"")</f>
+        <f>IF(OR(CY29="",DT29=""),"",IFERROR(CY29-DT29,""))</f>
         <v/>
       </c>
       <c r="EP29" s="17">
-        <f>IFERROR(CZ29-DU29,"")</f>
+        <f>IF(OR(CZ29="",DU29=""),"",IFERROR(CZ29-DU29,""))</f>
         <v/>
       </c>
       <c r="EQ29" s="17">
-        <f>IFERROR(DA29-DV29,"")</f>
+        <f>IF(OR(DA29="",DV29=""),"",IFERROR(DA29-DV29,""))</f>
         <v/>
       </c>
       <c r="ER29" s="17">
-        <f>IFERROR(DB29-DW29,"")</f>
+        <f>IF(OR(DB29="",DW29=""),"",IFERROR(DB29-DW29,""))</f>
         <v/>
       </c>
       <c r="ES29" s="17">
-        <f>IFERROR(DC29-DX29,"")</f>
+        <f>IF(OR(DC29="",DX29=""),"",IFERROR(DC29-DX29,""))</f>
         <v/>
       </c>
       <c r="EU29" s="16" t="n"/>
@@ -6949,83 +6949,83 @@
       <c r="DW30" s="18" t="n"/>
       <c r="DX30" s="18" t="n"/>
       <c r="DZ30" s="17">
-        <f>IFERROR(CJ30-DE30,"")</f>
+        <f>IF(OR(CJ30="",DE30=""),"",IFERROR(CJ30-DE30,""))</f>
         <v/>
       </c>
       <c r="EA30" s="17">
-        <f>IFERROR(CK30-DF30,"")</f>
+        <f>IF(OR(CK30="",DF30=""),"",IFERROR(CK30-DF30,""))</f>
         <v/>
       </c>
       <c r="EB30" s="17">
-        <f>IFERROR(CL30-DG30,"")</f>
+        <f>IF(OR(CL30="",DG30=""),"",IFERROR(CL30-DG30,""))</f>
         <v/>
       </c>
       <c r="EC30" s="17">
-        <f>IFERROR(CM30-DH30,"")</f>
+        <f>IF(OR(CM30="",DH30=""),"",IFERROR(CM30-DH30,""))</f>
         <v/>
       </c>
       <c r="ED30" s="17">
-        <f>IFERROR(CN30-DI30,"")</f>
+        <f>IF(OR(CN30="",DI30=""),"",IFERROR(CN30-DI30,""))</f>
         <v/>
       </c>
       <c r="EE30" s="17">
-        <f>IFERROR(CO30-DJ30,"")</f>
+        <f>IF(OR(CO30="",DJ30=""),"",IFERROR(CO30-DJ30,""))</f>
         <v/>
       </c>
       <c r="EF30" s="17">
-        <f>IFERROR(CP30-DK30,"")</f>
+        <f>IF(OR(CP30="",DK30=""),"",IFERROR(CP30-DK30,""))</f>
         <v/>
       </c>
       <c r="EG30" s="17">
-        <f>IFERROR(CQ30-DL30,"")</f>
+        <f>IF(OR(CQ30="",DL30=""),"",IFERROR(CQ30-DL30,""))</f>
         <v/>
       </c>
       <c r="EH30" s="17">
-        <f>IFERROR(CR30-DM30,"")</f>
+        <f>IF(OR(CR30="",DM30=""),"",IFERROR(CR30-DM30,""))</f>
         <v/>
       </c>
       <c r="EI30" s="17">
-        <f>IFERROR(CS30-DN30,"")</f>
+        <f>IF(OR(CS30="",DN30=""),"",IFERROR(CS30-DN30,""))</f>
         <v/>
       </c>
       <c r="EJ30" s="17">
-        <f>IFERROR(CT30-DO30,"")</f>
+        <f>IF(OR(CT30="",DO30=""),"",IFERROR(CT30-DO30,""))</f>
         <v/>
       </c>
       <c r="EK30" s="17">
-        <f>IFERROR(CU30-DP30,"")</f>
+        <f>IF(OR(CU30="",DP30=""),"",IFERROR(CU30-DP30,""))</f>
         <v/>
       </c>
       <c r="EL30" s="17">
-        <f>IFERROR(CV30-DQ30,"")</f>
+        <f>IF(OR(CV30="",DQ30=""),"",IFERROR(CV30-DQ30,""))</f>
         <v/>
       </c>
       <c r="EM30" s="17">
-        <f>IFERROR(CW30-DR30,"")</f>
+        <f>IF(OR(CW30="",DR30=""),"",IFERROR(CW30-DR30,""))</f>
         <v/>
       </c>
       <c r="EN30" s="17">
-        <f>IFERROR(CX30-DS30,"")</f>
+        <f>IF(OR(CX30="",DS30=""),"",IFERROR(CX30-DS30,""))</f>
         <v/>
       </c>
       <c r="EO30" s="17">
-        <f>IFERROR(CY30-DT30,"")</f>
+        <f>IF(OR(CY30="",DT30=""),"",IFERROR(CY30-DT30,""))</f>
         <v/>
       </c>
       <c r="EP30" s="17">
-        <f>IFERROR(CZ30-DU30,"")</f>
+        <f>IF(OR(CZ30="",DU30=""),"",IFERROR(CZ30-DU30,""))</f>
         <v/>
       </c>
       <c r="EQ30" s="17">
-        <f>IFERROR(DA30-DV30,"")</f>
+        <f>IF(OR(DA30="",DV30=""),"",IFERROR(DA30-DV30,""))</f>
         <v/>
       </c>
       <c r="ER30" s="17">
-        <f>IFERROR(DB30-DW30,"")</f>
+        <f>IF(OR(DB30="",DW30=""),"",IFERROR(DB30-DW30,""))</f>
         <v/>
       </c>
       <c r="ES30" s="17">
-        <f>IFERROR(DC30-DX30,"")</f>
+        <f>IF(OR(DC30="",DX30=""),"",IFERROR(DC30-DX30,""))</f>
         <v/>
       </c>
       <c r="EU30" s="16" t="n"/>
@@ -7179,83 +7179,83 @@
       <c r="DW31" s="18" t="n"/>
       <c r="DX31" s="18" t="n"/>
       <c r="DZ31" s="17">
-        <f>IFERROR(CJ31-DE31,"")</f>
+        <f>IF(OR(CJ31="",DE31=""),"",IFERROR(CJ31-DE31,""))</f>
         <v/>
       </c>
       <c r="EA31" s="17">
-        <f>IFERROR(CK31-DF31,"")</f>
+        <f>IF(OR(CK31="",DF31=""),"",IFERROR(CK31-DF31,""))</f>
         <v/>
       </c>
       <c r="EB31" s="17">
-        <f>IFERROR(CL31-DG31,"")</f>
+        <f>IF(OR(CL31="",DG31=""),"",IFERROR(CL31-DG31,""))</f>
         <v/>
       </c>
       <c r="EC31" s="17">
-        <f>IFERROR(CM31-DH31,"")</f>
+        <f>IF(OR(CM31="",DH31=""),"",IFERROR(CM31-DH31,""))</f>
         <v/>
       </c>
       <c r="ED31" s="17">
-        <f>IFERROR(CN31-DI31,"")</f>
+        <f>IF(OR(CN31="",DI31=""),"",IFERROR(CN31-DI31,""))</f>
         <v/>
       </c>
       <c r="EE31" s="17">
-        <f>IFERROR(CO31-DJ31,"")</f>
+        <f>IF(OR(CO31="",DJ31=""),"",IFERROR(CO31-DJ31,""))</f>
         <v/>
       </c>
       <c r="EF31" s="17">
-        <f>IFERROR(CP31-DK31,"")</f>
+        <f>IF(OR(CP31="",DK31=""),"",IFERROR(CP31-DK31,""))</f>
         <v/>
       </c>
       <c r="EG31" s="17">
-        <f>IFERROR(CQ31-DL31,"")</f>
+        <f>IF(OR(CQ31="",DL31=""),"",IFERROR(CQ31-DL31,""))</f>
         <v/>
       </c>
       <c r="EH31" s="17">
-        <f>IFERROR(CR31-DM31,"")</f>
+        <f>IF(OR(CR31="",DM31=""),"",IFERROR(CR31-DM31,""))</f>
         <v/>
       </c>
       <c r="EI31" s="17">
-        <f>IFERROR(CS31-DN31,"")</f>
+        <f>IF(OR(CS31="",DN31=""),"",IFERROR(CS31-DN31,""))</f>
         <v/>
       </c>
       <c r="EJ31" s="17">
-        <f>IFERROR(CT31-DO31,"")</f>
+        <f>IF(OR(CT31="",DO31=""),"",IFERROR(CT31-DO31,""))</f>
         <v/>
       </c>
       <c r="EK31" s="17">
-        <f>IFERROR(CU31-DP31,"")</f>
+        <f>IF(OR(CU31="",DP31=""),"",IFERROR(CU31-DP31,""))</f>
         <v/>
       </c>
       <c r="EL31" s="17">
-        <f>IFERROR(CV31-DQ31,"")</f>
+        <f>IF(OR(CV31="",DQ31=""),"",IFERROR(CV31-DQ31,""))</f>
         <v/>
       </c>
       <c r="EM31" s="17">
-        <f>IFERROR(CW31-DR31,"")</f>
+        <f>IF(OR(CW31="",DR31=""),"",IFERROR(CW31-DR31,""))</f>
         <v/>
       </c>
       <c r="EN31" s="17">
-        <f>IFERROR(CX31-DS31,"")</f>
+        <f>IF(OR(CX31="",DS31=""),"",IFERROR(CX31-DS31,""))</f>
         <v/>
       </c>
       <c r="EO31" s="17">
-        <f>IFERROR(CY31-DT31,"")</f>
+        <f>IF(OR(CY31="",DT31=""),"",IFERROR(CY31-DT31,""))</f>
         <v/>
       </c>
       <c r="EP31" s="17">
-        <f>IFERROR(CZ31-DU31,"")</f>
+        <f>IF(OR(CZ31="",DU31=""),"",IFERROR(CZ31-DU31,""))</f>
         <v/>
       </c>
       <c r="EQ31" s="17">
-        <f>IFERROR(DA31-DV31,"")</f>
+        <f>IF(OR(DA31="",DV31=""),"",IFERROR(DA31-DV31,""))</f>
         <v/>
       </c>
       <c r="ER31" s="17">
-        <f>IFERROR(DB31-DW31,"")</f>
+        <f>IF(OR(DB31="",DW31=""),"",IFERROR(DB31-DW31,""))</f>
         <v/>
       </c>
       <c r="ES31" s="17">
-        <f>IFERROR(DC31-DX31,"")</f>
+        <f>IF(OR(DC31="",DX31=""),"",IFERROR(DC31-DX31,""))</f>
         <v/>
       </c>
       <c r="EU31" s="16" t="n"/>
@@ -7409,83 +7409,83 @@
       <c r="DW32" s="18" t="n"/>
       <c r="DX32" s="18" t="n"/>
       <c r="DZ32" s="17">
-        <f>IFERROR(CJ32-DE32,"")</f>
+        <f>IF(OR(CJ32="",DE32=""),"",IFERROR(CJ32-DE32,""))</f>
         <v/>
       </c>
       <c r="EA32" s="17">
-        <f>IFERROR(CK32-DF32,"")</f>
+        <f>IF(OR(CK32="",DF32=""),"",IFERROR(CK32-DF32,""))</f>
         <v/>
       </c>
       <c r="EB32" s="17">
-        <f>IFERROR(CL32-DG32,"")</f>
+        <f>IF(OR(CL32="",DG32=""),"",IFERROR(CL32-DG32,""))</f>
         <v/>
       </c>
       <c r="EC32" s="17">
-        <f>IFERROR(CM32-DH32,"")</f>
+        <f>IF(OR(CM32="",DH32=""),"",IFERROR(CM32-DH32,""))</f>
         <v/>
       </c>
       <c r="ED32" s="17">
-        <f>IFERROR(CN32-DI32,"")</f>
+        <f>IF(OR(CN32="",DI32=""),"",IFERROR(CN32-DI32,""))</f>
         <v/>
       </c>
       <c r="EE32" s="17">
-        <f>IFERROR(CO32-DJ32,"")</f>
+        <f>IF(OR(CO32="",DJ32=""),"",IFERROR(CO32-DJ32,""))</f>
         <v/>
       </c>
       <c r="EF32" s="17">
-        <f>IFERROR(CP32-DK32,"")</f>
+        <f>IF(OR(CP32="",DK32=""),"",IFERROR(CP32-DK32,""))</f>
         <v/>
       </c>
       <c r="EG32" s="17">
-        <f>IFERROR(CQ32-DL32,"")</f>
+        <f>IF(OR(CQ32="",DL32=""),"",IFERROR(CQ32-DL32,""))</f>
         <v/>
       </c>
       <c r="EH32" s="17">
-        <f>IFERROR(CR32-DM32,"")</f>
+        <f>IF(OR(CR32="",DM32=""),"",IFERROR(CR32-DM32,""))</f>
         <v/>
       </c>
       <c r="EI32" s="17">
-        <f>IFERROR(CS32-DN32,"")</f>
+        <f>IF(OR(CS32="",DN32=""),"",IFERROR(CS32-DN32,""))</f>
         <v/>
       </c>
       <c r="EJ32" s="17">
-        <f>IFERROR(CT32-DO32,"")</f>
+        <f>IF(OR(CT32="",DO32=""),"",IFERROR(CT32-DO32,""))</f>
         <v/>
       </c>
       <c r="EK32" s="17">
-        <f>IFERROR(CU32-DP32,"")</f>
+        <f>IF(OR(CU32="",DP32=""),"",IFERROR(CU32-DP32,""))</f>
         <v/>
       </c>
       <c r="EL32" s="17">
-        <f>IFERROR(CV32-DQ32,"")</f>
+        <f>IF(OR(CV32="",DQ32=""),"",IFERROR(CV32-DQ32,""))</f>
         <v/>
       </c>
       <c r="EM32" s="17">
-        <f>IFERROR(CW32-DR32,"")</f>
+        <f>IF(OR(CW32="",DR32=""),"",IFERROR(CW32-DR32,""))</f>
         <v/>
       </c>
       <c r="EN32" s="17">
-        <f>IFERROR(CX32-DS32,"")</f>
+        <f>IF(OR(CX32="",DS32=""),"",IFERROR(CX32-DS32,""))</f>
         <v/>
       </c>
       <c r="EO32" s="17">
-        <f>IFERROR(CY32-DT32,"")</f>
+        <f>IF(OR(CY32="",DT32=""),"",IFERROR(CY32-DT32,""))</f>
         <v/>
       </c>
       <c r="EP32" s="17">
-        <f>IFERROR(CZ32-DU32,"")</f>
+        <f>IF(OR(CZ32="",DU32=""),"",IFERROR(CZ32-DU32,""))</f>
         <v/>
       </c>
       <c r="EQ32" s="17">
-        <f>IFERROR(DA32-DV32,"")</f>
+        <f>IF(OR(DA32="",DV32=""),"",IFERROR(DA32-DV32,""))</f>
         <v/>
       </c>
       <c r="ER32" s="17">
-        <f>IFERROR(DB32-DW32,"")</f>
+        <f>IF(OR(DB32="",DW32=""),"",IFERROR(DB32-DW32,""))</f>
         <v/>
       </c>
       <c r="ES32" s="17">
-        <f>IFERROR(DC32-DX32,"")</f>
+        <f>IF(OR(DC32="",DX32=""),"",IFERROR(DC32-DX32,""))</f>
         <v/>
       </c>
       <c r="EU32" s="16" t="n"/>
@@ -7639,83 +7639,83 @@
       <c r="DW33" s="18" t="n"/>
       <c r="DX33" s="18" t="n"/>
       <c r="DZ33" s="17">
-        <f>IFERROR(CJ33-DE33,"")</f>
+        <f>IF(OR(CJ33="",DE33=""),"",IFERROR(CJ33-DE33,""))</f>
         <v/>
       </c>
       <c r="EA33" s="17">
-        <f>IFERROR(CK33-DF33,"")</f>
+        <f>IF(OR(CK33="",DF33=""),"",IFERROR(CK33-DF33,""))</f>
         <v/>
       </c>
       <c r="EB33" s="17">
-        <f>IFERROR(CL33-DG33,"")</f>
+        <f>IF(OR(CL33="",DG33=""),"",IFERROR(CL33-DG33,""))</f>
         <v/>
       </c>
       <c r="EC33" s="17">
-        <f>IFERROR(CM33-DH33,"")</f>
+        <f>IF(OR(CM33="",DH33=""),"",IFERROR(CM33-DH33,""))</f>
         <v/>
       </c>
       <c r="ED33" s="17">
-        <f>IFERROR(CN33-DI33,"")</f>
+        <f>IF(OR(CN33="",DI33=""),"",IFERROR(CN33-DI33,""))</f>
         <v/>
       </c>
       <c r="EE33" s="17">
-        <f>IFERROR(CO33-DJ33,"")</f>
+        <f>IF(OR(CO33="",DJ33=""),"",IFERROR(CO33-DJ33,""))</f>
         <v/>
       </c>
       <c r="EF33" s="17">
-        <f>IFERROR(CP33-DK33,"")</f>
+        <f>IF(OR(CP33="",DK33=""),"",IFERROR(CP33-DK33,""))</f>
         <v/>
       </c>
       <c r="EG33" s="17">
-        <f>IFERROR(CQ33-DL33,"")</f>
+        <f>IF(OR(CQ33="",DL33=""),"",IFERROR(CQ33-DL33,""))</f>
         <v/>
       </c>
       <c r="EH33" s="17">
-        <f>IFERROR(CR33-DM33,"")</f>
+        <f>IF(OR(CR33="",DM33=""),"",IFERROR(CR33-DM33,""))</f>
         <v/>
       </c>
       <c r="EI33" s="17">
-        <f>IFERROR(CS33-DN33,"")</f>
+        <f>IF(OR(CS33="",DN33=""),"",IFERROR(CS33-DN33,""))</f>
         <v/>
       </c>
       <c r="EJ33" s="17">
-        <f>IFERROR(CT33-DO33,"")</f>
+        <f>IF(OR(CT33="",DO33=""),"",IFERROR(CT33-DO33,""))</f>
         <v/>
       </c>
       <c r="EK33" s="17">
-        <f>IFERROR(CU33-DP33,"")</f>
+        <f>IF(OR(CU33="",DP33=""),"",IFERROR(CU33-DP33,""))</f>
         <v/>
       </c>
       <c r="EL33" s="17">
-        <f>IFERROR(CV33-DQ33,"")</f>
+        <f>IF(OR(CV33="",DQ33=""),"",IFERROR(CV33-DQ33,""))</f>
         <v/>
       </c>
       <c r="EM33" s="17">
-        <f>IFERROR(CW33-DR33,"")</f>
+        <f>IF(OR(CW33="",DR33=""),"",IFERROR(CW33-DR33,""))</f>
         <v/>
       </c>
       <c r="EN33" s="17">
-        <f>IFERROR(CX33-DS33,"")</f>
+        <f>IF(OR(CX33="",DS33=""),"",IFERROR(CX33-DS33,""))</f>
         <v/>
       </c>
       <c r="EO33" s="17">
-        <f>IFERROR(CY33-DT33,"")</f>
+        <f>IF(OR(CY33="",DT33=""),"",IFERROR(CY33-DT33,""))</f>
         <v/>
       </c>
       <c r="EP33" s="17">
-        <f>IFERROR(CZ33-DU33,"")</f>
+        <f>IF(OR(CZ33="",DU33=""),"",IFERROR(CZ33-DU33,""))</f>
         <v/>
       </c>
       <c r="EQ33" s="17">
-        <f>IFERROR(DA33-DV33,"")</f>
+        <f>IF(OR(DA33="",DV33=""),"",IFERROR(DA33-DV33,""))</f>
         <v/>
       </c>
       <c r="ER33" s="17">
-        <f>IFERROR(DB33-DW33,"")</f>
+        <f>IF(OR(DB33="",DW33=""),"",IFERROR(DB33-DW33,""))</f>
         <v/>
       </c>
       <c r="ES33" s="17">
-        <f>IFERROR(DC33-DX33,"")</f>
+        <f>IF(OR(DC33="",DX33=""),"",IFERROR(DC33-DX33,""))</f>
         <v/>
       </c>
       <c r="EU33" s="16" t="n"/>
@@ -7869,83 +7869,83 @@
       <c r="DW34" s="18" t="n"/>
       <c r="DX34" s="18" t="n"/>
       <c r="DZ34" s="17">
-        <f>IFERROR(CJ34-DE34,"")</f>
+        <f>IF(OR(CJ34="",DE34=""),"",IFERROR(CJ34-DE34,""))</f>
         <v/>
       </c>
       <c r="EA34" s="17">
-        <f>IFERROR(CK34-DF34,"")</f>
+        <f>IF(OR(CK34="",DF34=""),"",IFERROR(CK34-DF34,""))</f>
         <v/>
       </c>
       <c r="EB34" s="17">
-        <f>IFERROR(CL34-DG34,"")</f>
+        <f>IF(OR(CL34="",DG34=""),"",IFERROR(CL34-DG34,""))</f>
         <v/>
       </c>
       <c r="EC34" s="17">
-        <f>IFERROR(CM34-DH34,"")</f>
+        <f>IF(OR(CM34="",DH34=""),"",IFERROR(CM34-DH34,""))</f>
         <v/>
       </c>
       <c r="ED34" s="17">
-        <f>IFERROR(CN34-DI34,"")</f>
+        <f>IF(OR(CN34="",DI34=""),"",IFERROR(CN34-DI34,""))</f>
         <v/>
       </c>
       <c r="EE34" s="17">
-        <f>IFERROR(CO34-DJ34,"")</f>
+        <f>IF(OR(CO34="",DJ34=""),"",IFERROR(CO34-DJ34,""))</f>
         <v/>
       </c>
       <c r="EF34" s="17">
-        <f>IFERROR(CP34-DK34,"")</f>
+        <f>IF(OR(CP34="",DK34=""),"",IFERROR(CP34-DK34,""))</f>
         <v/>
       </c>
       <c r="EG34" s="17">
-        <f>IFERROR(CQ34-DL34,"")</f>
+        <f>IF(OR(CQ34="",DL34=""),"",IFERROR(CQ34-DL34,""))</f>
         <v/>
       </c>
       <c r="EH34" s="17">
-        <f>IFERROR(CR34-DM34,"")</f>
+        <f>IF(OR(CR34="",DM34=""),"",IFERROR(CR34-DM34,""))</f>
         <v/>
       </c>
       <c r="EI34" s="17">
-        <f>IFERROR(CS34-DN34,"")</f>
+        <f>IF(OR(CS34="",DN34=""),"",IFERROR(CS34-DN34,""))</f>
         <v/>
       </c>
       <c r="EJ34" s="17">
-        <f>IFERROR(CT34-DO34,"")</f>
+        <f>IF(OR(CT34="",DO34=""),"",IFERROR(CT34-DO34,""))</f>
         <v/>
       </c>
       <c r="EK34" s="17">
-        <f>IFERROR(CU34-DP34,"")</f>
+        <f>IF(OR(CU34="",DP34=""),"",IFERROR(CU34-DP34,""))</f>
         <v/>
       </c>
       <c r="EL34" s="17">
-        <f>IFERROR(CV34-DQ34,"")</f>
+        <f>IF(OR(CV34="",DQ34=""),"",IFERROR(CV34-DQ34,""))</f>
         <v/>
       </c>
       <c r="EM34" s="17">
-        <f>IFERROR(CW34-DR34,"")</f>
+        <f>IF(OR(CW34="",DR34=""),"",IFERROR(CW34-DR34,""))</f>
         <v/>
       </c>
       <c r="EN34" s="17">
-        <f>IFERROR(CX34-DS34,"")</f>
+        <f>IF(OR(CX34="",DS34=""),"",IFERROR(CX34-DS34,""))</f>
         <v/>
       </c>
       <c r="EO34" s="17">
-        <f>IFERROR(CY34-DT34,"")</f>
+        <f>IF(OR(CY34="",DT34=""),"",IFERROR(CY34-DT34,""))</f>
         <v/>
       </c>
       <c r="EP34" s="17">
-        <f>IFERROR(CZ34-DU34,"")</f>
+        <f>IF(OR(CZ34="",DU34=""),"",IFERROR(CZ34-DU34,""))</f>
         <v/>
       </c>
       <c r="EQ34" s="17">
-        <f>IFERROR(DA34-DV34,"")</f>
+        <f>IF(OR(DA34="",DV34=""),"",IFERROR(DA34-DV34,""))</f>
         <v/>
       </c>
       <c r="ER34" s="17">
-        <f>IFERROR(DB34-DW34,"")</f>
+        <f>IF(OR(DB34="",DW34=""),"",IFERROR(DB34-DW34,""))</f>
         <v/>
       </c>
       <c r="ES34" s="17">
-        <f>IFERROR(DC34-DX34,"")</f>
+        <f>IF(OR(DC34="",DX34=""),"",IFERROR(DC34-DX34,""))</f>
         <v/>
       </c>
       <c r="EU34" s="16" t="n"/>
@@ -8099,83 +8099,83 @@
       <c r="DW35" s="18" t="n"/>
       <c r="DX35" s="18" t="n"/>
       <c r="DZ35" s="17">
-        <f>IFERROR(CJ35-DE35,"")</f>
+        <f>IF(OR(CJ35="",DE35=""),"",IFERROR(CJ35-DE35,""))</f>
         <v/>
       </c>
       <c r="EA35" s="17">
-        <f>IFERROR(CK35-DF35,"")</f>
+        <f>IF(OR(CK35="",DF35=""),"",IFERROR(CK35-DF35,""))</f>
         <v/>
       </c>
       <c r="EB35" s="17">
-        <f>IFERROR(CL35-DG35,"")</f>
+        <f>IF(OR(CL35="",DG35=""),"",IFERROR(CL35-DG35,""))</f>
         <v/>
       </c>
       <c r="EC35" s="17">
-        <f>IFERROR(CM35-DH35,"")</f>
+        <f>IF(OR(CM35="",DH35=""),"",IFERROR(CM35-DH35,""))</f>
         <v/>
       </c>
       <c r="ED35" s="17">
-        <f>IFERROR(CN35-DI35,"")</f>
+        <f>IF(OR(CN35="",DI35=""),"",IFERROR(CN35-DI35,""))</f>
         <v/>
       </c>
       <c r="EE35" s="17">
-        <f>IFERROR(CO35-DJ35,"")</f>
+        <f>IF(OR(CO35="",DJ35=""),"",IFERROR(CO35-DJ35,""))</f>
         <v/>
       </c>
       <c r="EF35" s="17">
-        <f>IFERROR(CP35-DK35,"")</f>
+        <f>IF(OR(CP35="",DK35=""),"",IFERROR(CP35-DK35,""))</f>
         <v/>
       </c>
       <c r="EG35" s="17">
-        <f>IFERROR(CQ35-DL35,"")</f>
+        <f>IF(OR(CQ35="",DL35=""),"",IFERROR(CQ35-DL35,""))</f>
         <v/>
       </c>
       <c r="EH35" s="17">
-        <f>IFERROR(CR35-DM35,"")</f>
+        <f>IF(OR(CR35="",DM35=""),"",IFERROR(CR35-DM35,""))</f>
         <v/>
       </c>
       <c r="EI35" s="17">
-        <f>IFERROR(CS35-DN35,"")</f>
+        <f>IF(OR(CS35="",DN35=""),"",IFERROR(CS35-DN35,""))</f>
         <v/>
       </c>
       <c r="EJ35" s="17">
-        <f>IFERROR(CT35-DO35,"")</f>
+        <f>IF(OR(CT35="",DO35=""),"",IFERROR(CT35-DO35,""))</f>
         <v/>
       </c>
       <c r="EK35" s="17">
-        <f>IFERROR(CU35-DP35,"")</f>
+        <f>IF(OR(CU35="",DP35=""),"",IFERROR(CU35-DP35,""))</f>
         <v/>
       </c>
       <c r="EL35" s="17">
-        <f>IFERROR(CV35-DQ35,"")</f>
+        <f>IF(OR(CV35="",DQ35=""),"",IFERROR(CV35-DQ35,""))</f>
         <v/>
       </c>
       <c r="EM35" s="17">
-        <f>IFERROR(CW35-DR35,"")</f>
+        <f>IF(OR(CW35="",DR35=""),"",IFERROR(CW35-DR35,""))</f>
         <v/>
       </c>
       <c r="EN35" s="17">
-        <f>IFERROR(CX35-DS35,"")</f>
+        <f>IF(OR(CX35="",DS35=""),"",IFERROR(CX35-DS35,""))</f>
         <v/>
       </c>
       <c r="EO35" s="17">
-        <f>IFERROR(CY35-DT35,"")</f>
+        <f>IF(OR(CY35="",DT35=""),"",IFERROR(CY35-DT35,""))</f>
         <v/>
       </c>
       <c r="EP35" s="17">
-        <f>IFERROR(CZ35-DU35,"")</f>
+        <f>IF(OR(CZ35="",DU35=""),"",IFERROR(CZ35-DU35,""))</f>
         <v/>
       </c>
       <c r="EQ35" s="17">
-        <f>IFERROR(DA35-DV35,"")</f>
+        <f>IF(OR(DA35="",DV35=""),"",IFERROR(DA35-DV35,""))</f>
         <v/>
       </c>
       <c r="ER35" s="17">
-        <f>IFERROR(DB35-DW35,"")</f>
+        <f>IF(OR(DB35="",DW35=""),"",IFERROR(DB35-DW35,""))</f>
         <v/>
       </c>
       <c r="ES35" s="17">
-        <f>IFERROR(DC35-DX35,"")</f>
+        <f>IF(OR(DC35="",DX35=""),"",IFERROR(DC35-DX35,""))</f>
         <v/>
       </c>
       <c r="EU35" s="16" t="n"/>
@@ -8329,83 +8329,83 @@
       <c r="DW36" s="18" t="n"/>
       <c r="DX36" s="18" t="n"/>
       <c r="DZ36" s="17">
-        <f>IFERROR(CJ36-DE36,"")</f>
+        <f>IF(OR(CJ36="",DE36=""),"",IFERROR(CJ36-DE36,""))</f>
         <v/>
       </c>
       <c r="EA36" s="17">
-        <f>IFERROR(CK36-DF36,"")</f>
+        <f>IF(OR(CK36="",DF36=""),"",IFERROR(CK36-DF36,""))</f>
         <v/>
       </c>
       <c r="EB36" s="17">
-        <f>IFERROR(CL36-DG36,"")</f>
+        <f>IF(OR(CL36="",DG36=""),"",IFERROR(CL36-DG36,""))</f>
         <v/>
       </c>
       <c r="EC36" s="17">
-        <f>IFERROR(CM36-DH36,"")</f>
+        <f>IF(OR(CM36="",DH36=""),"",IFERROR(CM36-DH36,""))</f>
         <v/>
       </c>
       <c r="ED36" s="17">
-        <f>IFERROR(CN36-DI36,"")</f>
+        <f>IF(OR(CN36="",DI36=""),"",IFERROR(CN36-DI36,""))</f>
         <v/>
       </c>
       <c r="EE36" s="17">
-        <f>IFERROR(CO36-DJ36,"")</f>
+        <f>IF(OR(CO36="",DJ36=""),"",IFERROR(CO36-DJ36,""))</f>
         <v/>
       </c>
       <c r="EF36" s="17">
-        <f>IFERROR(CP36-DK36,"")</f>
+        <f>IF(OR(CP36="",DK36=""),"",IFERROR(CP36-DK36,""))</f>
         <v/>
       </c>
       <c r="EG36" s="17">
-        <f>IFERROR(CQ36-DL36,"")</f>
+        <f>IF(OR(CQ36="",DL36=""),"",IFERROR(CQ36-DL36,""))</f>
         <v/>
       </c>
       <c r="EH36" s="17">
-        <f>IFERROR(CR36-DM36,"")</f>
+        <f>IF(OR(CR36="",DM36=""),"",IFERROR(CR36-DM36,""))</f>
         <v/>
       </c>
       <c r="EI36" s="17">
-        <f>IFERROR(CS36-DN36,"")</f>
+        <f>IF(OR(CS36="",DN36=""),"",IFERROR(CS36-DN36,""))</f>
         <v/>
       </c>
       <c r="EJ36" s="17">
-        <f>IFERROR(CT36-DO36,"")</f>
+        <f>IF(OR(CT36="",DO36=""),"",IFERROR(CT36-DO36,""))</f>
         <v/>
       </c>
       <c r="EK36" s="17">
-        <f>IFERROR(CU36-DP36,"")</f>
+        <f>IF(OR(CU36="",DP36=""),"",IFERROR(CU36-DP36,""))</f>
         <v/>
       </c>
       <c r="EL36" s="17">
-        <f>IFERROR(CV36-DQ36,"")</f>
+        <f>IF(OR(CV36="",DQ36=""),"",IFERROR(CV36-DQ36,""))</f>
         <v/>
       </c>
       <c r="EM36" s="17">
-        <f>IFERROR(CW36-DR36,"")</f>
+        <f>IF(OR(CW36="",DR36=""),"",IFERROR(CW36-DR36,""))</f>
         <v/>
       </c>
       <c r="EN36" s="17">
-        <f>IFERROR(CX36-DS36,"")</f>
+        <f>IF(OR(CX36="",DS36=""),"",IFERROR(CX36-DS36,""))</f>
         <v/>
       </c>
       <c r="EO36" s="17">
-        <f>IFERROR(CY36-DT36,"")</f>
+        <f>IF(OR(CY36="",DT36=""),"",IFERROR(CY36-DT36,""))</f>
         <v/>
       </c>
       <c r="EP36" s="17">
-        <f>IFERROR(CZ36-DU36,"")</f>
+        <f>IF(OR(CZ36="",DU36=""),"",IFERROR(CZ36-DU36,""))</f>
         <v/>
       </c>
       <c r="EQ36" s="17">
-        <f>IFERROR(DA36-DV36,"")</f>
+        <f>IF(OR(DA36="",DV36=""),"",IFERROR(DA36-DV36,""))</f>
         <v/>
       </c>
       <c r="ER36" s="17">
-        <f>IFERROR(DB36-DW36,"")</f>
+        <f>IF(OR(DB36="",DW36=""),"",IFERROR(DB36-DW36,""))</f>
         <v/>
       </c>
       <c r="ES36" s="17">
-        <f>IFERROR(DC36-DX36,"")</f>
+        <f>IF(OR(DC36="",DX36=""),"",IFERROR(DC36-DX36,""))</f>
         <v/>
       </c>
       <c r="EU36" s="16" t="n"/>
@@ -8559,83 +8559,83 @@
       <c r="DW37" s="18" t="n"/>
       <c r="DX37" s="18" t="n"/>
       <c r="DZ37" s="17">
-        <f>IFERROR(CJ37-DE37,"")</f>
+        <f>IF(OR(CJ37="",DE37=""),"",IFERROR(CJ37-DE37,""))</f>
         <v/>
       </c>
       <c r="EA37" s="17">
-        <f>IFERROR(CK37-DF37,"")</f>
+        <f>IF(OR(CK37="",DF37=""),"",IFERROR(CK37-DF37,""))</f>
         <v/>
       </c>
       <c r="EB37" s="17">
-        <f>IFERROR(CL37-DG37,"")</f>
+        <f>IF(OR(CL37="",DG37=""),"",IFERROR(CL37-DG37,""))</f>
         <v/>
       </c>
       <c r="EC37" s="17">
-        <f>IFERROR(CM37-DH37,"")</f>
+        <f>IF(OR(CM37="",DH37=""),"",IFERROR(CM37-DH37,""))</f>
         <v/>
       </c>
       <c r="ED37" s="17">
-        <f>IFERROR(CN37-DI37,"")</f>
+        <f>IF(OR(CN37="",DI37=""),"",IFERROR(CN37-DI37,""))</f>
         <v/>
       </c>
       <c r="EE37" s="17">
-        <f>IFERROR(CO37-DJ37,"")</f>
+        <f>IF(OR(CO37="",DJ37=""),"",IFERROR(CO37-DJ37,""))</f>
         <v/>
       </c>
       <c r="EF37" s="17">
-        <f>IFERROR(CP37-DK37,"")</f>
+        <f>IF(OR(CP37="",DK37=""),"",IFERROR(CP37-DK37,""))</f>
         <v/>
       </c>
       <c r="EG37" s="17">
-        <f>IFERROR(CQ37-DL37,"")</f>
+        <f>IF(OR(CQ37="",DL37=""),"",IFERROR(CQ37-DL37,""))</f>
         <v/>
       </c>
       <c r="EH37" s="17">
-        <f>IFERROR(CR37-DM37,"")</f>
+        <f>IF(OR(CR37="",DM37=""),"",IFERROR(CR37-DM37,""))</f>
         <v/>
       </c>
       <c r="EI37" s="17">
-        <f>IFERROR(CS37-DN37,"")</f>
+        <f>IF(OR(CS37="",DN37=""),"",IFERROR(CS37-DN37,""))</f>
         <v/>
       </c>
       <c r="EJ37" s="17">
-        <f>IFERROR(CT37-DO37,"")</f>
+        <f>IF(OR(CT37="",DO37=""),"",IFERROR(CT37-DO37,""))</f>
         <v/>
       </c>
       <c r="EK37" s="17">
-        <f>IFERROR(CU37-DP37,"")</f>
+        <f>IF(OR(CU37="",DP37=""),"",IFERROR(CU37-DP37,""))</f>
         <v/>
       </c>
       <c r="EL37" s="17">
-        <f>IFERROR(CV37-DQ37,"")</f>
+        <f>IF(OR(CV37="",DQ37=""),"",IFERROR(CV37-DQ37,""))</f>
         <v/>
       </c>
       <c r="EM37" s="17">
-        <f>IFERROR(CW37-DR37,"")</f>
+        <f>IF(OR(CW37="",DR37=""),"",IFERROR(CW37-DR37,""))</f>
         <v/>
       </c>
       <c r="EN37" s="17">
-        <f>IFERROR(CX37-DS37,"")</f>
+        <f>IF(OR(CX37="",DS37=""),"",IFERROR(CX37-DS37,""))</f>
         <v/>
       </c>
       <c r="EO37" s="17">
-        <f>IFERROR(CY37-DT37,"")</f>
+        <f>IF(OR(CY37="",DT37=""),"",IFERROR(CY37-DT37,""))</f>
         <v/>
       </c>
       <c r="EP37" s="17">
-        <f>IFERROR(CZ37-DU37,"")</f>
+        <f>IF(OR(CZ37="",DU37=""),"",IFERROR(CZ37-DU37,""))</f>
         <v/>
       </c>
       <c r="EQ37" s="17">
-        <f>IFERROR(DA37-DV37,"")</f>
+        <f>IF(OR(DA37="",DV37=""),"",IFERROR(DA37-DV37,""))</f>
         <v/>
       </c>
       <c r="ER37" s="17">
-        <f>IFERROR(DB37-DW37,"")</f>
+        <f>IF(OR(DB37="",DW37=""),"",IFERROR(DB37-DW37,""))</f>
         <v/>
       </c>
       <c r="ES37" s="17">
-        <f>IFERROR(DC37-DX37,"")</f>
+        <f>IF(OR(DC37="",DX37=""),"",IFERROR(DC37-DX37,""))</f>
         <v/>
       </c>
       <c r="EU37" s="16" t="n"/>
@@ -8789,83 +8789,83 @@
       <c r="DW38" s="18" t="n"/>
       <c r="DX38" s="18" t="n"/>
       <c r="DZ38" s="17">
-        <f>IFERROR(CJ38-DE38,"")</f>
+        <f>IF(OR(CJ38="",DE38=""),"",IFERROR(CJ38-DE38,""))</f>
         <v/>
       </c>
       <c r="EA38" s="17">
-        <f>IFERROR(CK38-DF38,"")</f>
+        <f>IF(OR(CK38="",DF38=""),"",IFERROR(CK38-DF38,""))</f>
         <v/>
       </c>
       <c r="EB38" s="17">
-        <f>IFERROR(CL38-DG38,"")</f>
+        <f>IF(OR(CL38="",DG38=""),"",IFERROR(CL38-DG38,""))</f>
         <v/>
       </c>
       <c r="EC38" s="17">
-        <f>IFERROR(CM38-DH38,"")</f>
+        <f>IF(OR(CM38="",DH38=""),"",IFERROR(CM38-DH38,""))</f>
         <v/>
       </c>
       <c r="ED38" s="17">
-        <f>IFERROR(CN38-DI38,"")</f>
+        <f>IF(OR(CN38="",DI38=""),"",IFERROR(CN38-DI38,""))</f>
         <v/>
       </c>
       <c r="EE38" s="17">
-        <f>IFERROR(CO38-DJ38,"")</f>
+        <f>IF(OR(CO38="",DJ38=""),"",IFERROR(CO38-DJ38,""))</f>
         <v/>
       </c>
       <c r="EF38" s="17">
-        <f>IFERROR(CP38-DK38,"")</f>
+        <f>IF(OR(CP38="",DK38=""),"",IFERROR(CP38-DK38,""))</f>
         <v/>
       </c>
       <c r="EG38" s="17">
-        <f>IFERROR(CQ38-DL38,"")</f>
+        <f>IF(OR(CQ38="",DL38=""),"",IFERROR(CQ38-DL38,""))</f>
         <v/>
       </c>
       <c r="EH38" s="17">
-        <f>IFERROR(CR38-DM38,"")</f>
+        <f>IF(OR(CR38="",DM38=""),"",IFERROR(CR38-DM38,""))</f>
         <v/>
       </c>
       <c r="EI38" s="17">
-        <f>IFERROR(CS38-DN38,"")</f>
+        <f>IF(OR(CS38="",DN38=""),"",IFERROR(CS38-DN38,""))</f>
         <v/>
       </c>
       <c r="EJ38" s="17">
-        <f>IFERROR(CT38-DO38,"")</f>
+        <f>IF(OR(CT38="",DO38=""),"",IFERROR(CT38-DO38,""))</f>
         <v/>
       </c>
       <c r="EK38" s="17">
-        <f>IFERROR(CU38-DP38,"")</f>
+        <f>IF(OR(CU38="",DP38=""),"",IFERROR(CU38-DP38,""))</f>
         <v/>
       </c>
       <c r="EL38" s="17">
-        <f>IFERROR(CV38-DQ38,"")</f>
+        <f>IF(OR(CV38="",DQ38=""),"",IFERROR(CV38-DQ38,""))</f>
         <v/>
       </c>
       <c r="EM38" s="17">
-        <f>IFERROR(CW38-DR38,"")</f>
+        <f>IF(OR(CW38="",DR38=""),"",IFERROR(CW38-DR38,""))</f>
         <v/>
       </c>
       <c r="EN38" s="17">
-        <f>IFERROR(CX38-DS38,"")</f>
+        <f>IF(OR(CX38="",DS38=""),"",IFERROR(CX38-DS38,""))</f>
         <v/>
       </c>
       <c r="EO38" s="17">
-        <f>IFERROR(CY38-DT38,"")</f>
+        <f>IF(OR(CY38="",DT38=""),"",IFERROR(CY38-DT38,""))</f>
         <v/>
       </c>
       <c r="EP38" s="17">
-        <f>IFERROR(CZ38-DU38,"")</f>
+        <f>IF(OR(CZ38="",DU38=""),"",IFERROR(CZ38-DU38,""))</f>
         <v/>
       </c>
       <c r="EQ38" s="17">
-        <f>IFERROR(DA38-DV38,"")</f>
+        <f>IF(OR(DA38="",DV38=""),"",IFERROR(DA38-DV38,""))</f>
         <v/>
       </c>
       <c r="ER38" s="17">
-        <f>IFERROR(DB38-DW38,"")</f>
+        <f>IF(OR(DB38="",DW38=""),"",IFERROR(DB38-DW38,""))</f>
         <v/>
       </c>
       <c r="ES38" s="17">
-        <f>IFERROR(DC38-DX38,"")</f>
+        <f>IF(OR(DC38="",DX38=""),"",IFERROR(DC38-DX38,""))</f>
         <v/>
       </c>
       <c r="EU38" s="16" t="n"/>
@@ -9019,83 +9019,83 @@
       <c r="DW39" s="18" t="n"/>
       <c r="DX39" s="18" t="n"/>
       <c r="DZ39" s="17">
-        <f>IFERROR(CJ39-DE39,"")</f>
+        <f>IF(OR(CJ39="",DE39=""),"",IFERROR(CJ39-DE39,""))</f>
         <v/>
       </c>
       <c r="EA39" s="17">
-        <f>IFERROR(CK39-DF39,"")</f>
+        <f>IF(OR(CK39="",DF39=""),"",IFERROR(CK39-DF39,""))</f>
         <v/>
       </c>
       <c r="EB39" s="17">
-        <f>IFERROR(CL39-DG39,"")</f>
+        <f>IF(OR(CL39="",DG39=""),"",IFERROR(CL39-DG39,""))</f>
         <v/>
       </c>
       <c r="EC39" s="17">
-        <f>IFERROR(CM39-DH39,"")</f>
+        <f>IF(OR(CM39="",DH39=""),"",IFERROR(CM39-DH39,""))</f>
         <v/>
       </c>
       <c r="ED39" s="17">
-        <f>IFERROR(CN39-DI39,"")</f>
+        <f>IF(OR(CN39="",DI39=""),"",IFERROR(CN39-DI39,""))</f>
         <v/>
       </c>
       <c r="EE39" s="17">
-        <f>IFERROR(CO39-DJ39,"")</f>
+        <f>IF(OR(CO39="",DJ39=""),"",IFERROR(CO39-DJ39,""))</f>
         <v/>
       </c>
       <c r="EF39" s="17">
-        <f>IFERROR(CP39-DK39,"")</f>
+        <f>IF(OR(CP39="",DK39=""),"",IFERROR(CP39-DK39,""))</f>
         <v/>
       </c>
       <c r="EG39" s="17">
-        <f>IFERROR(CQ39-DL39,"")</f>
+        <f>IF(OR(CQ39="",DL39=""),"",IFERROR(CQ39-DL39,""))</f>
         <v/>
       </c>
       <c r="EH39" s="17">
-        <f>IFERROR(CR39-DM39,"")</f>
+        <f>IF(OR(CR39="",DM39=""),"",IFERROR(CR39-DM39,""))</f>
         <v/>
       </c>
       <c r="EI39" s="17">
-        <f>IFERROR(CS39-DN39,"")</f>
+        <f>IF(OR(CS39="",DN39=""),"",IFERROR(CS39-DN39,""))</f>
         <v/>
       </c>
       <c r="EJ39" s="17">
-        <f>IFERROR(CT39-DO39,"")</f>
+        <f>IF(OR(CT39="",DO39=""),"",IFERROR(CT39-DO39,""))</f>
         <v/>
       </c>
       <c r="EK39" s="17">
-        <f>IFERROR(CU39-DP39,"")</f>
+        <f>IF(OR(CU39="",DP39=""),"",IFERROR(CU39-DP39,""))</f>
         <v/>
       </c>
       <c r="EL39" s="17">
-        <f>IFERROR(CV39-DQ39,"")</f>
+        <f>IF(OR(CV39="",DQ39=""),"",IFERROR(CV39-DQ39,""))</f>
         <v/>
       </c>
       <c r="EM39" s="17">
-        <f>IFERROR(CW39-DR39,"")</f>
+        <f>IF(OR(CW39="",DR39=""),"",IFERROR(CW39-DR39,""))</f>
         <v/>
       </c>
       <c r="EN39" s="17">
-        <f>IFERROR(CX39-DS39,"")</f>
+        <f>IF(OR(CX39="",DS39=""),"",IFERROR(CX39-DS39,""))</f>
         <v/>
       </c>
       <c r="EO39" s="17">
-        <f>IFERROR(CY39-DT39,"")</f>
+        <f>IF(OR(CY39="",DT39=""),"",IFERROR(CY39-DT39,""))</f>
         <v/>
       </c>
       <c r="EP39" s="17">
-        <f>IFERROR(CZ39-DU39,"")</f>
+        <f>IF(OR(CZ39="",DU39=""),"",IFERROR(CZ39-DU39,""))</f>
         <v/>
       </c>
       <c r="EQ39" s="17">
-        <f>IFERROR(DA39-DV39,"")</f>
+        <f>IF(OR(DA39="",DV39=""),"",IFERROR(DA39-DV39,""))</f>
         <v/>
       </c>
       <c r="ER39" s="17">
-        <f>IFERROR(DB39-DW39,"")</f>
+        <f>IF(OR(DB39="",DW39=""),"",IFERROR(DB39-DW39,""))</f>
         <v/>
       </c>
       <c r="ES39" s="17">
-        <f>IFERROR(DC39-DX39,"")</f>
+        <f>IF(OR(DC39="",DX39=""),"",IFERROR(DC39-DX39,""))</f>
         <v/>
       </c>
       <c r="EU39" s="16" t="n"/>
@@ -9249,83 +9249,83 @@
       <c r="DW40" s="18" t="n"/>
       <c r="DX40" s="18" t="n"/>
       <c r="DZ40" s="17">
-        <f>IFERROR(CJ40-DE40,"")</f>
+        <f>IF(OR(CJ40="",DE40=""),"",IFERROR(CJ40-DE40,""))</f>
         <v/>
       </c>
       <c r="EA40" s="17">
-        <f>IFERROR(CK40-DF40,"")</f>
+        <f>IF(OR(CK40="",DF40=""),"",IFERROR(CK40-DF40,""))</f>
         <v/>
       </c>
       <c r="EB40" s="17">
-        <f>IFERROR(CL40-DG40,"")</f>
+        <f>IF(OR(CL40="",DG40=""),"",IFERROR(CL40-DG40,""))</f>
         <v/>
       </c>
       <c r="EC40" s="17">
-        <f>IFERROR(CM40-DH40,"")</f>
+        <f>IF(OR(CM40="",DH40=""),"",IFERROR(CM40-DH40,""))</f>
         <v/>
       </c>
       <c r="ED40" s="17">
-        <f>IFERROR(CN40-DI40,"")</f>
+        <f>IF(OR(CN40="",DI40=""),"",IFERROR(CN40-DI40,""))</f>
         <v/>
       </c>
       <c r="EE40" s="17">
-        <f>IFERROR(CO40-DJ40,"")</f>
+        <f>IF(OR(CO40="",DJ40=""),"",IFERROR(CO40-DJ40,""))</f>
         <v/>
       </c>
       <c r="EF40" s="17">
-        <f>IFERROR(CP40-DK40,"")</f>
+        <f>IF(OR(CP40="",DK40=""),"",IFERROR(CP40-DK40,""))</f>
         <v/>
       </c>
       <c r="EG40" s="17">
-        <f>IFERROR(CQ40-DL40,"")</f>
+        <f>IF(OR(CQ40="",DL40=""),"",IFERROR(CQ40-DL40,""))</f>
         <v/>
       </c>
       <c r="EH40" s="17">
-        <f>IFERROR(CR40-DM40,"")</f>
+        <f>IF(OR(CR40="",DM40=""),"",IFERROR(CR40-DM40,""))</f>
         <v/>
       </c>
       <c r="EI40" s="17">
-        <f>IFERROR(CS40-DN40,"")</f>
+        <f>IF(OR(CS40="",DN40=""),"",IFERROR(CS40-DN40,""))</f>
         <v/>
       </c>
       <c r="EJ40" s="17">
-        <f>IFERROR(CT40-DO40,"")</f>
+        <f>IF(OR(CT40="",DO40=""),"",IFERROR(CT40-DO40,""))</f>
         <v/>
       </c>
       <c r="EK40" s="17">
-        <f>IFERROR(CU40-DP40,"")</f>
+        <f>IF(OR(CU40="",DP40=""),"",IFERROR(CU40-DP40,""))</f>
         <v/>
       </c>
       <c r="EL40" s="17">
-        <f>IFERROR(CV40-DQ40,"")</f>
+        <f>IF(OR(CV40="",DQ40=""),"",IFERROR(CV40-DQ40,""))</f>
         <v/>
       </c>
       <c r="EM40" s="17">
-        <f>IFERROR(CW40-DR40,"")</f>
+        <f>IF(OR(CW40="",DR40=""),"",IFERROR(CW40-DR40,""))</f>
         <v/>
       </c>
       <c r="EN40" s="17">
-        <f>IFERROR(CX40-DS40,"")</f>
+        <f>IF(OR(CX40="",DS40=""),"",IFERROR(CX40-DS40,""))</f>
         <v/>
       </c>
       <c r="EO40" s="17">
-        <f>IFERROR(CY40-DT40,"")</f>
+        <f>IF(OR(CY40="",DT40=""),"",IFERROR(CY40-DT40,""))</f>
         <v/>
       </c>
       <c r="EP40" s="17">
-        <f>IFERROR(CZ40-DU40,"")</f>
+        <f>IF(OR(CZ40="",DU40=""),"",IFERROR(CZ40-DU40,""))</f>
         <v/>
       </c>
       <c r="EQ40" s="17">
-        <f>IFERROR(DA40-DV40,"")</f>
+        <f>IF(OR(DA40="",DV40=""),"",IFERROR(DA40-DV40,""))</f>
         <v/>
       </c>
       <c r="ER40" s="17">
-        <f>IFERROR(DB40-DW40,"")</f>
+        <f>IF(OR(DB40="",DW40=""),"",IFERROR(DB40-DW40,""))</f>
         <v/>
       </c>
       <c r="ES40" s="17">
-        <f>IFERROR(DC40-DX40,"")</f>
+        <f>IF(OR(DC40="",DX40=""),"",IFERROR(DC40-DX40,""))</f>
         <v/>
       </c>
       <c r="EU40" s="16" t="n"/>
@@ -9479,83 +9479,83 @@
       <c r="DW41" s="18" t="n"/>
       <c r="DX41" s="18" t="n"/>
       <c r="DZ41" s="17">
-        <f>IFERROR(CJ41-DE41,"")</f>
+        <f>IF(OR(CJ41="",DE41=""),"",IFERROR(CJ41-DE41,""))</f>
         <v/>
       </c>
       <c r="EA41" s="17">
-        <f>IFERROR(CK41-DF41,"")</f>
+        <f>IF(OR(CK41="",DF41=""),"",IFERROR(CK41-DF41,""))</f>
         <v/>
       </c>
       <c r="EB41" s="17">
-        <f>IFERROR(CL41-DG41,"")</f>
+        <f>IF(OR(CL41="",DG41=""),"",IFERROR(CL41-DG41,""))</f>
         <v/>
       </c>
       <c r="EC41" s="17">
-        <f>IFERROR(CM41-DH41,"")</f>
+        <f>IF(OR(CM41="",DH41=""),"",IFERROR(CM41-DH41,""))</f>
         <v/>
       </c>
       <c r="ED41" s="17">
-        <f>IFERROR(CN41-DI41,"")</f>
+        <f>IF(OR(CN41="",DI41=""),"",IFERROR(CN41-DI41,""))</f>
         <v/>
       </c>
       <c r="EE41" s="17">
-        <f>IFERROR(CO41-DJ41,"")</f>
+        <f>IF(OR(CO41="",DJ41=""),"",IFERROR(CO41-DJ41,""))</f>
         <v/>
       </c>
       <c r="EF41" s="17">
-        <f>IFERROR(CP41-DK41,"")</f>
+        <f>IF(OR(CP41="",DK41=""),"",IFERROR(CP41-DK41,""))</f>
         <v/>
       </c>
       <c r="EG41" s="17">
-        <f>IFERROR(CQ41-DL41,"")</f>
+        <f>IF(OR(CQ41="",DL41=""),"",IFERROR(CQ41-DL41,""))</f>
         <v/>
       </c>
       <c r="EH41" s="17">
-        <f>IFERROR(CR41-DM41,"")</f>
+        <f>IF(OR(CR41="",DM41=""),"",IFERROR(CR41-DM41,""))</f>
         <v/>
       </c>
       <c r="EI41" s="17">
-        <f>IFERROR(CS41-DN41,"")</f>
+        <f>IF(OR(CS41="",DN41=""),"",IFERROR(CS41-DN41,""))</f>
         <v/>
       </c>
       <c r="EJ41" s="17">
-        <f>IFERROR(CT41-DO41,"")</f>
+        <f>IF(OR(CT41="",DO41=""),"",IFERROR(CT41-DO41,""))</f>
         <v/>
       </c>
       <c r="EK41" s="17">
-        <f>IFERROR(CU41-DP41,"")</f>
+        <f>IF(OR(CU41="",DP41=""),"",IFERROR(CU41-DP41,""))</f>
         <v/>
       </c>
       <c r="EL41" s="17">
-        <f>IFERROR(CV41-DQ41,"")</f>
+        <f>IF(OR(CV41="",DQ41=""),"",IFERROR(CV41-DQ41,""))</f>
         <v/>
       </c>
       <c r="EM41" s="17">
-        <f>IFERROR(CW41-DR41,"")</f>
+        <f>IF(OR(CW41="",DR41=""),"",IFERROR(CW41-DR41,""))</f>
         <v/>
       </c>
       <c r="EN41" s="17">
-        <f>IFERROR(CX41-DS41,"")</f>
+        <f>IF(OR(CX41="",DS41=""),"",IFERROR(CX41-DS41,""))</f>
         <v/>
       </c>
       <c r="EO41" s="17">
-        <f>IFERROR(CY41-DT41,"")</f>
+        <f>IF(OR(CY41="",DT41=""),"",IFERROR(CY41-DT41,""))</f>
         <v/>
       </c>
       <c r="EP41" s="17">
-        <f>IFERROR(CZ41-DU41,"")</f>
+        <f>IF(OR(CZ41="",DU41=""),"",IFERROR(CZ41-DU41,""))</f>
         <v/>
       </c>
       <c r="EQ41" s="17">
-        <f>IFERROR(DA41-DV41,"")</f>
+        <f>IF(OR(DA41="",DV41=""),"",IFERROR(DA41-DV41,""))</f>
         <v/>
       </c>
       <c r="ER41" s="17">
-        <f>IFERROR(DB41-DW41,"")</f>
+        <f>IF(OR(DB41="",DW41=""),"",IFERROR(DB41-DW41,""))</f>
         <v/>
       </c>
       <c r="ES41" s="17">
-        <f>IFERROR(DC41-DX41,"")</f>
+        <f>IF(OR(DC41="",DX41=""),"",IFERROR(DC41-DX41,""))</f>
         <v/>
       </c>
       <c r="EU41" s="16" t="n"/>

</xml_diff>

<commit_message>
D74b: the daily display sheet is as long as the counted window (28 days)
EcoGainsSim_Daily_v3.xlsx is rebuilt with 28 day rows (9..36), TOTAL on row 37, the legend
below it; --days N builds another length. The DoW column is a formula on cal_new's weekday row
at the column holding the first 1 on row 4 - the rule the engine reads the window by - so the
weekend tint follows the calendar instead of a hardcoded Wednesday start. Title and legend say
28-day window and how day 1 is found. harness/_display_formulas.json re-dumped (the fill
harness's builder-parity source); _mock_simfill 79/0.

Import order matters: a 28-row sheet under a 33-day calendar is overrun by the spill (TOTAL row
in the way), so renumber row 4 on both calendars first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/display/EcoGainsSim_Daily_v3.xlsx
+++ b/display/EcoGainsSim_Daily_v3.xlsx
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:FP52"/>
+  <dimension ref="B1:FP48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.75" customWidth="1" min="1" max="1"/>
@@ -778,7 +778,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>DAILY RESOURCE GAINS + NET — data vs sim, 33-day calendar, per earner (weekdays from the calendar sheets)</t>
+          <t>DAILY RESOURCE GAINS + NET — data vs sim, 28-day window, per earner (days and weekdays from the calendar sheets: day 1 = the first 1 on row 4)</t>
         </is>
       </c>
       <c r="FP1" s="2" t="inlineStr">
@@ -1877,10 +1877,9 @@
       <c r="B9" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
+      <c r="C9" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B9-1),3),"")</f>
+        <v/>
       </c>
       <c r="D9" s="16">
         <f>LET(payer,$C$3, segment,$C$4, source,$C$5, ECOGAINS_DAILY(payer, segment, source, "DATA", sim_refresh!$A$1))</f>
@@ -2133,10 +2132,9 @@
       <c r="B10" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
+      <c r="C10" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B10-1),3),"")</f>
+        <v/>
       </c>
       <c r="D10" s="16" t="n"/>
       <c r="E10" s="16" t="n"/>
@@ -2368,10 +2366,9 @@
       <c r="B11" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="15" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
+      <c r="C11" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B11-1),3),"")</f>
+        <v/>
       </c>
       <c r="D11" s="16" t="n"/>
       <c r="E11" s="16" t="n"/>
@@ -2603,10 +2600,9 @@
       <c r="B12" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
+      <c r="C12" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B12-1),3),"")</f>
+        <v/>
       </c>
       <c r="D12" s="16" t="n"/>
       <c r="E12" s="16" t="n"/>
@@ -2838,10 +2834,9 @@
       <c r="B13" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
+      <c r="C13" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B13-1),3),"")</f>
+        <v/>
       </c>
       <c r="D13" s="16" t="n"/>
       <c r="E13" s="16" t="n"/>
@@ -3073,10 +3068,9 @@
       <c r="B14" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
+      <c r="C14" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B14-1),3),"")</f>
+        <v/>
       </c>
       <c r="D14" s="16" t="n"/>
       <c r="E14" s="16" t="n"/>
@@ -3308,10 +3302,9 @@
       <c r="B15" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
+      <c r="C15" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B15-1),3),"")</f>
+        <v/>
       </c>
       <c r="D15" s="16" t="n"/>
       <c r="E15" s="16" t="n"/>
@@ -3543,10 +3536,9 @@
       <c r="B16" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
+      <c r="C16" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B16-1),3),"")</f>
+        <v/>
       </c>
       <c r="D16" s="16" t="n"/>
       <c r="E16" s="16" t="n"/>
@@ -3778,10 +3770,9 @@
       <c r="B17" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
+      <c r="C17" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B17-1),3),"")</f>
+        <v/>
       </c>
       <c r="D17" s="16" t="n"/>
       <c r="E17" s="16" t="n"/>
@@ -4013,10 +4004,9 @@
       <c r="B18" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
+      <c r="C18" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B18-1),3),"")</f>
+        <v/>
       </c>
       <c r="D18" s="16" t="n"/>
       <c r="E18" s="16" t="n"/>
@@ -4248,10 +4238,9 @@
       <c r="B19" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
+      <c r="C19" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B19-1),3),"")</f>
+        <v/>
       </c>
       <c r="D19" s="16" t="n"/>
       <c r="E19" s="16" t="n"/>
@@ -4483,10 +4472,9 @@
       <c r="B20" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
+      <c r="C20" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B20-1),3),"")</f>
+        <v/>
       </c>
       <c r="D20" s="16" t="n"/>
       <c r="E20" s="16" t="n"/>
@@ -4718,10 +4706,9 @@
       <c r="B21" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
+      <c r="C21" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B21-1),3),"")</f>
+        <v/>
       </c>
       <c r="D21" s="16" t="n"/>
       <c r="E21" s="16" t="n"/>
@@ -4953,10 +4940,9 @@
       <c r="B22" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
+      <c r="C22" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B22-1),3),"")</f>
+        <v/>
       </c>
       <c r="D22" s="16" t="n"/>
       <c r="E22" s="16" t="n"/>
@@ -5188,10 +5174,9 @@
       <c r="B23" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
+      <c r="C23" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B23-1),3),"")</f>
+        <v/>
       </c>
       <c r="D23" s="16" t="n"/>
       <c r="E23" s="16" t="n"/>
@@ -5423,10 +5408,9 @@
       <c r="B24" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
+      <c r="C24" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B24-1),3),"")</f>
+        <v/>
       </c>
       <c r="D24" s="16" t="n"/>
       <c r="E24" s="16" t="n"/>
@@ -5658,10 +5642,9 @@
       <c r="B25" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
+      <c r="C25" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B25-1),3),"")</f>
+        <v/>
       </c>
       <c r="D25" s="16" t="n"/>
       <c r="E25" s="16" t="n"/>
@@ -5893,10 +5876,9 @@
       <c r="B26" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
+      <c r="C26" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B26-1),3),"")</f>
+        <v/>
       </c>
       <c r="D26" s="16" t="n"/>
       <c r="E26" s="16" t="n"/>
@@ -6128,10 +6110,9 @@
       <c r="B27" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
+      <c r="C27" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B27-1),3),"")</f>
+        <v/>
       </c>
       <c r="D27" s="16" t="n"/>
       <c r="E27" s="16" t="n"/>
@@ -6363,10 +6344,9 @@
       <c r="B28" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
+      <c r="C28" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B28-1),3),"")</f>
+        <v/>
       </c>
       <c r="D28" s="16" t="n"/>
       <c r="E28" s="16" t="n"/>
@@ -6593,10 +6573,9 @@
       <c r="B29" s="15" t="n">
         <v>21</v>
       </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
+      <c r="C29" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B29-1),3),"")</f>
+        <v/>
       </c>
       <c r="D29" s="16" t="n"/>
       <c r="E29" s="16" t="n"/>
@@ -6823,10 +6802,9 @@
       <c r="B30" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
+      <c r="C30" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B30-1),3),"")</f>
+        <v/>
       </c>
       <c r="D30" s="16" t="n"/>
       <c r="E30" s="16" t="n"/>
@@ -7053,10 +7031,9 @@
       <c r="B31" s="15" t="n">
         <v>23</v>
       </c>
-      <c r="C31" s="15" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
+      <c r="C31" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B31-1),3),"")</f>
+        <v/>
       </c>
       <c r="D31" s="16" t="n"/>
       <c r="E31" s="16" t="n"/>
@@ -7283,10 +7260,9 @@
       <c r="B32" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="C32" s="15" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
+      <c r="C32" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B32-1),3),"")</f>
+        <v/>
       </c>
       <c r="D32" s="16" t="n"/>
       <c r="E32" s="16" t="n"/>
@@ -7513,10 +7489,9 @@
       <c r="B33" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="C33" s="15" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
+      <c r="C33" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B33-1),3),"")</f>
+        <v/>
       </c>
       <c r="D33" s="16" t="n"/>
       <c r="E33" s="16" t="n"/>
@@ -7743,10 +7718,9 @@
       <c r="B34" s="15" t="n">
         <v>26</v>
       </c>
-      <c r="C34" s="15" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
+      <c r="C34" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B34-1),3),"")</f>
+        <v/>
       </c>
       <c r="D34" s="16" t="n"/>
       <c r="E34" s="16" t="n"/>
@@ -7973,10 +7947,9 @@
       <c r="B35" s="15" t="n">
         <v>27</v>
       </c>
-      <c r="C35" s="15" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
+      <c r="C35" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B35-1),3),"")</f>
+        <v/>
       </c>
       <c r="D35" s="16" t="n"/>
       <c r="E35" s="16" t="n"/>
@@ -8203,10 +8176,9 @@
       <c r="B36" s="15" t="n">
         <v>28</v>
       </c>
-      <c r="C36" s="15" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
+      <c r="C36" s="15">
+        <f>IFERROR(LEFT(INDEX(cal_new!$A$3:$AH$3,1,MATCH(1,cal_new!$A$4:$AH$4,0)+B36-1),3),"")</f>
+        <v/>
       </c>
       <c r="D36" s="16" t="n"/>
       <c r="E36" s="16" t="n"/>
@@ -8430,1868 +8402,725 @@
       <c r="FN36" s="16" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="15" t="n">
-        <v>29</v>
-      </c>
-      <c r="C37" s="15" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="n"/>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="16" t="n"/>
-      <c r="G37" s="16" t="n"/>
-      <c r="H37" s="16" t="n"/>
-      <c r="I37" s="16" t="n"/>
-      <c r="J37" s="16" t="n"/>
-      <c r="K37" s="16" t="n"/>
-      <c r="L37" s="16" t="n"/>
-      <c r="M37" s="16" t="n"/>
-      <c r="N37" s="16" t="n"/>
-      <c r="O37" s="16" t="n"/>
-      <c r="P37" s="16" t="n"/>
-      <c r="Q37" s="16" t="n"/>
-      <c r="R37" s="16" t="n"/>
-      <c r="S37" s="16" t="n"/>
-      <c r="T37" s="16" t="n"/>
-      <c r="U37" s="16" t="n"/>
-      <c r="V37" s="16" t="n"/>
-      <c r="W37" s="16" t="n"/>
-      <c r="Y37" s="16" t="n"/>
-      <c r="Z37" s="16" t="n"/>
-      <c r="AA37" s="16" t="n"/>
-      <c r="AB37" s="16" t="n"/>
-      <c r="AC37" s="16" t="n"/>
-      <c r="AD37" s="16" t="n"/>
-      <c r="AE37" s="16" t="n"/>
-      <c r="AF37" s="16" t="n"/>
-      <c r="AG37" s="16" t="n"/>
-      <c r="AH37" s="16" t="n"/>
-      <c r="AI37" s="16" t="n"/>
-      <c r="AJ37" s="16" t="n"/>
-      <c r="AK37" s="16" t="n"/>
-      <c r="AL37" s="16" t="n"/>
-      <c r="AM37" s="16" t="n"/>
-      <c r="AN37" s="16" t="n"/>
-      <c r="AO37" s="16" t="n"/>
-      <c r="AP37" s="16" t="n"/>
-      <c r="AQ37" s="16" t="n"/>
-      <c r="AR37" s="16" t="n"/>
-      <c r="AT37" s="17" t="n"/>
-      <c r="AU37" s="17" t="n"/>
-      <c r="AV37" s="17" t="n"/>
-      <c r="AW37" s="17" t="n"/>
-      <c r="AX37" s="17" t="n"/>
-      <c r="AY37" s="17" t="n"/>
-      <c r="AZ37" s="17" t="n"/>
-      <c r="BA37" s="17" t="n"/>
-      <c r="BB37" s="17" t="n"/>
-      <c r="BC37" s="17" t="n"/>
-      <c r="BD37" s="17" t="n"/>
-      <c r="BE37" s="17" t="n"/>
-      <c r="BF37" s="17" t="n"/>
-      <c r="BG37" s="17" t="n"/>
-      <c r="BH37" s="17" t="n"/>
-      <c r="BI37" s="17" t="n"/>
-      <c r="BJ37" s="17" t="n"/>
-      <c r="BK37" s="17" t="n"/>
-      <c r="BL37" s="17" t="n"/>
-      <c r="BM37" s="17" t="n"/>
-      <c r="BO37" s="16" t="n"/>
-      <c r="BP37" s="16" t="n"/>
-      <c r="BQ37" s="16" t="n"/>
-      <c r="BR37" s="16" t="n"/>
-      <c r="BS37" s="16" t="n"/>
-      <c r="BT37" s="16" t="n"/>
-      <c r="BU37" s="16" t="n"/>
-      <c r="BV37" s="16" t="n"/>
-      <c r="BW37" s="16" t="n"/>
-      <c r="BX37" s="16" t="n"/>
-      <c r="BY37" s="16" t="n"/>
-      <c r="BZ37" s="16" t="n"/>
-      <c r="CA37" s="16" t="n"/>
-      <c r="CB37" s="16" t="n"/>
-      <c r="CC37" s="16" t="n"/>
-      <c r="CD37" s="16" t="n"/>
-      <c r="CE37" s="16" t="n"/>
-      <c r="CF37" s="16" t="n"/>
-      <c r="CG37" s="16" t="n"/>
-      <c r="CH37" s="16" t="n"/>
-      <c r="CJ37" s="18" t="n"/>
-      <c r="CK37" s="18" t="n"/>
-      <c r="CL37" s="18" t="n"/>
-      <c r="CM37" s="18" t="n"/>
-      <c r="CN37" s="18" t="n"/>
-      <c r="CO37" s="18" t="n"/>
-      <c r="CP37" s="18" t="n"/>
-      <c r="CQ37" s="18" t="n"/>
-      <c r="CR37" s="18" t="n"/>
-      <c r="CS37" s="18" t="n"/>
-      <c r="CT37" s="18" t="n"/>
-      <c r="CU37" s="18" t="n"/>
-      <c r="CV37" s="18" t="n"/>
-      <c r="CW37" s="18" t="n"/>
-      <c r="CX37" s="18" t="n"/>
-      <c r="CY37" s="18" t="n"/>
-      <c r="CZ37" s="18" t="n"/>
-      <c r="DA37" s="18" t="n"/>
-      <c r="DB37" s="18" t="n"/>
-      <c r="DC37" s="18" t="n"/>
-      <c r="DE37" s="18" t="n"/>
-      <c r="DF37" s="18" t="n"/>
-      <c r="DG37" s="18" t="n"/>
-      <c r="DH37" s="18" t="n"/>
-      <c r="DI37" s="18" t="n"/>
-      <c r="DJ37" s="18" t="n"/>
-      <c r="DK37" s="18" t="n"/>
-      <c r="DL37" s="18" t="n"/>
-      <c r="DM37" s="18" t="n"/>
-      <c r="DN37" s="18" t="n"/>
-      <c r="DO37" s="18" t="n"/>
-      <c r="DP37" s="18" t="n"/>
-      <c r="DQ37" s="18" t="n"/>
-      <c r="DR37" s="18" t="n"/>
-      <c r="DS37" s="18" t="n"/>
-      <c r="DT37" s="18" t="n"/>
-      <c r="DU37" s="18" t="n"/>
-      <c r="DV37" s="18" t="n"/>
-      <c r="DW37" s="18" t="n"/>
-      <c r="DX37" s="18" t="n"/>
-      <c r="DZ37" s="17">
-        <f>IF(OR(CJ37="",DE37=""),"",IFERROR(CJ37-DE37,""))</f>
-        <v/>
-      </c>
-      <c r="EA37" s="17">
-        <f>IF(OR(CK37="",DF37=""),"",IFERROR(CK37-DF37,""))</f>
-        <v/>
-      </c>
-      <c r="EB37" s="17">
-        <f>IF(OR(CL37="",DG37=""),"",IFERROR(CL37-DG37,""))</f>
-        <v/>
-      </c>
-      <c r="EC37" s="17">
-        <f>IF(OR(CM37="",DH37=""),"",IFERROR(CM37-DH37,""))</f>
-        <v/>
-      </c>
-      <c r="ED37" s="17">
-        <f>IF(OR(CN37="",DI37=""),"",IFERROR(CN37-DI37,""))</f>
-        <v/>
-      </c>
-      <c r="EE37" s="17">
-        <f>IF(OR(CO37="",DJ37=""),"",IFERROR(CO37-DJ37,""))</f>
-        <v/>
-      </c>
-      <c r="EF37" s="17">
-        <f>IF(OR(CP37="",DK37=""),"",IFERROR(CP37-DK37,""))</f>
-        <v/>
-      </c>
-      <c r="EG37" s="17">
-        <f>IF(OR(CQ37="",DL37=""),"",IFERROR(CQ37-DL37,""))</f>
-        <v/>
-      </c>
-      <c r="EH37" s="17">
-        <f>IF(OR(CR37="",DM37=""),"",IFERROR(CR37-DM37,""))</f>
-        <v/>
-      </c>
-      <c r="EI37" s="17">
-        <f>IF(OR(CS37="",DN37=""),"",IFERROR(CS37-DN37,""))</f>
-        <v/>
-      </c>
-      <c r="EJ37" s="17">
-        <f>IF(OR(CT37="",DO37=""),"",IFERROR(CT37-DO37,""))</f>
-        <v/>
-      </c>
-      <c r="EK37" s="17">
-        <f>IF(OR(CU37="",DP37=""),"",IFERROR(CU37-DP37,""))</f>
-        <v/>
-      </c>
-      <c r="EL37" s="17">
-        <f>IF(OR(CV37="",DQ37=""),"",IFERROR(CV37-DQ37,""))</f>
-        <v/>
-      </c>
-      <c r="EM37" s="17">
-        <f>IF(OR(CW37="",DR37=""),"",IFERROR(CW37-DR37,""))</f>
-        <v/>
-      </c>
-      <c r="EN37" s="17">
-        <f>IF(OR(CX37="",DS37=""),"",IFERROR(CX37-DS37,""))</f>
-        <v/>
-      </c>
-      <c r="EO37" s="17">
-        <f>IF(OR(CY37="",DT37=""),"",IFERROR(CY37-DT37,""))</f>
-        <v/>
-      </c>
-      <c r="EP37" s="17">
-        <f>IF(OR(CZ37="",DU37=""),"",IFERROR(CZ37-DU37,""))</f>
-        <v/>
-      </c>
-      <c r="EQ37" s="17">
-        <f>IF(OR(DA37="",DV37=""),"",IFERROR(DA37-DV37,""))</f>
-        <v/>
-      </c>
-      <c r="ER37" s="17">
-        <f>IF(OR(DB37="",DW37=""),"",IFERROR(DB37-DW37,""))</f>
-        <v/>
-      </c>
-      <c r="ES37" s="17">
-        <f>IF(OR(DC37="",DX37=""),"",IFERROR(DC37-DX37,""))</f>
-        <v/>
-      </c>
-      <c r="EU37" s="16" t="n"/>
-      <c r="EV37" s="16" t="n"/>
-      <c r="EW37" s="16" t="n"/>
-      <c r="EX37" s="16" t="n"/>
-      <c r="EY37" s="16" t="n"/>
-      <c r="EZ37" s="16" t="n"/>
-      <c r="FA37" s="16" t="n"/>
-      <c r="FB37" s="16" t="n"/>
-      <c r="FC37" s="16" t="n"/>
-      <c r="FD37" s="16" t="n"/>
-      <c r="FE37" s="16" t="n"/>
-      <c r="FF37" s="16" t="n"/>
-      <c r="FG37" s="16" t="n"/>
-      <c r="FH37" s="16" t="n"/>
-      <c r="FI37" s="16" t="n"/>
-      <c r="FJ37" s="16" t="n"/>
-      <c r="FK37" s="16" t="n"/>
-      <c r="FL37" s="16" t="n"/>
-      <c r="FM37" s="16" t="n"/>
-      <c r="FN37" s="16" t="n"/>
-    </row>
-    <row r="38">
-      <c r="B38" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="C38" s="15" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="D38" s="16" t="n"/>
-      <c r="E38" s="16" t="n"/>
-      <c r="F38" s="16" t="n"/>
-      <c r="G38" s="16" t="n"/>
-      <c r="H38" s="16" t="n"/>
-      <c r="I38" s="16" t="n"/>
-      <c r="J38" s="16" t="n"/>
-      <c r="K38" s="16" t="n"/>
-      <c r="L38" s="16" t="n"/>
-      <c r="M38" s="16" t="n"/>
-      <c r="N38" s="16" t="n"/>
-      <c r="O38" s="16" t="n"/>
-      <c r="P38" s="16" t="n"/>
-      <c r="Q38" s="16" t="n"/>
-      <c r="R38" s="16" t="n"/>
-      <c r="S38" s="16" t="n"/>
-      <c r="T38" s="16" t="n"/>
-      <c r="U38" s="16" t="n"/>
-      <c r="V38" s="16" t="n"/>
-      <c r="W38" s="16" t="n"/>
-      <c r="Y38" s="16" t="n"/>
-      <c r="Z38" s="16" t="n"/>
-      <c r="AA38" s="16" t="n"/>
-      <c r="AB38" s="16" t="n"/>
-      <c r="AC38" s="16" t="n"/>
-      <c r="AD38" s="16" t="n"/>
-      <c r="AE38" s="16" t="n"/>
-      <c r="AF38" s="16" t="n"/>
-      <c r="AG38" s="16" t="n"/>
-      <c r="AH38" s="16" t="n"/>
-      <c r="AI38" s="16" t="n"/>
-      <c r="AJ38" s="16" t="n"/>
-      <c r="AK38" s="16" t="n"/>
-      <c r="AL38" s="16" t="n"/>
-      <c r="AM38" s="16" t="n"/>
-      <c r="AN38" s="16" t="n"/>
-      <c r="AO38" s="16" t="n"/>
-      <c r="AP38" s="16" t="n"/>
-      <c r="AQ38" s="16" t="n"/>
-      <c r="AR38" s="16" t="n"/>
-      <c r="AT38" s="17" t="n"/>
-      <c r="AU38" s="17" t="n"/>
-      <c r="AV38" s="17" t="n"/>
-      <c r="AW38" s="17" t="n"/>
-      <c r="AX38" s="17" t="n"/>
-      <c r="AY38" s="17" t="n"/>
-      <c r="AZ38" s="17" t="n"/>
-      <c r="BA38" s="17" t="n"/>
-      <c r="BB38" s="17" t="n"/>
-      <c r="BC38" s="17" t="n"/>
-      <c r="BD38" s="17" t="n"/>
-      <c r="BE38" s="17" t="n"/>
-      <c r="BF38" s="17" t="n"/>
-      <c r="BG38" s="17" t="n"/>
-      <c r="BH38" s="17" t="n"/>
-      <c r="BI38" s="17" t="n"/>
-      <c r="BJ38" s="17" t="n"/>
-      <c r="BK38" s="17" t="n"/>
-      <c r="BL38" s="17" t="n"/>
-      <c r="BM38" s="17" t="n"/>
-      <c r="BO38" s="16" t="n"/>
-      <c r="BP38" s="16" t="n"/>
-      <c r="BQ38" s="16" t="n"/>
-      <c r="BR38" s="16" t="n"/>
-      <c r="BS38" s="16" t="n"/>
-      <c r="BT38" s="16" t="n"/>
-      <c r="BU38" s="16" t="n"/>
-      <c r="BV38" s="16" t="n"/>
-      <c r="BW38" s="16" t="n"/>
-      <c r="BX38" s="16" t="n"/>
-      <c r="BY38" s="16" t="n"/>
-      <c r="BZ38" s="16" t="n"/>
-      <c r="CA38" s="16" t="n"/>
-      <c r="CB38" s="16" t="n"/>
-      <c r="CC38" s="16" t="n"/>
-      <c r="CD38" s="16" t="n"/>
-      <c r="CE38" s="16" t="n"/>
-      <c r="CF38" s="16" t="n"/>
-      <c r="CG38" s="16" t="n"/>
-      <c r="CH38" s="16" t="n"/>
-      <c r="CJ38" s="18" t="n"/>
-      <c r="CK38" s="18" t="n"/>
-      <c r="CL38" s="18" t="n"/>
-      <c r="CM38" s="18" t="n"/>
-      <c r="CN38" s="18" t="n"/>
-      <c r="CO38" s="18" t="n"/>
-      <c r="CP38" s="18" t="n"/>
-      <c r="CQ38" s="18" t="n"/>
-      <c r="CR38" s="18" t="n"/>
-      <c r="CS38" s="18" t="n"/>
-      <c r="CT38" s="18" t="n"/>
-      <c r="CU38" s="18" t="n"/>
-      <c r="CV38" s="18" t="n"/>
-      <c r="CW38" s="18" t="n"/>
-      <c r="CX38" s="18" t="n"/>
-      <c r="CY38" s="18" t="n"/>
-      <c r="CZ38" s="18" t="n"/>
-      <c r="DA38" s="18" t="n"/>
-      <c r="DB38" s="18" t="n"/>
-      <c r="DC38" s="18" t="n"/>
-      <c r="DE38" s="18" t="n"/>
-      <c r="DF38" s="18" t="n"/>
-      <c r="DG38" s="18" t="n"/>
-      <c r="DH38" s="18" t="n"/>
-      <c r="DI38" s="18" t="n"/>
-      <c r="DJ38" s="18" t="n"/>
-      <c r="DK38" s="18" t="n"/>
-      <c r="DL38" s="18" t="n"/>
-      <c r="DM38" s="18" t="n"/>
-      <c r="DN38" s="18" t="n"/>
-      <c r="DO38" s="18" t="n"/>
-      <c r="DP38" s="18" t="n"/>
-      <c r="DQ38" s="18" t="n"/>
-      <c r="DR38" s="18" t="n"/>
-      <c r="DS38" s="18" t="n"/>
-      <c r="DT38" s="18" t="n"/>
-      <c r="DU38" s="18" t="n"/>
-      <c r="DV38" s="18" t="n"/>
-      <c r="DW38" s="18" t="n"/>
-      <c r="DX38" s="18" t="n"/>
-      <c r="DZ38" s="17">
-        <f>IF(OR(CJ38="",DE38=""),"",IFERROR(CJ38-DE38,""))</f>
-        <v/>
-      </c>
-      <c r="EA38" s="17">
-        <f>IF(OR(CK38="",DF38=""),"",IFERROR(CK38-DF38,""))</f>
-        <v/>
-      </c>
-      <c r="EB38" s="17">
-        <f>IF(OR(CL38="",DG38=""),"",IFERROR(CL38-DG38,""))</f>
-        <v/>
-      </c>
-      <c r="EC38" s="17">
-        <f>IF(OR(CM38="",DH38=""),"",IFERROR(CM38-DH38,""))</f>
-        <v/>
-      </c>
-      <c r="ED38" s="17">
-        <f>IF(OR(CN38="",DI38=""),"",IFERROR(CN38-DI38,""))</f>
-        <v/>
-      </c>
-      <c r="EE38" s="17">
-        <f>IF(OR(CO38="",DJ38=""),"",IFERROR(CO38-DJ38,""))</f>
-        <v/>
-      </c>
-      <c r="EF38" s="17">
-        <f>IF(OR(CP38="",DK38=""),"",IFERROR(CP38-DK38,""))</f>
-        <v/>
-      </c>
-      <c r="EG38" s="17">
-        <f>IF(OR(CQ38="",DL38=""),"",IFERROR(CQ38-DL38,""))</f>
-        <v/>
-      </c>
-      <c r="EH38" s="17">
-        <f>IF(OR(CR38="",DM38=""),"",IFERROR(CR38-DM38,""))</f>
-        <v/>
-      </c>
-      <c r="EI38" s="17">
-        <f>IF(OR(CS38="",DN38=""),"",IFERROR(CS38-DN38,""))</f>
-        <v/>
-      </c>
-      <c r="EJ38" s="17">
-        <f>IF(OR(CT38="",DO38=""),"",IFERROR(CT38-DO38,""))</f>
-        <v/>
-      </c>
-      <c r="EK38" s="17">
-        <f>IF(OR(CU38="",DP38=""),"",IFERROR(CU38-DP38,""))</f>
-        <v/>
-      </c>
-      <c r="EL38" s="17">
-        <f>IF(OR(CV38="",DQ38=""),"",IFERROR(CV38-DQ38,""))</f>
-        <v/>
-      </c>
-      <c r="EM38" s="17">
-        <f>IF(OR(CW38="",DR38=""),"",IFERROR(CW38-DR38,""))</f>
-        <v/>
-      </c>
-      <c r="EN38" s="17">
-        <f>IF(OR(CX38="",DS38=""),"",IFERROR(CX38-DS38,""))</f>
-        <v/>
-      </c>
-      <c r="EO38" s="17">
-        <f>IF(OR(CY38="",DT38=""),"",IFERROR(CY38-DT38,""))</f>
-        <v/>
-      </c>
-      <c r="EP38" s="17">
-        <f>IF(OR(CZ38="",DU38=""),"",IFERROR(CZ38-DU38,""))</f>
-        <v/>
-      </c>
-      <c r="EQ38" s="17">
-        <f>IF(OR(DA38="",DV38=""),"",IFERROR(DA38-DV38,""))</f>
-        <v/>
-      </c>
-      <c r="ER38" s="17">
-        <f>IF(OR(DB38="",DW38=""),"",IFERROR(DB38-DW38,""))</f>
-        <v/>
-      </c>
-      <c r="ES38" s="17">
-        <f>IF(OR(DC38="",DX38=""),"",IFERROR(DC38-DX38,""))</f>
-        <v/>
-      </c>
-      <c r="EU38" s="16" t="n"/>
-      <c r="EV38" s="16" t="n"/>
-      <c r="EW38" s="16" t="n"/>
-      <c r="EX38" s="16" t="n"/>
-      <c r="EY38" s="16" t="n"/>
-      <c r="EZ38" s="16" t="n"/>
-      <c r="FA38" s="16" t="n"/>
-      <c r="FB38" s="16" t="n"/>
-      <c r="FC38" s="16" t="n"/>
-      <c r="FD38" s="16" t="n"/>
-      <c r="FE38" s="16" t="n"/>
-      <c r="FF38" s="16" t="n"/>
-      <c r="FG38" s="16" t="n"/>
-      <c r="FH38" s="16" t="n"/>
-      <c r="FI38" s="16" t="n"/>
-      <c r="FJ38" s="16" t="n"/>
-      <c r="FK38" s="16" t="n"/>
-      <c r="FL38" s="16" t="n"/>
-      <c r="FM38" s="16" t="n"/>
-      <c r="FN38" s="16" t="n"/>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C37" s="20" t="n"/>
+      <c r="D37" s="21">
+        <f>IF(COUNT(D9:D36)=0,"",SUM(D9:D36))</f>
+        <v/>
+      </c>
+      <c r="E37" s="21">
+        <f>IF(COUNT(E9:E36)=0,"",SUM(E9:E36))</f>
+        <v/>
+      </c>
+      <c r="F37" s="21">
+        <f>IF(COUNT(F9:F36)=0,"",SUM(F9:F36))</f>
+        <v/>
+      </c>
+      <c r="G37" s="21">
+        <f>IF(COUNT(G9:G36)=0,"",SUM(G9:G36))</f>
+        <v/>
+      </c>
+      <c r="H37" s="21">
+        <f>IF(COUNT(H9:H36)=0,"",SUM(H9:H36))</f>
+        <v/>
+      </c>
+      <c r="I37" s="21">
+        <f>IF(COUNT(I9:I36)=0,"",SUM(I9:I36))</f>
+        <v/>
+      </c>
+      <c r="J37" s="21">
+        <f>IF(COUNT(J9:J36)=0,"",SUM(J9:J36))</f>
+        <v/>
+      </c>
+      <c r="K37" s="21">
+        <f>IF(COUNT(K9:K36)=0,"",SUM(K9:K36))</f>
+        <v/>
+      </c>
+      <c r="L37" s="21">
+        <f>IF(COUNT(L9:L36)=0,"",SUM(L9:L36))</f>
+        <v/>
+      </c>
+      <c r="M37" s="21">
+        <f>IF(COUNT(M9:M36)=0,"",SUM(M9:M36))</f>
+        <v/>
+      </c>
+      <c r="N37" s="21">
+        <f>IF(COUNT(N9:N36)=0,"",SUM(N9:N36))</f>
+        <v/>
+      </c>
+      <c r="O37" s="21">
+        <f>IF(COUNT(O9:O36)=0,"",SUM(O9:O36))</f>
+        <v/>
+      </c>
+      <c r="P37" s="21">
+        <f>IF(COUNT(P9:P36)=0,"",SUM(P9:P36))</f>
+        <v/>
+      </c>
+      <c r="Q37" s="21">
+        <f>IF(COUNT(Q9:Q36)=0,"",SUM(Q9:Q36))</f>
+        <v/>
+      </c>
+      <c r="R37" s="21">
+        <f>IF(COUNT(R9:R36)=0,"",SUM(R9:R36))</f>
+        <v/>
+      </c>
+      <c r="S37" s="21">
+        <f>IF(COUNT(S9:S36)=0,"",SUM(S9:S36))</f>
+        <v/>
+      </c>
+      <c r="T37" s="21">
+        <f>IF(COUNT(T9:T36)=0,"",SUM(T9:T36))</f>
+        <v/>
+      </c>
+      <c r="U37" s="21">
+        <f>IF(COUNT(U9:U36)=0,"",SUM(U9:U36))</f>
+        <v/>
+      </c>
+      <c r="V37" s="21">
+        <f>IF(COUNT(V9:V36)=0,"",SUM(V9:V36))</f>
+        <v/>
+      </c>
+      <c r="W37" s="21">
+        <f>IF(COUNT(W9:W36)=0,"",SUM(W9:W36))</f>
+        <v/>
+      </c>
+      <c r="Y37" s="22">
+        <f>SUM(Y9:Y36)</f>
+        <v/>
+      </c>
+      <c r="Z37" s="22">
+        <f>SUM(Z9:Z36)</f>
+        <v/>
+      </c>
+      <c r="AA37" s="22">
+        <f>SUM(AA9:AA36)</f>
+        <v/>
+      </c>
+      <c r="AB37" s="22">
+        <f>SUM(AB9:AB36)</f>
+        <v/>
+      </c>
+      <c r="AC37" s="22">
+        <f>SUM(AC9:AC36)</f>
+        <v/>
+      </c>
+      <c r="AD37" s="22">
+        <f>SUM(AD9:AD36)</f>
+        <v/>
+      </c>
+      <c r="AE37" s="22">
+        <f>SUM(AE9:AE36)</f>
+        <v/>
+      </c>
+      <c r="AF37" s="22">
+        <f>SUM(AF9:AF36)</f>
+        <v/>
+      </c>
+      <c r="AG37" s="22">
+        <f>SUM(AG9:AG36)</f>
+        <v/>
+      </c>
+      <c r="AH37" s="22">
+        <f>SUM(AH9:AH36)</f>
+        <v/>
+      </c>
+      <c r="AI37" s="22">
+        <f>SUM(AI9:AI36)</f>
+        <v/>
+      </c>
+      <c r="AJ37" s="22">
+        <f>SUM(AJ9:AJ36)</f>
+        <v/>
+      </c>
+      <c r="AK37" s="22">
+        <f>SUM(AK9:AK36)</f>
+        <v/>
+      </c>
+      <c r="AL37" s="22">
+        <f>SUM(AL9:AL36)</f>
+        <v/>
+      </c>
+      <c r="AM37" s="22">
+        <f>SUM(AM9:AM36)</f>
+        <v/>
+      </c>
+      <c r="AN37" s="22">
+        <f>SUM(AN9:AN36)</f>
+        <v/>
+      </c>
+      <c r="AO37" s="22">
+        <f>SUM(AO9:AO36)</f>
+        <v/>
+      </c>
+      <c r="AP37" s="22">
+        <f>SUM(AP9:AP36)</f>
+        <v/>
+      </c>
+      <c r="AQ37" s="22">
+        <f>SUM(AQ9:AQ36)</f>
+        <v/>
+      </c>
+      <c r="AR37" s="22">
+        <f>SUM(AR9:AR36)</f>
+        <v/>
+      </c>
+      <c r="AT37" s="23">
+        <f>IF(COUNT(AT9:AT36)=0,"",SUM(AT9:AT36))</f>
+        <v/>
+      </c>
+      <c r="AU37" s="23">
+        <f>IF(COUNT(AU9:AU36)=0,"",SUM(AU9:AU36))</f>
+        <v/>
+      </c>
+      <c r="AV37" s="23">
+        <f>IF(COUNT(AV9:AV36)=0,"",SUM(AV9:AV36))</f>
+        <v/>
+      </c>
+      <c r="AW37" s="23">
+        <f>IF(COUNT(AW9:AW36)=0,"",SUM(AW9:AW36))</f>
+        <v/>
+      </c>
+      <c r="AX37" s="23">
+        <f>IF(COUNT(AX9:AX36)=0,"",SUM(AX9:AX36))</f>
+        <v/>
+      </c>
+      <c r="AY37" s="23">
+        <f>IF(COUNT(AY9:AY36)=0,"",SUM(AY9:AY36))</f>
+        <v/>
+      </c>
+      <c r="AZ37" s="23">
+        <f>IF(COUNT(AZ9:AZ36)=0,"",SUM(AZ9:AZ36))</f>
+        <v/>
+      </c>
+      <c r="BA37" s="23">
+        <f>IF(COUNT(BA9:BA36)=0,"",SUM(BA9:BA36))</f>
+        <v/>
+      </c>
+      <c r="BB37" s="23">
+        <f>IF(COUNT(BB9:BB36)=0,"",SUM(BB9:BB36))</f>
+        <v/>
+      </c>
+      <c r="BC37" s="23">
+        <f>IF(COUNT(BC9:BC36)=0,"",SUM(BC9:BC36))</f>
+        <v/>
+      </c>
+      <c r="BD37" s="23">
+        <f>IF(COUNT(BD9:BD36)=0,"",SUM(BD9:BD36))</f>
+        <v/>
+      </c>
+      <c r="BE37" s="23">
+        <f>IF(COUNT(BE9:BE36)=0,"",SUM(BE9:BE36))</f>
+        <v/>
+      </c>
+      <c r="BF37" s="23">
+        <f>IF(COUNT(BF9:BF36)=0,"",SUM(BF9:BF36))</f>
+        <v/>
+      </c>
+      <c r="BG37" s="23">
+        <f>IF(COUNT(BG9:BG36)=0,"",SUM(BG9:BG36))</f>
+        <v/>
+      </c>
+      <c r="BH37" s="23">
+        <f>IF(COUNT(BH9:BH36)=0,"",SUM(BH9:BH36))</f>
+        <v/>
+      </c>
+      <c r="BI37" s="23">
+        <f>IF(COUNT(BI9:BI36)=0,"",SUM(BI9:BI36))</f>
+        <v/>
+      </c>
+      <c r="BJ37" s="23">
+        <f>IF(COUNT(BJ9:BJ36)=0,"",SUM(BJ9:BJ36))</f>
+        <v/>
+      </c>
+      <c r="BK37" s="23">
+        <f>IF(COUNT(BK9:BK36)=0,"",SUM(BK9:BK36))</f>
+        <v/>
+      </c>
+      <c r="BL37" s="23">
+        <f>IF(COUNT(BL9:BL36)=0,"",SUM(BL9:BL36))</f>
+        <v/>
+      </c>
+      <c r="BM37" s="23">
+        <f>IF(COUNT(BM9:BM36)=0,"",SUM(BM9:BM36))</f>
+        <v/>
+      </c>
+      <c r="BO37" s="24">
+        <f>IF(COUNT(BO9:BO36)=0,"",SUM(BO9:BO36))</f>
+        <v/>
+      </c>
+      <c r="BP37" s="24">
+        <f>IF(COUNT(BP9:BP36)=0,"",SUM(BP9:BP36))</f>
+        <v/>
+      </c>
+      <c r="BQ37" s="24">
+        <f>IF(COUNT(BQ9:BQ36)=0,"",SUM(BQ9:BQ36))</f>
+        <v/>
+      </c>
+      <c r="BR37" s="24">
+        <f>IF(COUNT(BR9:BR36)=0,"",SUM(BR9:BR36))</f>
+        <v/>
+      </c>
+      <c r="BS37" s="24">
+        <f>IF(COUNT(BS9:BS36)=0,"",SUM(BS9:BS36))</f>
+        <v/>
+      </c>
+      <c r="BT37" s="24">
+        <f>IF(COUNT(BT9:BT36)=0,"",SUM(BT9:BT36))</f>
+        <v/>
+      </c>
+      <c r="BU37" s="24">
+        <f>IF(COUNT(BU9:BU36)=0,"",SUM(BU9:BU36))</f>
+        <v/>
+      </c>
+      <c r="BV37" s="24">
+        <f>IF(COUNT(BV9:BV36)=0,"",SUM(BV9:BV36))</f>
+        <v/>
+      </c>
+      <c r="BW37" s="24">
+        <f>IF(COUNT(BW9:BW36)=0,"",SUM(BW9:BW36))</f>
+        <v/>
+      </c>
+      <c r="BX37" s="24">
+        <f>IF(COUNT(BX9:BX36)=0,"",SUM(BX9:BX36))</f>
+        <v/>
+      </c>
+      <c r="BY37" s="24">
+        <f>IF(COUNT(BY9:BY36)=0,"",SUM(BY9:BY36))</f>
+        <v/>
+      </c>
+      <c r="BZ37" s="24">
+        <f>IF(COUNT(BZ9:BZ36)=0,"",SUM(BZ9:BZ36))</f>
+        <v/>
+      </c>
+      <c r="CA37" s="24">
+        <f>IF(COUNT(CA9:CA36)=0,"",SUM(CA9:CA36))</f>
+        <v/>
+      </c>
+      <c r="CB37" s="24">
+        <f>IF(COUNT(CB9:CB36)=0,"",SUM(CB9:CB36))</f>
+        <v/>
+      </c>
+      <c r="CC37" s="24">
+        <f>IF(COUNT(CC9:CC36)=0,"",SUM(CC9:CC36))</f>
+        <v/>
+      </c>
+      <c r="CD37" s="24">
+        <f>IF(COUNT(CD9:CD36)=0,"",SUM(CD9:CD36))</f>
+        <v/>
+      </c>
+      <c r="CE37" s="24">
+        <f>IF(COUNT(CE9:CE36)=0,"",SUM(CE9:CE36))</f>
+        <v/>
+      </c>
+      <c r="CF37" s="24">
+        <f>IF(COUNT(CF9:CF36)=0,"",SUM(CF9:CF36))</f>
+        <v/>
+      </c>
+      <c r="CG37" s="24">
+        <f>IF(COUNT(CG9:CG36)=0,"",SUM(CG9:CG36))</f>
+        <v/>
+      </c>
+      <c r="CH37" s="24">
+        <f>IF(COUNT(CH9:CH36)=0,"",SUM(CH9:CH36))</f>
+        <v/>
+      </c>
+      <c r="CJ37" s="25">
+        <f>IF(COUNT(CJ9:CJ36)=0,"",SUM(CJ9:CJ36))</f>
+        <v/>
+      </c>
+      <c r="CK37" s="25">
+        <f>IF(COUNT(CK9:CK36)=0,"",SUM(CK9:CK36))</f>
+        <v/>
+      </c>
+      <c r="CL37" s="25">
+        <f>IF(COUNT(CL9:CL36)=0,"",SUM(CL9:CL36))</f>
+        <v/>
+      </c>
+      <c r="CM37" s="25">
+        <f>IF(COUNT(CM9:CM36)=0,"",SUM(CM9:CM36))</f>
+        <v/>
+      </c>
+      <c r="CN37" s="25">
+        <f>IF(COUNT(CN9:CN36)=0,"",SUM(CN9:CN36))</f>
+        <v/>
+      </c>
+      <c r="CO37" s="25">
+        <f>IF(COUNT(CO9:CO36)=0,"",SUM(CO9:CO36))</f>
+        <v/>
+      </c>
+      <c r="CP37" s="25">
+        <f>IF(COUNT(CP9:CP36)=0,"",SUM(CP9:CP36))</f>
+        <v/>
+      </c>
+      <c r="CQ37" s="25">
+        <f>IF(COUNT(CQ9:CQ36)=0,"",SUM(CQ9:CQ36))</f>
+        <v/>
+      </c>
+      <c r="CR37" s="25">
+        <f>IF(COUNT(CR9:CR36)=0,"",SUM(CR9:CR36))</f>
+        <v/>
+      </c>
+      <c r="CS37" s="25">
+        <f>IF(COUNT(CS9:CS36)=0,"",SUM(CS9:CS36))</f>
+        <v/>
+      </c>
+      <c r="CT37" s="25">
+        <f>IF(COUNT(CT9:CT36)=0,"",SUM(CT9:CT36))</f>
+        <v/>
+      </c>
+      <c r="CU37" s="25">
+        <f>IF(COUNT(CU9:CU36)=0,"",SUM(CU9:CU36))</f>
+        <v/>
+      </c>
+      <c r="CV37" s="25">
+        <f>IF(COUNT(CV9:CV36)=0,"",SUM(CV9:CV36))</f>
+        <v/>
+      </c>
+      <c r="CW37" s="25">
+        <f>IF(COUNT(CW9:CW36)=0,"",SUM(CW9:CW36))</f>
+        <v/>
+      </c>
+      <c r="CX37" s="25">
+        <f>IF(COUNT(CX9:CX36)=0,"",SUM(CX9:CX36))</f>
+        <v/>
+      </c>
+      <c r="CY37" s="25">
+        <f>IF(COUNT(CY9:CY36)=0,"",SUM(CY9:CY36))</f>
+        <v/>
+      </c>
+      <c r="CZ37" s="25">
+        <f>IF(COUNT(CZ9:CZ36)=0,"",SUM(CZ9:CZ36))</f>
+        <v/>
+      </c>
+      <c r="DA37" s="25">
+        <f>IF(COUNT(DA9:DA36)=0,"",SUM(DA9:DA36))</f>
+        <v/>
+      </c>
+      <c r="DB37" s="25">
+        <f>IF(COUNT(DB9:DB36)=0,"",SUM(DB9:DB36))</f>
+        <v/>
+      </c>
+      <c r="DC37" s="25">
+        <f>IF(COUNT(DC9:DC36)=0,"",SUM(DC9:DC36))</f>
+        <v/>
+      </c>
+      <c r="DE37" s="25">
+        <f>IF(COUNT(DE9:DE36)=0,"",SUM(DE9:DE36))</f>
+        <v/>
+      </c>
+      <c r="DF37" s="25">
+        <f>IF(COUNT(DF9:DF36)=0,"",SUM(DF9:DF36))</f>
+        <v/>
+      </c>
+      <c r="DG37" s="25">
+        <f>IF(COUNT(DG9:DG36)=0,"",SUM(DG9:DG36))</f>
+        <v/>
+      </c>
+      <c r="DH37" s="25">
+        <f>IF(COUNT(DH9:DH36)=0,"",SUM(DH9:DH36))</f>
+        <v/>
+      </c>
+      <c r="DI37" s="25">
+        <f>IF(COUNT(DI9:DI36)=0,"",SUM(DI9:DI36))</f>
+        <v/>
+      </c>
+      <c r="DJ37" s="25">
+        <f>IF(COUNT(DJ9:DJ36)=0,"",SUM(DJ9:DJ36))</f>
+        <v/>
+      </c>
+      <c r="DK37" s="25">
+        <f>IF(COUNT(DK9:DK36)=0,"",SUM(DK9:DK36))</f>
+        <v/>
+      </c>
+      <c r="DL37" s="25">
+        <f>IF(COUNT(DL9:DL36)=0,"",SUM(DL9:DL36))</f>
+        <v/>
+      </c>
+      <c r="DM37" s="25">
+        <f>IF(COUNT(DM9:DM36)=0,"",SUM(DM9:DM36))</f>
+        <v/>
+      </c>
+      <c r="DN37" s="25">
+        <f>IF(COUNT(DN9:DN36)=0,"",SUM(DN9:DN36))</f>
+        <v/>
+      </c>
+      <c r="DO37" s="25">
+        <f>IF(COUNT(DO9:DO36)=0,"",SUM(DO9:DO36))</f>
+        <v/>
+      </c>
+      <c r="DP37" s="25">
+        <f>IF(COUNT(DP9:DP36)=0,"",SUM(DP9:DP36))</f>
+        <v/>
+      </c>
+      <c r="DQ37" s="25">
+        <f>IF(COUNT(DQ9:DQ36)=0,"",SUM(DQ9:DQ36))</f>
+        <v/>
+      </c>
+      <c r="DR37" s="25">
+        <f>IF(COUNT(DR9:DR36)=0,"",SUM(DR9:DR36))</f>
+        <v/>
+      </c>
+      <c r="DS37" s="25">
+        <f>IF(COUNT(DS9:DS36)=0,"",SUM(DS9:DS36))</f>
+        <v/>
+      </c>
+      <c r="DT37" s="25">
+        <f>IF(COUNT(DT9:DT36)=0,"",SUM(DT9:DT36))</f>
+        <v/>
+      </c>
+      <c r="DU37" s="25">
+        <f>IF(COUNT(DU9:DU36)=0,"",SUM(DU9:DU36))</f>
+        <v/>
+      </c>
+      <c r="DV37" s="25">
+        <f>IF(COUNT(DV9:DV36)=0,"",SUM(DV9:DV36))</f>
+        <v/>
+      </c>
+      <c r="DW37" s="25">
+        <f>IF(COUNT(DW9:DW36)=0,"",SUM(DW9:DW36))</f>
+        <v/>
+      </c>
+      <c r="DX37" s="25">
+        <f>IF(COUNT(DX9:DX36)=0,"",SUM(DX9:DX36))</f>
+        <v/>
+      </c>
+      <c r="DZ37" s="23">
+        <f>IF(COUNT(DZ9:DZ36)=0,"",SUM(DZ9:DZ36))</f>
+        <v/>
+      </c>
+      <c r="EA37" s="23">
+        <f>IF(COUNT(EA9:EA36)=0,"",SUM(EA9:EA36))</f>
+        <v/>
+      </c>
+      <c r="EB37" s="23">
+        <f>IF(COUNT(EB9:EB36)=0,"",SUM(EB9:EB36))</f>
+        <v/>
+      </c>
+      <c r="EC37" s="23">
+        <f>IF(COUNT(EC9:EC36)=0,"",SUM(EC9:EC36))</f>
+        <v/>
+      </c>
+      <c r="ED37" s="23">
+        <f>IF(COUNT(ED9:ED36)=0,"",SUM(ED9:ED36))</f>
+        <v/>
+      </c>
+      <c r="EE37" s="23">
+        <f>IF(COUNT(EE9:EE36)=0,"",SUM(EE9:EE36))</f>
+        <v/>
+      </c>
+      <c r="EF37" s="23">
+        <f>IF(COUNT(EF9:EF36)=0,"",SUM(EF9:EF36))</f>
+        <v/>
+      </c>
+      <c r="EG37" s="23">
+        <f>IF(COUNT(EG9:EG36)=0,"",SUM(EG9:EG36))</f>
+        <v/>
+      </c>
+      <c r="EH37" s="23">
+        <f>IF(COUNT(EH9:EH36)=0,"",SUM(EH9:EH36))</f>
+        <v/>
+      </c>
+      <c r="EI37" s="23">
+        <f>IF(COUNT(EI9:EI36)=0,"",SUM(EI9:EI36))</f>
+        <v/>
+      </c>
+      <c r="EJ37" s="23">
+        <f>IF(COUNT(EJ9:EJ36)=0,"",SUM(EJ9:EJ36))</f>
+        <v/>
+      </c>
+      <c r="EK37" s="23">
+        <f>IF(COUNT(EK9:EK36)=0,"",SUM(EK9:EK36))</f>
+        <v/>
+      </c>
+      <c r="EL37" s="23">
+        <f>IF(COUNT(EL9:EL36)=0,"",SUM(EL9:EL36))</f>
+        <v/>
+      </c>
+      <c r="EM37" s="23">
+        <f>IF(COUNT(EM9:EM36)=0,"",SUM(EM9:EM36))</f>
+        <v/>
+      </c>
+      <c r="EN37" s="23">
+        <f>IF(COUNT(EN9:EN36)=0,"",SUM(EN9:EN36))</f>
+        <v/>
+      </c>
+      <c r="EO37" s="23">
+        <f>IF(COUNT(EO9:EO36)=0,"",SUM(EO9:EO36))</f>
+        <v/>
+      </c>
+      <c r="EP37" s="23">
+        <f>IF(COUNT(EP9:EP36)=0,"",SUM(EP9:EP36))</f>
+        <v/>
+      </c>
+      <c r="EQ37" s="23">
+        <f>IF(COUNT(EQ9:EQ36)=0,"",SUM(EQ9:EQ36))</f>
+        <v/>
+      </c>
+      <c r="ER37" s="23">
+        <f>IF(COUNT(ER9:ER36)=0,"",SUM(ER9:ER36))</f>
+        <v/>
+      </c>
+      <c r="ES37" s="23">
+        <f>IF(COUNT(ES9:ES36)=0,"",SUM(ES9:ES36))</f>
+        <v/>
+      </c>
+      <c r="EU37" s="21">
+        <f>SUM(EU9:EU36)</f>
+        <v/>
+      </c>
+      <c r="EV37" s="21">
+        <f>SUM(EV9:EV36)</f>
+        <v/>
+      </c>
+      <c r="EW37" s="21">
+        <f>SUM(EW9:EW36)</f>
+        <v/>
+      </c>
+      <c r="EX37" s="21">
+        <f>SUM(EX9:EX36)</f>
+        <v/>
+      </c>
+      <c r="EY37" s="21">
+        <f>SUM(EY9:EY36)</f>
+        <v/>
+      </c>
+      <c r="EZ37" s="21">
+        <f>SUM(EZ9:EZ36)</f>
+        <v/>
+      </c>
+      <c r="FA37" s="21">
+        <f>SUM(FA9:FA36)</f>
+        <v/>
+      </c>
+      <c r="FB37" s="21">
+        <f>SUM(FB9:FB36)</f>
+        <v/>
+      </c>
+      <c r="FC37" s="21">
+        <f>SUM(FC9:FC36)</f>
+        <v/>
+      </c>
+      <c r="FD37" s="21">
+        <f>SUM(FD9:FD36)</f>
+        <v/>
+      </c>
+      <c r="FE37" s="21">
+        <f>SUM(FE9:FE36)</f>
+        <v/>
+      </c>
+      <c r="FF37" s="21">
+        <f>SUM(FF9:FF36)</f>
+        <v/>
+      </c>
+      <c r="FG37" s="21">
+        <f>SUM(FG9:FG36)</f>
+        <v/>
+      </c>
+      <c r="FH37" s="21">
+        <f>SUM(FH9:FH36)</f>
+        <v/>
+      </c>
+      <c r="FI37" s="21">
+        <f>SUM(FI9:FI36)</f>
+        <v/>
+      </c>
+      <c r="FJ37" s="21">
+        <f>SUM(FJ9:FJ36)</f>
+        <v/>
+      </c>
+      <c r="FK37" s="21">
+        <f>SUM(FK9:FK36)</f>
+        <v/>
+      </c>
+      <c r="FL37" s="21">
+        <f>SUM(FL9:FL36)</f>
+        <v/>
+      </c>
+      <c r="FM37" s="21">
+        <f>SUM(FM9:FM36)</f>
+        <v/>
+      </c>
+      <c r="FN37" s="21">
+        <f>SUM(FN9:FN36)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="B39" s="15" t="n">
-        <v>31</v>
-      </c>
-      <c r="C39" s="15" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="n"/>
-      <c r="E39" s="16" t="n"/>
-      <c r="F39" s="16" t="n"/>
-      <c r="G39" s="16" t="n"/>
-      <c r="H39" s="16" t="n"/>
-      <c r="I39" s="16" t="n"/>
-      <c r="J39" s="16" t="n"/>
-      <c r="K39" s="16" t="n"/>
-      <c r="L39" s="16" t="n"/>
-      <c r="M39" s="16" t="n"/>
-      <c r="N39" s="16" t="n"/>
-      <c r="O39" s="16" t="n"/>
-      <c r="P39" s="16" t="n"/>
-      <c r="Q39" s="16" t="n"/>
-      <c r="R39" s="16" t="n"/>
-      <c r="S39" s="16" t="n"/>
-      <c r="T39" s="16" t="n"/>
-      <c r="U39" s="16" t="n"/>
-      <c r="V39" s="16" t="n"/>
-      <c r="W39" s="16" t="n"/>
-      <c r="Y39" s="16" t="n"/>
-      <c r="Z39" s="16" t="n"/>
-      <c r="AA39" s="16" t="n"/>
-      <c r="AB39" s="16" t="n"/>
-      <c r="AC39" s="16" t="n"/>
-      <c r="AD39" s="16" t="n"/>
-      <c r="AE39" s="16" t="n"/>
-      <c r="AF39" s="16" t="n"/>
-      <c r="AG39" s="16" t="n"/>
-      <c r="AH39" s="16" t="n"/>
-      <c r="AI39" s="16" t="n"/>
-      <c r="AJ39" s="16" t="n"/>
-      <c r="AK39" s="16" t="n"/>
-      <c r="AL39" s="16" t="n"/>
-      <c r="AM39" s="16" t="n"/>
-      <c r="AN39" s="16" t="n"/>
-      <c r="AO39" s="16" t="n"/>
-      <c r="AP39" s="16" t="n"/>
-      <c r="AQ39" s="16" t="n"/>
-      <c r="AR39" s="16" t="n"/>
-      <c r="AT39" s="17" t="n"/>
-      <c r="AU39" s="17" t="n"/>
-      <c r="AV39" s="17" t="n"/>
-      <c r="AW39" s="17" t="n"/>
-      <c r="AX39" s="17" t="n"/>
-      <c r="AY39" s="17" t="n"/>
-      <c r="AZ39" s="17" t="n"/>
-      <c r="BA39" s="17" t="n"/>
-      <c r="BB39" s="17" t="n"/>
-      <c r="BC39" s="17" t="n"/>
-      <c r="BD39" s="17" t="n"/>
-      <c r="BE39" s="17" t="n"/>
-      <c r="BF39" s="17" t="n"/>
-      <c r="BG39" s="17" t="n"/>
-      <c r="BH39" s="17" t="n"/>
-      <c r="BI39" s="17" t="n"/>
-      <c r="BJ39" s="17" t="n"/>
-      <c r="BK39" s="17" t="n"/>
-      <c r="BL39" s="17" t="n"/>
-      <c r="BM39" s="17" t="n"/>
-      <c r="BO39" s="16" t="n"/>
-      <c r="BP39" s="16" t="n"/>
-      <c r="BQ39" s="16" t="n"/>
-      <c r="BR39" s="16" t="n"/>
-      <c r="BS39" s="16" t="n"/>
-      <c r="BT39" s="16" t="n"/>
-      <c r="BU39" s="16" t="n"/>
-      <c r="BV39" s="16" t="n"/>
-      <c r="BW39" s="16" t="n"/>
-      <c r="BX39" s="16" t="n"/>
-      <c r="BY39" s="16" t="n"/>
-      <c r="BZ39" s="16" t="n"/>
-      <c r="CA39" s="16" t="n"/>
-      <c r="CB39" s="16" t="n"/>
-      <c r="CC39" s="16" t="n"/>
-      <c r="CD39" s="16" t="n"/>
-      <c r="CE39" s="16" t="n"/>
-      <c r="CF39" s="16" t="n"/>
-      <c r="CG39" s="16" t="n"/>
-      <c r="CH39" s="16" t="n"/>
-      <c r="CJ39" s="18" t="n"/>
-      <c r="CK39" s="18" t="n"/>
-      <c r="CL39" s="18" t="n"/>
-      <c r="CM39" s="18" t="n"/>
-      <c r="CN39" s="18" t="n"/>
-      <c r="CO39" s="18" t="n"/>
-      <c r="CP39" s="18" t="n"/>
-      <c r="CQ39" s="18" t="n"/>
-      <c r="CR39" s="18" t="n"/>
-      <c r="CS39" s="18" t="n"/>
-      <c r="CT39" s="18" t="n"/>
-      <c r="CU39" s="18" t="n"/>
-      <c r="CV39" s="18" t="n"/>
-      <c r="CW39" s="18" t="n"/>
-      <c r="CX39" s="18" t="n"/>
-      <c r="CY39" s="18" t="n"/>
-      <c r="CZ39" s="18" t="n"/>
-      <c r="DA39" s="18" t="n"/>
-      <c r="DB39" s="18" t="n"/>
-      <c r="DC39" s="18" t="n"/>
-      <c r="DE39" s="18" t="n"/>
-      <c r="DF39" s="18" t="n"/>
-      <c r="DG39" s="18" t="n"/>
-      <c r="DH39" s="18" t="n"/>
-      <c r="DI39" s="18" t="n"/>
-      <c r="DJ39" s="18" t="n"/>
-      <c r="DK39" s="18" t="n"/>
-      <c r="DL39" s="18" t="n"/>
-      <c r="DM39" s="18" t="n"/>
-      <c r="DN39" s="18" t="n"/>
-      <c r="DO39" s="18" t="n"/>
-      <c r="DP39" s="18" t="n"/>
-      <c r="DQ39" s="18" t="n"/>
-      <c r="DR39" s="18" t="n"/>
-      <c r="DS39" s="18" t="n"/>
-      <c r="DT39" s="18" t="n"/>
-      <c r="DU39" s="18" t="n"/>
-      <c r="DV39" s="18" t="n"/>
-      <c r="DW39" s="18" t="n"/>
-      <c r="DX39" s="18" t="n"/>
-      <c r="DZ39" s="17">
-        <f>IF(OR(CJ39="",DE39=""),"",IFERROR(CJ39-DE39,""))</f>
-        <v/>
-      </c>
-      <c r="EA39" s="17">
-        <f>IF(OR(CK39="",DF39=""),"",IFERROR(CK39-DF39,""))</f>
-        <v/>
-      </c>
-      <c r="EB39" s="17">
-        <f>IF(OR(CL39="",DG39=""),"",IFERROR(CL39-DG39,""))</f>
-        <v/>
-      </c>
-      <c r="EC39" s="17">
-        <f>IF(OR(CM39="",DH39=""),"",IFERROR(CM39-DH39,""))</f>
-        <v/>
-      </c>
-      <c r="ED39" s="17">
-        <f>IF(OR(CN39="",DI39=""),"",IFERROR(CN39-DI39,""))</f>
-        <v/>
-      </c>
-      <c r="EE39" s="17">
-        <f>IF(OR(CO39="",DJ39=""),"",IFERROR(CO39-DJ39,""))</f>
-        <v/>
-      </c>
-      <c r="EF39" s="17">
-        <f>IF(OR(CP39="",DK39=""),"",IFERROR(CP39-DK39,""))</f>
-        <v/>
-      </c>
-      <c r="EG39" s="17">
-        <f>IF(OR(CQ39="",DL39=""),"",IFERROR(CQ39-DL39,""))</f>
-        <v/>
-      </c>
-      <c r="EH39" s="17">
-        <f>IF(OR(CR39="",DM39=""),"",IFERROR(CR39-DM39,""))</f>
-        <v/>
-      </c>
-      <c r="EI39" s="17">
-        <f>IF(OR(CS39="",DN39=""),"",IFERROR(CS39-DN39,""))</f>
-        <v/>
-      </c>
-      <c r="EJ39" s="17">
-        <f>IF(OR(CT39="",DO39=""),"",IFERROR(CT39-DO39,""))</f>
-        <v/>
-      </c>
-      <c r="EK39" s="17">
-        <f>IF(OR(CU39="",DP39=""),"",IFERROR(CU39-DP39,""))</f>
-        <v/>
-      </c>
-      <c r="EL39" s="17">
-        <f>IF(OR(CV39="",DQ39=""),"",IFERROR(CV39-DQ39,""))</f>
-        <v/>
-      </c>
-      <c r="EM39" s="17">
-        <f>IF(OR(CW39="",DR39=""),"",IFERROR(CW39-DR39,""))</f>
-        <v/>
-      </c>
-      <c r="EN39" s="17">
-        <f>IF(OR(CX39="",DS39=""),"",IFERROR(CX39-DS39,""))</f>
-        <v/>
-      </c>
-      <c r="EO39" s="17">
-        <f>IF(OR(CY39="",DT39=""),"",IFERROR(CY39-DT39,""))</f>
-        <v/>
-      </c>
-      <c r="EP39" s="17">
-        <f>IF(OR(CZ39="",DU39=""),"",IFERROR(CZ39-DU39,""))</f>
-        <v/>
-      </c>
-      <c r="EQ39" s="17">
-        <f>IF(OR(DA39="",DV39=""),"",IFERROR(DA39-DV39,""))</f>
-        <v/>
-      </c>
-      <c r="ER39" s="17">
-        <f>IF(OR(DB39="",DW39=""),"",IFERROR(DB39-DW39,""))</f>
-        <v/>
-      </c>
-      <c r="ES39" s="17">
-        <f>IF(OR(DC39="",DX39=""),"",IFERROR(DC39-DX39,""))</f>
-        <v/>
-      </c>
-      <c r="EU39" s="16" t="n"/>
-      <c r="EV39" s="16" t="n"/>
-      <c r="EW39" s="16" t="n"/>
-      <c r="EX39" s="16" t="n"/>
-      <c r="EY39" s="16" t="n"/>
-      <c r="EZ39" s="16" t="n"/>
-      <c r="FA39" s="16" t="n"/>
-      <c r="FB39" s="16" t="n"/>
-      <c r="FC39" s="16" t="n"/>
-      <c r="FD39" s="16" t="n"/>
-      <c r="FE39" s="16" t="n"/>
-      <c r="FF39" s="16" t="n"/>
-      <c r="FG39" s="16" t="n"/>
-      <c r="FH39" s="16" t="n"/>
-      <c r="FI39" s="16" t="n"/>
-      <c r="FJ39" s="16" t="n"/>
-      <c r="FK39" s="16" t="n"/>
-      <c r="FL39" s="16" t="n"/>
-      <c r="FM39" s="16" t="n"/>
-      <c r="FN39" s="16" t="n"/>
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>LEGEND / ALLOCATION RULES (D60, 2026-10-14 — EcoGainsSim_Daily.gs, DAILY_ALLOC_MODEL = settle)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="B40" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="n"/>
-      <c r="E40" s="16" t="n"/>
-      <c r="F40" s="16" t="n"/>
-      <c r="G40" s="16" t="n"/>
-      <c r="H40" s="16" t="n"/>
-      <c r="I40" s="16" t="n"/>
-      <c r="J40" s="16" t="n"/>
-      <c r="K40" s="16" t="n"/>
-      <c r="L40" s="16" t="n"/>
-      <c r="M40" s="16" t="n"/>
-      <c r="N40" s="16" t="n"/>
-      <c r="O40" s="16" t="n"/>
-      <c r="P40" s="16" t="n"/>
-      <c r="Q40" s="16" t="n"/>
-      <c r="R40" s="16" t="n"/>
-      <c r="S40" s="16" t="n"/>
-      <c r="T40" s="16" t="n"/>
-      <c r="U40" s="16" t="n"/>
-      <c r="V40" s="16" t="n"/>
-      <c r="W40" s="16" t="n"/>
-      <c r="Y40" s="16" t="n"/>
-      <c r="Z40" s="16" t="n"/>
-      <c r="AA40" s="16" t="n"/>
-      <c r="AB40" s="16" t="n"/>
-      <c r="AC40" s="16" t="n"/>
-      <c r="AD40" s="16" t="n"/>
-      <c r="AE40" s="16" t="n"/>
-      <c r="AF40" s="16" t="n"/>
-      <c r="AG40" s="16" t="n"/>
-      <c r="AH40" s="16" t="n"/>
-      <c r="AI40" s="16" t="n"/>
-      <c r="AJ40" s="16" t="n"/>
-      <c r="AK40" s="16" t="n"/>
-      <c r="AL40" s="16" t="n"/>
-      <c r="AM40" s="16" t="n"/>
-      <c r="AN40" s="16" t="n"/>
-      <c r="AO40" s="16" t="n"/>
-      <c r="AP40" s="16" t="n"/>
-      <c r="AQ40" s="16" t="n"/>
-      <c r="AR40" s="16" t="n"/>
-      <c r="AT40" s="17" t="n"/>
-      <c r="AU40" s="17" t="n"/>
-      <c r="AV40" s="17" t="n"/>
-      <c r="AW40" s="17" t="n"/>
-      <c r="AX40" s="17" t="n"/>
-      <c r="AY40" s="17" t="n"/>
-      <c r="AZ40" s="17" t="n"/>
-      <c r="BA40" s="17" t="n"/>
-      <c r="BB40" s="17" t="n"/>
-      <c r="BC40" s="17" t="n"/>
-      <c r="BD40" s="17" t="n"/>
-      <c r="BE40" s="17" t="n"/>
-      <c r="BF40" s="17" t="n"/>
-      <c r="BG40" s="17" t="n"/>
-      <c r="BH40" s="17" t="n"/>
-      <c r="BI40" s="17" t="n"/>
-      <c r="BJ40" s="17" t="n"/>
-      <c r="BK40" s="17" t="n"/>
-      <c r="BL40" s="17" t="n"/>
-      <c r="BM40" s="17" t="n"/>
-      <c r="BO40" s="16" t="n"/>
-      <c r="BP40" s="16" t="n"/>
-      <c r="BQ40" s="16" t="n"/>
-      <c r="BR40" s="16" t="n"/>
-      <c r="BS40" s="16" t="n"/>
-      <c r="BT40" s="16" t="n"/>
-      <c r="BU40" s="16" t="n"/>
-      <c r="BV40" s="16" t="n"/>
-      <c r="BW40" s="16" t="n"/>
-      <c r="BX40" s="16" t="n"/>
-      <c r="BY40" s="16" t="n"/>
-      <c r="BZ40" s="16" t="n"/>
-      <c r="CA40" s="16" t="n"/>
-      <c r="CB40" s="16" t="n"/>
-      <c r="CC40" s="16" t="n"/>
-      <c r="CD40" s="16" t="n"/>
-      <c r="CE40" s="16" t="n"/>
-      <c r="CF40" s="16" t="n"/>
-      <c r="CG40" s="16" t="n"/>
-      <c r="CH40" s="16" t="n"/>
-      <c r="CJ40" s="18" t="n"/>
-      <c r="CK40" s="18" t="n"/>
-      <c r="CL40" s="18" t="n"/>
-      <c r="CM40" s="18" t="n"/>
-      <c r="CN40" s="18" t="n"/>
-      <c r="CO40" s="18" t="n"/>
-      <c r="CP40" s="18" t="n"/>
-      <c r="CQ40" s="18" t="n"/>
-      <c r="CR40" s="18" t="n"/>
-      <c r="CS40" s="18" t="n"/>
-      <c r="CT40" s="18" t="n"/>
-      <c r="CU40" s="18" t="n"/>
-      <c r="CV40" s="18" t="n"/>
-      <c r="CW40" s="18" t="n"/>
-      <c r="CX40" s="18" t="n"/>
-      <c r="CY40" s="18" t="n"/>
-      <c r="CZ40" s="18" t="n"/>
-      <c r="DA40" s="18" t="n"/>
-      <c r="DB40" s="18" t="n"/>
-      <c r="DC40" s="18" t="n"/>
-      <c r="DE40" s="18" t="n"/>
-      <c r="DF40" s="18" t="n"/>
-      <c r="DG40" s="18" t="n"/>
-      <c r="DH40" s="18" t="n"/>
-      <c r="DI40" s="18" t="n"/>
-      <c r="DJ40" s="18" t="n"/>
-      <c r="DK40" s="18" t="n"/>
-      <c r="DL40" s="18" t="n"/>
-      <c r="DM40" s="18" t="n"/>
-      <c r="DN40" s="18" t="n"/>
-      <c r="DO40" s="18" t="n"/>
-      <c r="DP40" s="18" t="n"/>
-      <c r="DQ40" s="18" t="n"/>
-      <c r="DR40" s="18" t="n"/>
-      <c r="DS40" s="18" t="n"/>
-      <c r="DT40" s="18" t="n"/>
-      <c r="DU40" s="18" t="n"/>
-      <c r="DV40" s="18" t="n"/>
-      <c r="DW40" s="18" t="n"/>
-      <c r="DX40" s="18" t="n"/>
-      <c r="DZ40" s="17">
-        <f>IF(OR(CJ40="",DE40=""),"",IFERROR(CJ40-DE40,""))</f>
-        <v/>
-      </c>
-      <c r="EA40" s="17">
-        <f>IF(OR(CK40="",DF40=""),"",IFERROR(CK40-DF40,""))</f>
-        <v/>
-      </c>
-      <c r="EB40" s="17">
-        <f>IF(OR(CL40="",DG40=""),"",IFERROR(CL40-DG40,""))</f>
-        <v/>
-      </c>
-      <c r="EC40" s="17">
-        <f>IF(OR(CM40="",DH40=""),"",IFERROR(CM40-DH40,""))</f>
-        <v/>
-      </c>
-      <c r="ED40" s="17">
-        <f>IF(OR(CN40="",DI40=""),"",IFERROR(CN40-DI40,""))</f>
-        <v/>
-      </c>
-      <c r="EE40" s="17">
-        <f>IF(OR(CO40="",DJ40=""),"",IFERROR(CO40-DJ40,""))</f>
-        <v/>
-      </c>
-      <c r="EF40" s="17">
-        <f>IF(OR(CP40="",DK40=""),"",IFERROR(CP40-DK40,""))</f>
-        <v/>
-      </c>
-      <c r="EG40" s="17">
-        <f>IF(OR(CQ40="",DL40=""),"",IFERROR(CQ40-DL40,""))</f>
-        <v/>
-      </c>
-      <c r="EH40" s="17">
-        <f>IF(OR(CR40="",DM40=""),"",IFERROR(CR40-DM40,""))</f>
-        <v/>
-      </c>
-      <c r="EI40" s="17">
-        <f>IF(OR(CS40="",DN40=""),"",IFERROR(CS40-DN40,""))</f>
-        <v/>
-      </c>
-      <c r="EJ40" s="17">
-        <f>IF(OR(CT40="",DO40=""),"",IFERROR(CT40-DO40,""))</f>
-        <v/>
-      </c>
-      <c r="EK40" s="17">
-        <f>IF(OR(CU40="",DP40=""),"",IFERROR(CU40-DP40,""))</f>
-        <v/>
-      </c>
-      <c r="EL40" s="17">
-        <f>IF(OR(CV40="",DQ40=""),"",IFERROR(CV40-DQ40,""))</f>
-        <v/>
-      </c>
-      <c r="EM40" s="17">
-        <f>IF(OR(CW40="",DR40=""),"",IFERROR(CW40-DR40,""))</f>
-        <v/>
-      </c>
-      <c r="EN40" s="17">
-        <f>IF(OR(CX40="",DS40=""),"",IFERROR(CX40-DS40,""))</f>
-        <v/>
-      </c>
-      <c r="EO40" s="17">
-        <f>IF(OR(CY40="",DT40=""),"",IFERROR(CY40-DT40,""))</f>
-        <v/>
-      </c>
-      <c r="EP40" s="17">
-        <f>IF(OR(CZ40="",DU40=""),"",IFERROR(CZ40-DU40,""))</f>
-        <v/>
-      </c>
-      <c r="EQ40" s="17">
-        <f>IF(OR(DA40="",DV40=""),"",IFERROR(DA40-DV40,""))</f>
-        <v/>
-      </c>
-      <c r="ER40" s="17">
-        <f>IF(OR(DB40="",DW40=""),"",IFERROR(DB40-DW40,""))</f>
-        <v/>
-      </c>
-      <c r="ES40" s="17">
-        <f>IF(OR(DC40="",DX40=""),"",IFERROR(DC40-DX40,""))</f>
-        <v/>
-      </c>
-      <c r="EU40" s="16" t="n"/>
-      <c r="EV40" s="16" t="n"/>
-      <c r="EW40" s="16" t="n"/>
-      <c r="EX40" s="16" t="n"/>
-      <c r="EY40" s="16" t="n"/>
-      <c r="EZ40" s="16" t="n"/>
-      <c r="FA40" s="16" t="n"/>
-      <c r="FB40" s="16" t="n"/>
-      <c r="FC40" s="16" t="n"/>
-      <c r="FD40" s="16" t="n"/>
-      <c r="FE40" s="16" t="n"/>
-      <c r="FF40" s="16" t="n"/>
-      <c r="FG40" s="16" t="n"/>
-      <c r="FH40" s="16" t="n"/>
-      <c r="FI40" s="16" t="n"/>
-      <c r="FJ40" s="16" t="n"/>
-      <c r="FK40" s="16" t="n"/>
-      <c r="FL40" s="16" t="n"/>
-      <c r="FM40" s="16" t="n"/>
-      <c r="FN40" s="16" t="n"/>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>CURRENT GAINS, CURRENT SPEND, CURRENT NET are DATA: data_econ_daily, per earner per day (window-earner denominator, so the days of the pull sum to the data_econ window total). They are BLANK past the last day the pull carries — a day with no row is "not pulled yet", never 0 — and blank unless Source = ALL (the data is game-wide).</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="B41" s="15" t="n">
-        <v>33</v>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="n"/>
-      <c r="E41" s="16" t="n"/>
-      <c r="F41" s="16" t="n"/>
-      <c r="G41" s="16" t="n"/>
-      <c r="H41" s="16" t="n"/>
-      <c r="I41" s="16" t="n"/>
-      <c r="J41" s="16" t="n"/>
-      <c r="K41" s="16" t="n"/>
-      <c r="L41" s="16" t="n"/>
-      <c r="M41" s="16" t="n"/>
-      <c r="N41" s="16" t="n"/>
-      <c r="O41" s="16" t="n"/>
-      <c r="P41" s="16" t="n"/>
-      <c r="Q41" s="16" t="n"/>
-      <c r="R41" s="16" t="n"/>
-      <c r="S41" s="16" t="n"/>
-      <c r="T41" s="16" t="n"/>
-      <c r="U41" s="16" t="n"/>
-      <c r="V41" s="16" t="n"/>
-      <c r="W41" s="16" t="n"/>
-      <c r="Y41" s="16" t="n"/>
-      <c r="Z41" s="16" t="n"/>
-      <c r="AA41" s="16" t="n"/>
-      <c r="AB41" s="16" t="n"/>
-      <c r="AC41" s="16" t="n"/>
-      <c r="AD41" s="16" t="n"/>
-      <c r="AE41" s="16" t="n"/>
-      <c r="AF41" s="16" t="n"/>
-      <c r="AG41" s="16" t="n"/>
-      <c r="AH41" s="16" t="n"/>
-      <c r="AI41" s="16" t="n"/>
-      <c r="AJ41" s="16" t="n"/>
-      <c r="AK41" s="16" t="n"/>
-      <c r="AL41" s="16" t="n"/>
-      <c r="AM41" s="16" t="n"/>
-      <c r="AN41" s="16" t="n"/>
-      <c r="AO41" s="16" t="n"/>
-      <c r="AP41" s="16" t="n"/>
-      <c r="AQ41" s="16" t="n"/>
-      <c r="AR41" s="16" t="n"/>
-      <c r="AT41" s="17" t="n"/>
-      <c r="AU41" s="17" t="n"/>
-      <c r="AV41" s="17" t="n"/>
-      <c r="AW41" s="17" t="n"/>
-      <c r="AX41" s="17" t="n"/>
-      <c r="AY41" s="17" t="n"/>
-      <c r="AZ41" s="17" t="n"/>
-      <c r="BA41" s="17" t="n"/>
-      <c r="BB41" s="17" t="n"/>
-      <c r="BC41" s="17" t="n"/>
-      <c r="BD41" s="17" t="n"/>
-      <c r="BE41" s="17" t="n"/>
-      <c r="BF41" s="17" t="n"/>
-      <c r="BG41" s="17" t="n"/>
-      <c r="BH41" s="17" t="n"/>
-      <c r="BI41" s="17" t="n"/>
-      <c r="BJ41" s="17" t="n"/>
-      <c r="BK41" s="17" t="n"/>
-      <c r="BL41" s="17" t="n"/>
-      <c r="BM41" s="17" t="n"/>
-      <c r="BO41" s="16" t="n"/>
-      <c r="BP41" s="16" t="n"/>
-      <c r="BQ41" s="16" t="n"/>
-      <c r="BR41" s="16" t="n"/>
-      <c r="BS41" s="16" t="n"/>
-      <c r="BT41" s="16" t="n"/>
-      <c r="BU41" s="16" t="n"/>
-      <c r="BV41" s="16" t="n"/>
-      <c r="BW41" s="16" t="n"/>
-      <c r="BX41" s="16" t="n"/>
-      <c r="BY41" s="16" t="n"/>
-      <c r="BZ41" s="16" t="n"/>
-      <c r="CA41" s="16" t="n"/>
-      <c r="CB41" s="16" t="n"/>
-      <c r="CC41" s="16" t="n"/>
-      <c r="CD41" s="16" t="n"/>
-      <c r="CE41" s="16" t="n"/>
-      <c r="CF41" s="16" t="n"/>
-      <c r="CG41" s="16" t="n"/>
-      <c r="CH41" s="16" t="n"/>
-      <c r="CJ41" s="18" t="n"/>
-      <c r="CK41" s="18" t="n"/>
-      <c r="CL41" s="18" t="n"/>
-      <c r="CM41" s="18" t="n"/>
-      <c r="CN41" s="18" t="n"/>
-      <c r="CO41" s="18" t="n"/>
-      <c r="CP41" s="18" t="n"/>
-      <c r="CQ41" s="18" t="n"/>
-      <c r="CR41" s="18" t="n"/>
-      <c r="CS41" s="18" t="n"/>
-      <c r="CT41" s="18" t="n"/>
-      <c r="CU41" s="18" t="n"/>
-      <c r="CV41" s="18" t="n"/>
-      <c r="CW41" s="18" t="n"/>
-      <c r="CX41" s="18" t="n"/>
-      <c r="CY41" s="18" t="n"/>
-      <c r="CZ41" s="18" t="n"/>
-      <c r="DA41" s="18" t="n"/>
-      <c r="DB41" s="18" t="n"/>
-      <c r="DC41" s="18" t="n"/>
-      <c r="DE41" s="18" t="n"/>
-      <c r="DF41" s="18" t="n"/>
-      <c r="DG41" s="18" t="n"/>
-      <c r="DH41" s="18" t="n"/>
-      <c r="DI41" s="18" t="n"/>
-      <c r="DJ41" s="18" t="n"/>
-      <c r="DK41" s="18" t="n"/>
-      <c r="DL41" s="18" t="n"/>
-      <c r="DM41" s="18" t="n"/>
-      <c r="DN41" s="18" t="n"/>
-      <c r="DO41" s="18" t="n"/>
-      <c r="DP41" s="18" t="n"/>
-      <c r="DQ41" s="18" t="n"/>
-      <c r="DR41" s="18" t="n"/>
-      <c r="DS41" s="18" t="n"/>
-      <c r="DT41" s="18" t="n"/>
-      <c r="DU41" s="18" t="n"/>
-      <c r="DV41" s="18" t="n"/>
-      <c r="DW41" s="18" t="n"/>
-      <c r="DX41" s="18" t="n"/>
-      <c r="DZ41" s="17">
-        <f>IF(OR(CJ41="",DE41=""),"",IFERROR(CJ41-DE41,""))</f>
-        <v/>
-      </c>
-      <c r="EA41" s="17">
-        <f>IF(OR(CK41="",DF41=""),"",IFERROR(CK41-DF41,""))</f>
-        <v/>
-      </c>
-      <c r="EB41" s="17">
-        <f>IF(OR(CL41="",DG41=""),"",IFERROR(CL41-DG41,""))</f>
-        <v/>
-      </c>
-      <c r="EC41" s="17">
-        <f>IF(OR(CM41="",DH41=""),"",IFERROR(CM41-DH41,""))</f>
-        <v/>
-      </c>
-      <c r="ED41" s="17">
-        <f>IF(OR(CN41="",DI41=""),"",IFERROR(CN41-DI41,""))</f>
-        <v/>
-      </c>
-      <c r="EE41" s="17">
-        <f>IF(OR(CO41="",DJ41=""),"",IFERROR(CO41-DJ41,""))</f>
-        <v/>
-      </c>
-      <c r="EF41" s="17">
-        <f>IF(OR(CP41="",DK41=""),"",IFERROR(CP41-DK41,""))</f>
-        <v/>
-      </c>
-      <c r="EG41" s="17">
-        <f>IF(OR(CQ41="",DL41=""),"",IFERROR(CQ41-DL41,""))</f>
-        <v/>
-      </c>
-      <c r="EH41" s="17">
-        <f>IF(OR(CR41="",DM41=""),"",IFERROR(CR41-DM41,""))</f>
-        <v/>
-      </c>
-      <c r="EI41" s="17">
-        <f>IF(OR(CS41="",DN41=""),"",IFERROR(CS41-DN41,""))</f>
-        <v/>
-      </c>
-      <c r="EJ41" s="17">
-        <f>IF(OR(CT41="",DO41=""),"",IFERROR(CT41-DO41,""))</f>
-        <v/>
-      </c>
-      <c r="EK41" s="17">
-        <f>IF(OR(CU41="",DP41=""),"",IFERROR(CU41-DP41,""))</f>
-        <v/>
-      </c>
-      <c r="EL41" s="17">
-        <f>IF(OR(CV41="",DQ41=""),"",IFERROR(CV41-DQ41,""))</f>
-        <v/>
-      </c>
-      <c r="EM41" s="17">
-        <f>IF(OR(CW41="",DR41=""),"",IFERROR(CW41-DR41,""))</f>
-        <v/>
-      </c>
-      <c r="EN41" s="17">
-        <f>IF(OR(CX41="",DS41=""),"",IFERROR(CX41-DS41,""))</f>
-        <v/>
-      </c>
-      <c r="EO41" s="17">
-        <f>IF(OR(CY41="",DT41=""),"",IFERROR(CY41-DT41,""))</f>
-        <v/>
-      </c>
-      <c r="EP41" s="17">
-        <f>IF(OR(CZ41="",DU41=""),"",IFERROR(CZ41-DU41,""))</f>
-        <v/>
-      </c>
-      <c r="EQ41" s="17">
-        <f>IF(OR(DA41="",DV41=""),"",IFERROR(DA41-DV41,""))</f>
-        <v/>
-      </c>
-      <c r="ER41" s="17">
-        <f>IF(OR(DB41="",DW41=""),"",IFERROR(DB41-DW41,""))</f>
-        <v/>
-      </c>
-      <c r="ES41" s="17">
-        <f>IF(OR(DC41="",DX41=""),"",IFERROR(DC41-DX41,""))</f>
-        <v/>
-      </c>
-      <c r="EU41" s="16" t="n"/>
-      <c r="EV41" s="16" t="n"/>
-      <c r="EW41" s="16" t="n"/>
-      <c r="EX41" s="16" t="n"/>
-      <c r="EY41" s="16" t="n"/>
-      <c r="EZ41" s="16" t="n"/>
-      <c r="FA41" s="16" t="n"/>
-      <c r="FB41" s="16" t="n"/>
-      <c r="FC41" s="16" t="n"/>
-      <c r="FD41" s="16" t="n"/>
-      <c r="FE41" s="16" t="n"/>
-      <c r="FF41" s="16" t="n"/>
-      <c r="FG41" s="16" t="n"/>
-      <c r="FH41" s="16" t="n"/>
-      <c r="FI41" s="16" t="n"/>
-      <c r="FJ41" s="16" t="n"/>
-      <c r="FK41" s="16" t="n"/>
-      <c r="FL41" s="16" t="n"/>
-      <c r="FM41" s="16" t="n"/>
-      <c r="FN41" s="16" t="n"/>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>NEW GAINS is the SIM of cal_new. Δ GAINS = data − sim: positive means the data sits above the sim. While cal_curr is the live calendar this Δ mixes the redesign with model error; the validation lane on the far right (SIM of cal_curr) separates them: data − sim_new = (data − sim_curr) + (sim_curr − sim_new).</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="B42" s="19" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C42" s="20" t="n"/>
-      <c r="D42" s="21">
-        <f>IF(COUNT(D9:D41)=0,"",SUM(D9:D41))</f>
-        <v/>
-      </c>
-      <c r="E42" s="21">
-        <f>IF(COUNT(E9:E41)=0,"",SUM(E9:E41))</f>
-        <v/>
-      </c>
-      <c r="F42" s="21">
-        <f>IF(COUNT(F9:F41)=0,"",SUM(F9:F41))</f>
-        <v/>
-      </c>
-      <c r="G42" s="21">
-        <f>IF(COUNT(G9:G41)=0,"",SUM(G9:G41))</f>
-        <v/>
-      </c>
-      <c r="H42" s="21">
-        <f>IF(COUNT(H9:H41)=0,"",SUM(H9:H41))</f>
-        <v/>
-      </c>
-      <c r="I42" s="21">
-        <f>IF(COUNT(I9:I41)=0,"",SUM(I9:I41))</f>
-        <v/>
-      </c>
-      <c r="J42" s="21">
-        <f>IF(COUNT(J9:J41)=0,"",SUM(J9:J41))</f>
-        <v/>
-      </c>
-      <c r="K42" s="21">
-        <f>IF(COUNT(K9:K41)=0,"",SUM(K9:K41))</f>
-        <v/>
-      </c>
-      <c r="L42" s="21">
-        <f>IF(COUNT(L9:L41)=0,"",SUM(L9:L41))</f>
-        <v/>
-      </c>
-      <c r="M42" s="21">
-        <f>IF(COUNT(M9:M41)=0,"",SUM(M9:M41))</f>
-        <v/>
-      </c>
-      <c r="N42" s="21">
-        <f>IF(COUNT(N9:N41)=0,"",SUM(N9:N41))</f>
-        <v/>
-      </c>
-      <c r="O42" s="21">
-        <f>IF(COUNT(O9:O41)=0,"",SUM(O9:O41))</f>
-        <v/>
-      </c>
-      <c r="P42" s="21">
-        <f>IF(COUNT(P9:P41)=0,"",SUM(P9:P41))</f>
-        <v/>
-      </c>
-      <c r="Q42" s="21">
-        <f>IF(COUNT(Q9:Q41)=0,"",SUM(Q9:Q41))</f>
-        <v/>
-      </c>
-      <c r="R42" s="21">
-        <f>IF(COUNT(R9:R41)=0,"",SUM(R9:R41))</f>
-        <v/>
-      </c>
-      <c r="S42" s="21">
-        <f>IF(COUNT(S9:S41)=0,"",SUM(S9:S41))</f>
-        <v/>
-      </c>
-      <c r="T42" s="21">
-        <f>IF(COUNT(T9:T41)=0,"",SUM(T9:T41))</f>
-        <v/>
-      </c>
-      <c r="U42" s="21">
-        <f>IF(COUNT(U9:U41)=0,"",SUM(U9:U41))</f>
-        <v/>
-      </c>
-      <c r="V42" s="21">
-        <f>IF(COUNT(V9:V41)=0,"",SUM(V9:V41))</f>
-        <v/>
-      </c>
-      <c r="W42" s="21">
-        <f>IF(COUNT(W9:W41)=0,"",SUM(W9:W41))</f>
-        <v/>
-      </c>
-      <c r="Y42" s="22">
-        <f>SUM(Y9:Y41)</f>
-        <v/>
-      </c>
-      <c r="Z42" s="22">
-        <f>SUM(Z9:Z41)</f>
-        <v/>
-      </c>
-      <c r="AA42" s="22">
-        <f>SUM(AA9:AA41)</f>
-        <v/>
-      </c>
-      <c r="AB42" s="22">
-        <f>SUM(AB9:AB41)</f>
-        <v/>
-      </c>
-      <c r="AC42" s="22">
-        <f>SUM(AC9:AC41)</f>
-        <v/>
-      </c>
-      <c r="AD42" s="22">
-        <f>SUM(AD9:AD41)</f>
-        <v/>
-      </c>
-      <c r="AE42" s="22">
-        <f>SUM(AE9:AE41)</f>
-        <v/>
-      </c>
-      <c r="AF42" s="22">
-        <f>SUM(AF9:AF41)</f>
-        <v/>
-      </c>
-      <c r="AG42" s="22">
-        <f>SUM(AG9:AG41)</f>
-        <v/>
-      </c>
-      <c r="AH42" s="22">
-        <f>SUM(AH9:AH41)</f>
-        <v/>
-      </c>
-      <c r="AI42" s="22">
-        <f>SUM(AI9:AI41)</f>
-        <v/>
-      </c>
-      <c r="AJ42" s="22">
-        <f>SUM(AJ9:AJ41)</f>
-        <v/>
-      </c>
-      <c r="AK42" s="22">
-        <f>SUM(AK9:AK41)</f>
-        <v/>
-      </c>
-      <c r="AL42" s="22">
-        <f>SUM(AL9:AL41)</f>
-        <v/>
-      </c>
-      <c r="AM42" s="22">
-        <f>SUM(AM9:AM41)</f>
-        <v/>
-      </c>
-      <c r="AN42" s="22">
-        <f>SUM(AN9:AN41)</f>
-        <v/>
-      </c>
-      <c r="AO42" s="22">
-        <f>SUM(AO9:AO41)</f>
-        <v/>
-      </c>
-      <c r="AP42" s="22">
-        <f>SUM(AP9:AP41)</f>
-        <v/>
-      </c>
-      <c r="AQ42" s="22">
-        <f>SUM(AQ9:AQ41)</f>
-        <v/>
-      </c>
-      <c r="AR42" s="22">
-        <f>SUM(AR9:AR41)</f>
-        <v/>
-      </c>
-      <c r="AT42" s="23">
-        <f>IF(COUNT(AT9:AT41)=0,"",SUM(AT9:AT41))</f>
-        <v/>
-      </c>
-      <c r="AU42" s="23">
-        <f>IF(COUNT(AU9:AU41)=0,"",SUM(AU9:AU41))</f>
-        <v/>
-      </c>
-      <c r="AV42" s="23">
-        <f>IF(COUNT(AV9:AV41)=0,"",SUM(AV9:AV41))</f>
-        <v/>
-      </c>
-      <c r="AW42" s="23">
-        <f>IF(COUNT(AW9:AW41)=0,"",SUM(AW9:AW41))</f>
-        <v/>
-      </c>
-      <c r="AX42" s="23">
-        <f>IF(COUNT(AX9:AX41)=0,"",SUM(AX9:AX41))</f>
-        <v/>
-      </c>
-      <c r="AY42" s="23">
-        <f>IF(COUNT(AY9:AY41)=0,"",SUM(AY9:AY41))</f>
-        <v/>
-      </c>
-      <c r="AZ42" s="23">
-        <f>IF(COUNT(AZ9:AZ41)=0,"",SUM(AZ9:AZ41))</f>
-        <v/>
-      </c>
-      <c r="BA42" s="23">
-        <f>IF(COUNT(BA9:BA41)=0,"",SUM(BA9:BA41))</f>
-        <v/>
-      </c>
-      <c r="BB42" s="23">
-        <f>IF(COUNT(BB9:BB41)=0,"",SUM(BB9:BB41))</f>
-        <v/>
-      </c>
-      <c r="BC42" s="23">
-        <f>IF(COUNT(BC9:BC41)=0,"",SUM(BC9:BC41))</f>
-        <v/>
-      </c>
-      <c r="BD42" s="23">
-        <f>IF(COUNT(BD9:BD41)=0,"",SUM(BD9:BD41))</f>
-        <v/>
-      </c>
-      <c r="BE42" s="23">
-        <f>IF(COUNT(BE9:BE41)=0,"",SUM(BE9:BE41))</f>
-        <v/>
-      </c>
-      <c r="BF42" s="23">
-        <f>IF(COUNT(BF9:BF41)=0,"",SUM(BF9:BF41))</f>
-        <v/>
-      </c>
-      <c r="BG42" s="23">
-        <f>IF(COUNT(BG9:BG41)=0,"",SUM(BG9:BG41))</f>
-        <v/>
-      </c>
-      <c r="BH42" s="23">
-        <f>IF(COUNT(BH9:BH41)=0,"",SUM(BH9:BH41))</f>
-        <v/>
-      </c>
-      <c r="BI42" s="23">
-        <f>IF(COUNT(BI9:BI41)=0,"",SUM(BI9:BI41))</f>
-        <v/>
-      </c>
-      <c r="BJ42" s="23">
-        <f>IF(COUNT(BJ9:BJ41)=0,"",SUM(BJ9:BJ41))</f>
-        <v/>
-      </c>
-      <c r="BK42" s="23">
-        <f>IF(COUNT(BK9:BK41)=0,"",SUM(BK9:BK41))</f>
-        <v/>
-      </c>
-      <c r="BL42" s="23">
-        <f>IF(COUNT(BL9:BL41)=0,"",SUM(BL9:BL41))</f>
-        <v/>
-      </c>
-      <c r="BM42" s="23">
-        <f>IF(COUNT(BM9:BM41)=0,"",SUM(BM9:BM41))</f>
-        <v/>
-      </c>
-      <c r="BO42" s="24">
-        <f>IF(COUNT(BO9:BO41)=0,"",SUM(BO9:BO41))</f>
-        <v/>
-      </c>
-      <c r="BP42" s="24">
-        <f>IF(COUNT(BP9:BP41)=0,"",SUM(BP9:BP41))</f>
-        <v/>
-      </c>
-      <c r="BQ42" s="24">
-        <f>IF(COUNT(BQ9:BQ41)=0,"",SUM(BQ9:BQ41))</f>
-        <v/>
-      </c>
-      <c r="BR42" s="24">
-        <f>IF(COUNT(BR9:BR41)=0,"",SUM(BR9:BR41))</f>
-        <v/>
-      </c>
-      <c r="BS42" s="24">
-        <f>IF(COUNT(BS9:BS41)=0,"",SUM(BS9:BS41))</f>
-        <v/>
-      </c>
-      <c r="BT42" s="24">
-        <f>IF(COUNT(BT9:BT41)=0,"",SUM(BT9:BT41))</f>
-        <v/>
-      </c>
-      <c r="BU42" s="24">
-        <f>IF(COUNT(BU9:BU41)=0,"",SUM(BU9:BU41))</f>
-        <v/>
-      </c>
-      <c r="BV42" s="24">
-        <f>IF(COUNT(BV9:BV41)=0,"",SUM(BV9:BV41))</f>
-        <v/>
-      </c>
-      <c r="BW42" s="24">
-        <f>IF(COUNT(BW9:BW41)=0,"",SUM(BW9:BW41))</f>
-        <v/>
-      </c>
-      <c r="BX42" s="24">
-        <f>IF(COUNT(BX9:BX41)=0,"",SUM(BX9:BX41))</f>
-        <v/>
-      </c>
-      <c r="BY42" s="24">
-        <f>IF(COUNT(BY9:BY41)=0,"",SUM(BY9:BY41))</f>
-        <v/>
-      </c>
-      <c r="BZ42" s="24">
-        <f>IF(COUNT(BZ9:BZ41)=0,"",SUM(BZ9:BZ41))</f>
-        <v/>
-      </c>
-      <c r="CA42" s="24">
-        <f>IF(COUNT(CA9:CA41)=0,"",SUM(CA9:CA41))</f>
-        <v/>
-      </c>
-      <c r="CB42" s="24">
-        <f>IF(COUNT(CB9:CB41)=0,"",SUM(CB9:CB41))</f>
-        <v/>
-      </c>
-      <c r="CC42" s="24">
-        <f>IF(COUNT(CC9:CC41)=0,"",SUM(CC9:CC41))</f>
-        <v/>
-      </c>
-      <c r="CD42" s="24">
-        <f>IF(COUNT(CD9:CD41)=0,"",SUM(CD9:CD41))</f>
-        <v/>
-      </c>
-      <c r="CE42" s="24">
-        <f>IF(COUNT(CE9:CE41)=0,"",SUM(CE9:CE41))</f>
-        <v/>
-      </c>
-      <c r="CF42" s="24">
-        <f>IF(COUNT(CF9:CF41)=0,"",SUM(CF9:CF41))</f>
-        <v/>
-      </c>
-      <c r="CG42" s="24">
-        <f>IF(COUNT(CG9:CG41)=0,"",SUM(CG9:CG41))</f>
-        <v/>
-      </c>
-      <c r="CH42" s="24">
-        <f>IF(COUNT(CH9:CH41)=0,"",SUM(CH9:CH41))</f>
-        <v/>
-      </c>
-      <c r="CJ42" s="25">
-        <f>IF(COUNT(CJ9:CJ41)=0,"",SUM(CJ9:CJ41))</f>
-        <v/>
-      </c>
-      <c r="CK42" s="25">
-        <f>IF(COUNT(CK9:CK41)=0,"",SUM(CK9:CK41))</f>
-        <v/>
-      </c>
-      <c r="CL42" s="25">
-        <f>IF(COUNT(CL9:CL41)=0,"",SUM(CL9:CL41))</f>
-        <v/>
-      </c>
-      <c r="CM42" s="25">
-        <f>IF(COUNT(CM9:CM41)=0,"",SUM(CM9:CM41))</f>
-        <v/>
-      </c>
-      <c r="CN42" s="25">
-        <f>IF(COUNT(CN9:CN41)=0,"",SUM(CN9:CN41))</f>
-        <v/>
-      </c>
-      <c r="CO42" s="25">
-        <f>IF(COUNT(CO9:CO41)=0,"",SUM(CO9:CO41))</f>
-        <v/>
-      </c>
-      <c r="CP42" s="25">
-        <f>IF(COUNT(CP9:CP41)=0,"",SUM(CP9:CP41))</f>
-        <v/>
-      </c>
-      <c r="CQ42" s="25">
-        <f>IF(COUNT(CQ9:CQ41)=0,"",SUM(CQ9:CQ41))</f>
-        <v/>
-      </c>
-      <c r="CR42" s="25">
-        <f>IF(COUNT(CR9:CR41)=0,"",SUM(CR9:CR41))</f>
-        <v/>
-      </c>
-      <c r="CS42" s="25">
-        <f>IF(COUNT(CS9:CS41)=0,"",SUM(CS9:CS41))</f>
-        <v/>
-      </c>
-      <c r="CT42" s="25">
-        <f>IF(COUNT(CT9:CT41)=0,"",SUM(CT9:CT41))</f>
-        <v/>
-      </c>
-      <c r="CU42" s="25">
-        <f>IF(COUNT(CU9:CU41)=0,"",SUM(CU9:CU41))</f>
-        <v/>
-      </c>
-      <c r="CV42" s="25">
-        <f>IF(COUNT(CV9:CV41)=0,"",SUM(CV9:CV41))</f>
-        <v/>
-      </c>
-      <c r="CW42" s="25">
-        <f>IF(COUNT(CW9:CW41)=0,"",SUM(CW9:CW41))</f>
-        <v/>
-      </c>
-      <c r="CX42" s="25">
-        <f>IF(COUNT(CX9:CX41)=0,"",SUM(CX9:CX41))</f>
-        <v/>
-      </c>
-      <c r="CY42" s="25">
-        <f>IF(COUNT(CY9:CY41)=0,"",SUM(CY9:CY41))</f>
-        <v/>
-      </c>
-      <c r="CZ42" s="25">
-        <f>IF(COUNT(CZ9:CZ41)=0,"",SUM(CZ9:CZ41))</f>
-        <v/>
-      </c>
-      <c r="DA42" s="25">
-        <f>IF(COUNT(DA9:DA41)=0,"",SUM(DA9:DA41))</f>
-        <v/>
-      </c>
-      <c r="DB42" s="25">
-        <f>IF(COUNT(DB9:DB41)=0,"",SUM(DB9:DB41))</f>
-        <v/>
-      </c>
-      <c r="DC42" s="25">
-        <f>IF(COUNT(DC9:DC41)=0,"",SUM(DC9:DC41))</f>
-        <v/>
-      </c>
-      <c r="DE42" s="25">
-        <f>IF(COUNT(DE9:DE41)=0,"",SUM(DE9:DE41))</f>
-        <v/>
-      </c>
-      <c r="DF42" s="25">
-        <f>IF(COUNT(DF9:DF41)=0,"",SUM(DF9:DF41))</f>
-        <v/>
-      </c>
-      <c r="DG42" s="25">
-        <f>IF(COUNT(DG9:DG41)=0,"",SUM(DG9:DG41))</f>
-        <v/>
-      </c>
-      <c r="DH42" s="25">
-        <f>IF(COUNT(DH9:DH41)=0,"",SUM(DH9:DH41))</f>
-        <v/>
-      </c>
-      <c r="DI42" s="25">
-        <f>IF(COUNT(DI9:DI41)=0,"",SUM(DI9:DI41))</f>
-        <v/>
-      </c>
-      <c r="DJ42" s="25">
-        <f>IF(COUNT(DJ9:DJ41)=0,"",SUM(DJ9:DJ41))</f>
-        <v/>
-      </c>
-      <c r="DK42" s="25">
-        <f>IF(COUNT(DK9:DK41)=0,"",SUM(DK9:DK41))</f>
-        <v/>
-      </c>
-      <c r="DL42" s="25">
-        <f>IF(COUNT(DL9:DL41)=0,"",SUM(DL9:DL41))</f>
-        <v/>
-      </c>
-      <c r="DM42" s="25">
-        <f>IF(COUNT(DM9:DM41)=0,"",SUM(DM9:DM41))</f>
-        <v/>
-      </c>
-      <c r="DN42" s="25">
-        <f>IF(COUNT(DN9:DN41)=0,"",SUM(DN9:DN41))</f>
-        <v/>
-      </c>
-      <c r="DO42" s="25">
-        <f>IF(COUNT(DO9:DO41)=0,"",SUM(DO9:DO41))</f>
-        <v/>
-      </c>
-      <c r="DP42" s="25">
-        <f>IF(COUNT(DP9:DP41)=0,"",SUM(DP9:DP41))</f>
-        <v/>
-      </c>
-      <c r="DQ42" s="25">
-        <f>IF(COUNT(DQ9:DQ41)=0,"",SUM(DQ9:DQ41))</f>
-        <v/>
-      </c>
-      <c r="DR42" s="25">
-        <f>IF(COUNT(DR9:DR41)=0,"",SUM(DR9:DR41))</f>
-        <v/>
-      </c>
-      <c r="DS42" s="25">
-        <f>IF(COUNT(DS9:DS41)=0,"",SUM(DS9:DS41))</f>
-        <v/>
-      </c>
-      <c r="DT42" s="25">
-        <f>IF(COUNT(DT9:DT41)=0,"",SUM(DT9:DT41))</f>
-        <v/>
-      </c>
-      <c r="DU42" s="25">
-        <f>IF(COUNT(DU9:DU41)=0,"",SUM(DU9:DU41))</f>
-        <v/>
-      </c>
-      <c r="DV42" s="25">
-        <f>IF(COUNT(DV9:DV41)=0,"",SUM(DV9:DV41))</f>
-        <v/>
-      </c>
-      <c r="DW42" s="25">
-        <f>IF(COUNT(DW9:DW41)=0,"",SUM(DW9:DW41))</f>
-        <v/>
-      </c>
-      <c r="DX42" s="25">
-        <f>IF(COUNT(DX9:DX41)=0,"",SUM(DX9:DX41))</f>
-        <v/>
-      </c>
-      <c r="DZ42" s="23">
-        <f>IF(COUNT(DZ9:DZ41)=0,"",SUM(DZ9:DZ41))</f>
-        <v/>
-      </c>
-      <c r="EA42" s="23">
-        <f>IF(COUNT(EA9:EA41)=0,"",SUM(EA9:EA41))</f>
-        <v/>
-      </c>
-      <c r="EB42" s="23">
-        <f>IF(COUNT(EB9:EB41)=0,"",SUM(EB9:EB41))</f>
-        <v/>
-      </c>
-      <c r="EC42" s="23">
-        <f>IF(COUNT(EC9:EC41)=0,"",SUM(EC9:EC41))</f>
-        <v/>
-      </c>
-      <c r="ED42" s="23">
-        <f>IF(COUNT(ED9:ED41)=0,"",SUM(ED9:ED41))</f>
-        <v/>
-      </c>
-      <c r="EE42" s="23">
-        <f>IF(COUNT(EE9:EE41)=0,"",SUM(EE9:EE41))</f>
-        <v/>
-      </c>
-      <c r="EF42" s="23">
-        <f>IF(COUNT(EF9:EF41)=0,"",SUM(EF9:EF41))</f>
-        <v/>
-      </c>
-      <c r="EG42" s="23">
-        <f>IF(COUNT(EG9:EG41)=0,"",SUM(EG9:EG41))</f>
-        <v/>
-      </c>
-      <c r="EH42" s="23">
-        <f>IF(COUNT(EH9:EH41)=0,"",SUM(EH9:EH41))</f>
-        <v/>
-      </c>
-      <c r="EI42" s="23">
-        <f>IF(COUNT(EI9:EI41)=0,"",SUM(EI9:EI41))</f>
-        <v/>
-      </c>
-      <c r="EJ42" s="23">
-        <f>IF(COUNT(EJ9:EJ41)=0,"",SUM(EJ9:EJ41))</f>
-        <v/>
-      </c>
-      <c r="EK42" s="23">
-        <f>IF(COUNT(EK9:EK41)=0,"",SUM(EK9:EK41))</f>
-        <v/>
-      </c>
-      <c r="EL42" s="23">
-        <f>IF(COUNT(EL9:EL41)=0,"",SUM(EL9:EL41))</f>
-        <v/>
-      </c>
-      <c r="EM42" s="23">
-        <f>IF(COUNT(EM9:EM41)=0,"",SUM(EM9:EM41))</f>
-        <v/>
-      </c>
-      <c r="EN42" s="23">
-        <f>IF(COUNT(EN9:EN41)=0,"",SUM(EN9:EN41))</f>
-        <v/>
-      </c>
-      <c r="EO42" s="23">
-        <f>IF(COUNT(EO9:EO41)=0,"",SUM(EO9:EO41))</f>
-        <v/>
-      </c>
-      <c r="EP42" s="23">
-        <f>IF(COUNT(EP9:EP41)=0,"",SUM(EP9:EP41))</f>
-        <v/>
-      </c>
-      <c r="EQ42" s="23">
-        <f>IF(COUNT(EQ9:EQ41)=0,"",SUM(EQ9:EQ41))</f>
-        <v/>
-      </c>
-      <c r="ER42" s="23">
-        <f>IF(COUNT(ER9:ER41)=0,"",SUM(ER9:ER41))</f>
-        <v/>
-      </c>
-      <c r="ES42" s="23">
-        <f>IF(COUNT(ES9:ES41)=0,"",SUM(ES9:ES41))</f>
-        <v/>
-      </c>
-      <c r="EU42" s="21">
-        <f>SUM(EU9:EU41)</f>
-        <v/>
-      </c>
-      <c r="EV42" s="21">
-        <f>SUM(EV9:EV41)</f>
-        <v/>
-      </c>
-      <c r="EW42" s="21">
-        <f>SUM(EW9:EW41)</f>
-        <v/>
-      </c>
-      <c r="EX42" s="21">
-        <f>SUM(EX9:EX41)</f>
-        <v/>
-      </c>
-      <c r="EY42" s="21">
-        <f>SUM(EY9:EY41)</f>
-        <v/>
-      </c>
-      <c r="EZ42" s="21">
-        <f>SUM(EZ9:EZ41)</f>
-        <v/>
-      </c>
-      <c r="FA42" s="21">
-        <f>SUM(FA9:FA41)</f>
-        <v/>
-      </c>
-      <c r="FB42" s="21">
-        <f>SUM(FB9:FB41)</f>
-        <v/>
-      </c>
-      <c r="FC42" s="21">
-        <f>SUM(FC9:FC41)</f>
-        <v/>
-      </c>
-      <c r="FD42" s="21">
-        <f>SUM(FD9:FD41)</f>
-        <v/>
-      </c>
-      <c r="FE42" s="21">
-        <f>SUM(FE9:FE41)</f>
-        <v/>
-      </c>
-      <c r="FF42" s="21">
-        <f>SUM(FF9:FF41)</f>
-        <v/>
-      </c>
-      <c r="FG42" s="21">
-        <f>SUM(FG9:FG41)</f>
-        <v/>
-      </c>
-      <c r="FH42" s="21">
-        <f>SUM(FH9:FH41)</f>
-        <v/>
-      </c>
-      <c r="FI42" s="21">
-        <f>SUM(FI9:FI41)</f>
-        <v/>
-      </c>
-      <c r="FJ42" s="21">
-        <f>SUM(FJ9:FJ41)</f>
-        <v/>
-      </c>
-      <c r="FK42" s="21">
-        <f>SUM(FK9:FK41)</f>
-        <v/>
-      </c>
-      <c r="FL42" s="21">
-        <f>SUM(FL9:FL41)</f>
-        <v/>
-      </c>
-      <c r="FM42" s="21">
-        <f>SUM(FM9:FM41)</f>
-        <v/>
-      </c>
-      <c r="FN42" s="21">
-        <f>SUM(FN9:FN41)</f>
-        <v/>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>NEW NET = data gain + the sim’s day shift (sim NEW − sim cal_curr) − data spend: anchored to the data, so when the redesign changes nothing it equals CURRENT NET exactly. Δ NET = CURRENT NET − NEW NET (data − sim).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>PLACEMENT (measured against the data before it was built, harness/_probe_daily_alloc*.js): rank-family lumps (Bomb/Chuck/Red Challenge, Level Race, Flash Race, Target Day, Kite, Team Event, Team Race, Flock Flurry) land the DATE AFTER the grid cell — a 1-day cell is a 2-date event, the board settles and pays on the next date. Authored per source on the optional sim_settle sheet (settle_days; lag_0..2 to spread a payout over +0/+1/+2 once the lag data exists). The 7-day view sums the EARN day instead.</t>
+        </is>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="26" t="inlineStr">
-        <is>
-          <t>LEGEND / ALLOCATION RULES (D60, 2026-10-14 — EcoGainsSim_Daily.gs, DAILY_ALLOC_MODEL = settle)</t>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Collections (Hatchling Hideaway, Bomb’s Ballet, Jigsaw, Photoshoot) spread by the MEAN accrual curve’s marginal; Season Pass (Free/Paid) spreads ∝ active rate over every day its lane is open (no reach split — the 3-day stub artefact is gone); Core / Saga / Daily Gift pay daily ∝ weekday/weekend active rate; Night Sky over its daily instances; Rainbow Maker ∝ active rate within its instances. Non-calendar sources (Ads, Other, IAPs, FlowerCoop) are flat over the window. River Rush must be DRAWN on cal_curr — off-grid it is flat and SPTx2 is placed on the wrong days.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>CURRENT GAINS, CURRENT SPEND, CURRENT NET are DATA: data_econ_daily, per earner per day (window-earner denominator, so the 33 days sum to the data_econ window total). They are BLANK past the last day the pull carries — a day with no row is "not pulled yet", never 0 — and blank unless Source = ALL (the data is game-wide).</t>
+          <t>Reading the comparison: a single day’s % is NOT a verdict — the data’s own day-to-day CV is 17–29% for the smooth resources. Read cumulative-through-day-N (N ≥ 7) against the resource’s week-over-week CV (HC 2–12%, boosters 3–22%, UL 10–30%), and timing on 3-day centred sums (±1 day). SPT is dominated by the synthetic Core anchor and SPTx2 by River Rush’s schedule until those are fixed.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>NEW GAINS is the SIM of cal_new. Δ GAINS = data − sim: positive means the data sits above the sim. While cal_curr is the live calendar this Δ mixes the redesign with model error; the validation lane on the far right (SIM of cal_curr) separates them: data − sim_new = (data − sim_curr) + (sim_curr − sim_new).</t>
+          <t>WINDOW: 28 days, day 1 = the column holding the first 1 on the calendars' day-number row (row 4); the blacked-out columns before it are not counted, but cal_curr's events there still scale the measured side to the window (D71). The data blocks read the pull by calendar day, so re-pull data_econ_daily_live with window_start_date = the date of day 1.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>NEW NET = data gain + the sim’s day shift (sim NEW − sim cal_curr) − data spend: anchored to the data, so when the redesign changes nothing it equals CURRENT NET exactly. Δ NET = CURRENT NET − NEW NET (data − sim).</t>
+          <t>Weekend rows (Fri/Sat/Sun) are tinted. Window totals of the SIM blocks reconcile with EcoGainsSim_HC (TOTAL row); the data blocks total only the days pulled (blank = no data, not zero).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>PLACEMENT (measured against the data before it was built, harness/_probe_daily_alloc*.js): rank-family lumps (Bomb/Chuck/Red Challenge, Level Race, Flash Race, Target Day, Kite, Team Event, Team Race, Flock Flurry) land the DATE AFTER the grid cell — a 1-day cell is a 2-date event, the board settles and pays on the next date. Authored per source on the optional sim_settle sheet (settle_days; lag_0..2 to spread a payout over +0/+1/+2 once the lag data exists). The 7-day view sums the EARN day instead.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Collections (Hatchling Hideaway, Bomb’s Ballet, Jigsaw, Photoshoot) spread by the MEAN accrual curve’s marginal; Season Pass (Free/Paid) spreads ∝ active rate over every day its lane is open (no reach split — the 3-day stub artefact is gone); Core / Saga / Daily Gift pay daily ∝ weekday/weekend active rate; Night Sky over its daily instances; Rainbow Maker ∝ active rate within its instances. Non-calendar sources (Ads, Other, IAPs, FlowerCoop) are flat ÷33. River Rush must be DRAWN on cal_curr (days 2–8, 16–22, 30–33) — off-grid it is flat and SPTx2 is placed on the wrong days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Reading the comparison: a single day’s % is NOT a verdict — the data’s own day-to-day CV is 17–29% for the smooth resources. Read cumulative-through-day-N (N ≥ 7) against the resource’s week-over-week CV (HC 2–12%, boosters 3–22%, UL 10–30%), and timing on 3-day centred sums (±1 day). SPT is dominated by the synthetic Core anchor and SPTx2 by River Rush’s schedule until those are fixed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Weekend rows (Fri/Sat/Sun) are tinted. Window totals of the SIM blocks reconcile with EcoGainsSim_HC (TOTAL row); the data blocks total only the days pulled (blank = no data, not zero).</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="5" t="inlineStr">
-        <is>
           <t>PACKS and ToF_Ticket are gains-only and simulated-side only: the data blocks leave their columns BLANK (no telemetry is not a measured 0).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="AT9:BM41">
+  <conditionalFormatting sqref="AT9:BM36">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
@@ -10299,7 +9128,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="DZ9:ES41">
+  <conditionalFormatting sqref="DZ9:ES36">
     <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
@@ -10307,7 +9136,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B9:FN41">
+  <conditionalFormatting sqref="B9:FN36">
     <cfRule type="expression" priority="5" dxfId="2">
       <formula>OR($C9="Fri",$C9="Sat",$C9="Sun")</formula>
     </cfRule>

</xml_diff>